<commit_message>
#8 BOM Changes pending due to another urgent Task
</commit_message>
<xml_diff>
--- a/Documents/Deliverables/BOM/LCSC_BOM.xlsx
+++ b/Documents/Deliverables/BOM/LCSC_BOM.xlsx
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="515" uniqueCount="339">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="517" uniqueCount="340">
   <si>
     <t>S. No.</t>
   </si>
@@ -1061,6 +1061,9 @@
   </si>
   <si>
     <t>C22548</t>
+  </si>
+  <si>
+    <t>WS2812B DIY RGB LED Ring 37 to 241 Pixels WS2812 Round Modules SK6812 5050 Built-in RGB Addressable DC5V LED Circle Arduino Ring</t>
   </si>
 </sst>
 </file>
@@ -1767,7 +1770,7 @@
       <protection locked="0"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="177">
+  <cellXfs count="178">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2132,45 +2135,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="26" xfId="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2232,9 +2196,6 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
@@ -2247,13 +2208,7 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2270,6 +2225,57 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -2557,7 +2563,7 @@
   <cols>
     <col min="1" max="1" width="6.140625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="17.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="93.28515625" customWidth="1"/>
+    <col min="3" max="3" width="80.140625" customWidth="1"/>
     <col min="4" max="4" width="41" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="20.28515625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="25.140625" bestFit="1" customWidth="1"/>
@@ -2577,27 +2583,27 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:19" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="126" t="s">
+      <c r="A1" s="161" t="s">
         <v>157</v>
       </c>
-      <c r="B1" s="127"/>
-      <c r="C1" s="127"/>
-      <c r="D1" s="127"/>
-      <c r="E1" s="127"/>
-      <c r="F1" s="127"/>
-      <c r="G1" s="127"/>
-      <c r="H1" s="127"/>
-      <c r="I1" s="127"/>
-      <c r="J1" s="127"/>
-      <c r="K1" s="127"/>
-      <c r="L1" s="127"/>
-      <c r="M1" s="127"/>
-      <c r="N1" s="127"/>
-      <c r="O1" s="127"/>
-      <c r="P1" s="127"/>
-      <c r="Q1" s="127"/>
-      <c r="R1" s="127"/>
-      <c r="S1" s="128"/>
+      <c r="B1" s="162"/>
+      <c r="C1" s="162"/>
+      <c r="D1" s="162"/>
+      <c r="E1" s="162"/>
+      <c r="F1" s="162"/>
+      <c r="G1" s="162"/>
+      <c r="H1" s="162"/>
+      <c r="I1" s="162"/>
+      <c r="J1" s="162"/>
+      <c r="K1" s="162"/>
+      <c r="L1" s="162"/>
+      <c r="M1" s="162"/>
+      <c r="N1" s="162"/>
+      <c r="O1" s="162"/>
+      <c r="P1" s="162"/>
+      <c r="Q1" s="162"/>
+      <c r="R1" s="162"/>
+      <c r="S1" s="163"/>
     </row>
     <row r="2" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="53" t="s">
@@ -2662,7 +2668,7 @@
       <c r="A3" s="27">
         <v>1</v>
       </c>
-      <c r="B3" s="136" t="s">
+      <c r="B3" s="171" t="s">
         <v>207</v>
       </c>
       <c r="C3" s="72" t="s">
@@ -2721,7 +2727,7 @@
       <c r="A4" s="27">
         <v>2</v>
       </c>
-      <c r="B4" s="137"/>
+      <c r="B4" s="172"/>
       <c r="C4" s="25" t="s">
         <v>17</v>
       </c>
@@ -2778,7 +2784,7 @@
       <c r="A5" s="27">
         <v>3</v>
       </c>
-      <c r="B5" s="137"/>
+      <c r="B5" s="172"/>
       <c r="C5" s="25" t="s">
         <v>19</v>
       </c>
@@ -2835,7 +2841,7 @@
       <c r="A6" s="27">
         <v>4</v>
       </c>
-      <c r="B6" s="137"/>
+      <c r="B6" s="172"/>
       <c r="C6" s="25" t="s">
         <v>22</v>
       </c>
@@ -2893,7 +2899,7 @@
       <c r="A7" s="27">
         <v>5</v>
       </c>
-      <c r="B7" s="137"/>
+      <c r="B7" s="172"/>
       <c r="C7" s="25" t="s">
         <v>25</v>
       </c>
@@ -2950,7 +2956,7 @@
       <c r="A8" s="27">
         <v>6</v>
       </c>
-      <c r="B8" s="137"/>
+      <c r="B8" s="172"/>
       <c r="C8" s="33" t="s">
         <v>28</v>
       </c>
@@ -3009,7 +3015,7 @@
       <c r="A9" s="27">
         <v>7</v>
       </c>
-      <c r="B9" s="137"/>
+      <c r="B9" s="172"/>
       <c r="C9" s="112" t="s">
         <v>266</v>
       </c>
@@ -3066,20 +3072,20 @@
       <c r="A10" s="27">
         <v>8</v>
       </c>
-      <c r="B10" s="138"/>
-      <c r="C10" s="145" t="s">
+      <c r="B10" s="173"/>
+      <c r="C10" s="132" t="s">
         <v>315</v>
       </c>
-      <c r="D10" s="146" t="s">
+      <c r="D10" s="133" t="s">
         <v>316</v>
       </c>
-      <c r="E10" s="147" t="s">
+      <c r="E10" s="134" t="s">
         <v>317</v>
       </c>
-      <c r="F10" s="147" t="s">
+      <c r="F10" s="134" t="s">
         <v>318</v>
       </c>
-      <c r="G10" s="148" t="s">
+      <c r="G10" s="135" t="s">
         <v>326</v>
       </c>
       <c r="H10" s="75" t="s">
@@ -3103,21 +3109,21 @@
       <c r="N10" s="116" t="s">
         <v>223</v>
       </c>
-      <c r="O10" s="149">
+      <c r="O10" s="136">
         <v>6.13E-2</v>
       </c>
       <c r="P10" s="85">
         <f>O10*K10</f>
         <v>0.61299999999999999</v>
       </c>
-      <c r="Q10" s="149">
+      <c r="Q10" s="136">
         <v>6.13E-2</v>
       </c>
-      <c r="R10" s="150">
+      <c r="R10" s="137">
         <f t="shared" si="0"/>
         <v>1.226</v>
       </c>
-      <c r="S10" s="151" t="s">
+      <c r="S10" s="138" t="s">
         <v>337</v>
       </c>
     </row>
@@ -3125,7 +3131,7 @@
       <c r="A11" s="27">
         <v>9</v>
       </c>
-      <c r="B11" s="136" t="s">
+      <c r="B11" s="171" t="s">
         <v>31</v>
       </c>
       <c r="C11" s="24" t="s">
@@ -3186,7 +3192,7 @@
       <c r="A12" s="27">
         <v>10</v>
       </c>
-      <c r="B12" s="137"/>
+      <c r="B12" s="172"/>
       <c r="C12" s="25" t="s">
         <v>169</v>
       </c>
@@ -3243,7 +3249,7 @@
       <c r="A13" s="27">
         <v>11</v>
       </c>
-      <c r="B13" s="137"/>
+      <c r="B13" s="172"/>
       <c r="C13" s="25" t="s">
         <v>40</v>
       </c>
@@ -3300,7 +3306,7 @@
       <c r="A14" s="27">
         <v>12</v>
       </c>
-      <c r="B14" s="138"/>
+      <c r="B14" s="173"/>
       <c r="C14" s="26" t="s">
         <v>170</v>
       </c>
@@ -3352,7 +3358,7 @@
         <f t="shared" si="0"/>
         <v>0.39149999999999996</v>
       </c>
-      <c r="S14" s="151" t="s">
+      <c r="S14" s="138" t="s">
         <v>265</v>
       </c>
     </row>
@@ -3360,7 +3366,7 @@
       <c r="A15" s="27">
         <v>13</v>
       </c>
-      <c r="B15" s="136" t="s">
+      <c r="B15" s="171" t="s">
         <v>298</v>
       </c>
       <c r="C15" s="24" t="s">
@@ -3396,7 +3402,7 @@
       <c r="M15" s="16">
         <v>20</v>
       </c>
-      <c r="N15" s="139" t="s">
+      <c r="N15" s="126" t="s">
         <v>223</v>
       </c>
       <c r="O15" s="18">
@@ -3419,7 +3425,7 @@
       <c r="A16" s="27">
         <v>14</v>
       </c>
-      <c r="B16" s="137"/>
+      <c r="B16" s="172"/>
       <c r="C16" s="25" t="s">
         <v>289</v>
       </c>
@@ -3476,7 +3482,7 @@
       <c r="A17" s="27">
         <v>15</v>
       </c>
-      <c r="B17" s="138"/>
+      <c r="B17" s="173"/>
       <c r="C17" s="26" t="s">
         <v>292</v>
       </c>
@@ -3510,7 +3516,7 @@
       <c r="M17" s="10">
         <v>20</v>
       </c>
-      <c r="N17" s="140" t="s">
+      <c r="N17" s="127" t="s">
         <v>223</v>
       </c>
       <c r="O17" s="13">
@@ -3533,7 +3539,7 @@
       <c r="A18" s="27">
         <v>16</v>
       </c>
-      <c r="B18" s="131" t="s">
+      <c r="B18" s="166" t="s">
         <v>44</v>
       </c>
       <c r="C18" s="24" t="s">
@@ -3551,7 +3557,7 @@
       <c r="G18" s="23" t="s">
         <v>148</v>
       </c>
-      <c r="H18" s="154" t="s">
+      <c r="H18" s="141" t="s">
         <v>274</v>
       </c>
       <c r="I18" s="45" t="s">
@@ -3587,7 +3593,7 @@
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="S18" s="155" t="s">
+      <c r="S18" s="142" t="s">
         <v>275</v>
       </c>
     </row>
@@ -3595,7 +3601,7 @@
       <c r="A19" s="27">
         <v>17</v>
       </c>
-      <c r="B19" s="133"/>
+      <c r="B19" s="168"/>
       <c r="C19" s="26" t="s">
         <v>47</v>
       </c>
@@ -3643,17 +3649,17 @@
       <c r="Q19" s="13">
         <v>0.35360000000000003</v>
       </c>
-      <c r="R19" s="150">
+      <c r="R19" s="137">
         <f t="shared" si="0"/>
         <v>1.7680000000000002</v>
       </c>
-      <c r="S19" s="156"/>
+      <c r="S19" s="143"/>
     </row>
     <row r="20" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="27">
         <v>18</v>
       </c>
-      <c r="B20" s="135" t="s">
+      <c r="B20" s="170" t="s">
         <v>50</v>
       </c>
       <c r="C20" s="86" t="s">
@@ -3668,7 +3674,7 @@
       <c r="F20" s="88" t="s">
         <v>53</v>
       </c>
-      <c r="G20" s="152" t="s">
+      <c r="G20" s="139" t="s">
         <v>39</v>
       </c>
       <c r="H20" s="99" t="s">
@@ -3707,13 +3713,13 @@
         <f t="shared" si="0"/>
         <v>0.28299999999999997</v>
       </c>
-      <c r="S20" s="153"/>
+      <c r="S20" s="140"/>
     </row>
     <row r="21" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="27">
         <v>19</v>
       </c>
-      <c r="B21" s="132"/>
+      <c r="B21" s="167"/>
       <c r="C21" s="25" t="s">
         <v>175</v>
       </c>
@@ -3770,7 +3776,7 @@
       <c r="A22" s="27">
         <v>20</v>
       </c>
-      <c r="B22" s="134"/>
+      <c r="B22" s="169"/>
       <c r="C22" s="90" t="s">
         <v>54</v>
       </c>
@@ -3780,13 +3786,13 @@
       <c r="E22" s="92" t="s">
         <v>168</v>
       </c>
-      <c r="F22" s="157" t="s">
+      <c r="F22" s="144" t="s">
         <v>56</v>
       </c>
       <c r="G22" s="93" t="s">
         <v>57</v>
       </c>
-      <c r="H22" s="158" t="s">
+      <c r="H22" s="145" t="s">
         <v>276</v>
       </c>
       <c r="I22" s="100" t="s">
@@ -3830,7 +3836,7 @@
       <c r="A23" s="27">
         <v>21</v>
       </c>
-      <c r="B23" s="131" t="s">
+      <c r="B23" s="166" t="s">
         <v>208</v>
       </c>
       <c r="C23" s="41" t="s">
@@ -3891,7 +3897,7 @@
       <c r="A24" s="27">
         <v>22</v>
       </c>
-      <c r="B24" s="132"/>
+      <c r="B24" s="167"/>
       <c r="C24" s="25" t="s">
         <v>61</v>
       </c>
@@ -3949,7 +3955,7 @@
       <c r="A25" s="27">
         <v>23</v>
       </c>
-      <c r="B25" s="132"/>
+      <c r="B25" s="167"/>
       <c r="C25" s="25" t="s">
         <v>324</v>
       </c>
@@ -4006,7 +4012,7 @@
       <c r="A26" s="27">
         <v>24</v>
       </c>
-      <c r="B26" s="132"/>
+      <c r="B26" s="167"/>
       <c r="C26" s="25" t="s">
         <v>178</v>
       </c>
@@ -4064,7 +4070,7 @@
       <c r="A27" s="27">
         <v>25</v>
       </c>
-      <c r="B27" s="132"/>
+      <c r="B27" s="167"/>
       <c r="C27" s="43" t="s">
         <v>184</v>
       </c>
@@ -4124,7 +4130,7 @@
       <c r="A28" s="27">
         <v>26</v>
       </c>
-      <c r="B28" s="132"/>
+      <c r="B28" s="167"/>
       <c r="C28" s="25" t="s">
         <v>65</v>
       </c>
@@ -4184,7 +4190,7 @@
       <c r="A29" s="27">
         <v>27</v>
       </c>
-      <c r="B29" s="132"/>
+      <c r="B29" s="167"/>
       <c r="C29" s="43" t="s">
         <v>67</v>
       </c>
@@ -4242,7 +4248,7 @@
       <c r="A30" s="27">
         <v>28</v>
       </c>
-      <c r="B30" s="132"/>
+      <c r="B30" s="167"/>
       <c r="C30" s="25" t="s">
         <v>69</v>
       </c>
@@ -4302,7 +4308,7 @@
       <c r="A31" s="27">
         <v>29</v>
       </c>
-      <c r="B31" s="132"/>
+      <c r="B31" s="167"/>
       <c r="C31" s="25" t="s">
         <v>71</v>
       </c>
@@ -4362,7 +4368,7 @@
       <c r="A32" s="27">
         <v>30</v>
       </c>
-      <c r="B32" s="132"/>
+      <c r="B32" s="167"/>
       <c r="C32" s="25" t="s">
         <v>165</v>
       </c>
@@ -4422,7 +4428,7 @@
       <c r="A33" s="27">
         <v>31</v>
       </c>
-      <c r="B33" s="132"/>
+      <c r="B33" s="167"/>
       <c r="C33" s="25" t="s">
         <v>74</v>
       </c>
@@ -4482,7 +4488,7 @@
       <c r="A34" s="27">
         <v>32</v>
       </c>
-      <c r="B34" s="132"/>
+      <c r="B34" s="167"/>
       <c r="C34" s="25" t="s">
         <v>77</v>
       </c>
@@ -4542,7 +4548,7 @@
       <c r="A35" s="27">
         <v>33</v>
       </c>
-      <c r="B35" s="133"/>
+      <c r="B35" s="168"/>
       <c r="C35" s="26" t="s">
         <v>80</v>
       </c>
@@ -4561,7 +4567,7 @@
       <c r="H35" s="9" t="s">
         <v>241</v>
       </c>
-      <c r="I35" s="159" t="s">
+      <c r="I35" s="146" t="s">
         <v>240</v>
       </c>
       <c r="J35" s="8" t="s">
@@ -4583,14 +4589,14 @@
       <c r="O35" s="13">
         <v>1.8E-3</v>
       </c>
-      <c r="P35" s="150">
+      <c r="P35" s="137">
         <f t="shared" si="2"/>
         <v>0.18</v>
       </c>
       <c r="Q35" s="13">
         <v>1.8E-3</v>
       </c>
-      <c r="R35" s="150">
+      <c r="R35" s="137">
         <f t="shared" si="0"/>
         <v>3.5999999999999997E-2</v>
       </c>
@@ -4662,7 +4668,7 @@
       <c r="A37" s="27">
         <v>35</v>
       </c>
-      <c r="B37" s="131" t="s">
+      <c r="B37" s="166" t="s">
         <v>85</v>
       </c>
       <c r="C37" s="69" t="s">
@@ -4722,7 +4728,7 @@
       <c r="A38" s="27">
         <v>36</v>
       </c>
-      <c r="B38" s="132"/>
+      <c r="B38" s="167"/>
       <c r="C38" s="33" t="s">
         <v>90</v>
       </c>
@@ -4782,7 +4788,7 @@
       <c r="A39" s="27">
         <v>37</v>
       </c>
-      <c r="B39" s="132"/>
+      <c r="B39" s="167"/>
       <c r="C39" s="25" t="s">
         <v>94</v>
       </c>
@@ -4840,7 +4846,7 @@
       <c r="A40" s="27">
         <v>38</v>
       </c>
-      <c r="B40" s="132"/>
+      <c r="B40" s="167"/>
       <c r="C40" s="25" t="s">
         <v>191</v>
       </c>
@@ -4898,7 +4904,7 @@
       <c r="A41" s="27">
         <v>39</v>
       </c>
-      <c r="B41" s="132"/>
+      <c r="B41" s="167"/>
       <c r="C41" s="33" t="s">
         <v>99</v>
       </c>
@@ -4956,7 +4962,7 @@
       <c r="A42" s="27">
         <v>40</v>
       </c>
-      <c r="B42" s="132"/>
+      <c r="B42" s="167"/>
       <c r="C42" s="25" t="s">
         <v>103</v>
       </c>
@@ -5014,7 +5020,7 @@
       <c r="A43" s="27">
         <v>41</v>
       </c>
-      <c r="B43" s="132"/>
+      <c r="B43" s="167"/>
       <c r="C43" s="25" t="s">
         <v>195</v>
       </c>
@@ -5072,7 +5078,7 @@
       <c r="A44" s="27">
         <v>42</v>
       </c>
-      <c r="B44" s="132"/>
+      <c r="B44" s="167"/>
       <c r="C44" s="25" t="s">
         <v>199</v>
       </c>
@@ -5130,7 +5136,7 @@
       <c r="A45" s="27">
         <v>43</v>
       </c>
-      <c r="B45" s="133"/>
+      <c r="B45" s="168"/>
       <c r="C45" s="26" t="s">
         <v>199</v>
       </c>
@@ -5190,7 +5196,7 @@
       <c r="A46" s="27">
         <v>44</v>
       </c>
-      <c r="B46" s="131" t="s">
+      <c r="B46" s="166" t="s">
         <v>109</v>
       </c>
       <c r="C46" s="24" t="s">
@@ -5250,7 +5256,7 @@
       <c r="A47" s="27">
         <v>45</v>
       </c>
-      <c r="B47" s="132"/>
+      <c r="B47" s="167"/>
       <c r="C47" s="25" t="s">
         <v>112</v>
       </c>
@@ -5308,7 +5314,7 @@
       <c r="A48" s="27">
         <v>46</v>
       </c>
-      <c r="B48" s="132"/>
+      <c r="B48" s="167"/>
       <c r="C48" s="25" t="s">
         <v>115</v>
       </c>
@@ -5365,7 +5371,7 @@
       <c r="A49" s="27">
         <v>47</v>
       </c>
-      <c r="B49" s="132"/>
+      <c r="B49" s="167"/>
       <c r="C49" s="25" t="s">
         <v>117</v>
       </c>
@@ -5423,7 +5429,7 @@
       <c r="A50" s="27">
         <v>48</v>
       </c>
-      <c r="B50" s="132"/>
+      <c r="B50" s="167"/>
       <c r="C50" s="25" t="s">
         <v>120</v>
       </c>
@@ -5481,7 +5487,7 @@
       <c r="A51" s="27">
         <v>49</v>
       </c>
-      <c r="B51" s="134"/>
+      <c r="B51" s="169"/>
       <c r="C51" s="68" t="s">
         <v>210</v>
       </c>
@@ -5535,7 +5541,7 @@
       <c r="A52" s="27">
         <v>50</v>
       </c>
-      <c r="B52" s="133"/>
+      <c r="B52" s="168"/>
       <c r="C52" s="55" t="s">
         <v>124</v>
       </c>
@@ -5586,142 +5592,146 @@
       </c>
     </row>
     <row r="53" spans="1:19" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A53" s="141">
+      <c r="A53" s="128">
         <v>51</v>
       </c>
-      <c r="B53" s="160" t="s">
+      <c r="B53" s="174" t="s">
         <v>328</v>
       </c>
-      <c r="C53" s="161" t="s">
+      <c r="C53" s="147" t="s">
         <v>329</v>
       </c>
-      <c r="D53" s="162"/>
+      <c r="D53" s="148"/>
       <c r="E53" s="14" t="s">
         <v>162</v>
       </c>
       <c r="F53" s="14" t="s">
         <v>330</v>
       </c>
-      <c r="G53" s="163"/>
-      <c r="H53" s="163"/>
-      <c r="I53" s="163"/>
-      <c r="J53" s="163"/>
-      <c r="K53" s="163"/>
-      <c r="L53" s="164">
+      <c r="G53" s="149"/>
+      <c r="H53" s="149"/>
+      <c r="I53" s="149"/>
+      <c r="J53" s="149"/>
+      <c r="K53" s="149"/>
+      <c r="L53" s="150">
+        <v>3</v>
+      </c>
+      <c r="M53" s="151">
+        <f t="shared" si="3"/>
+        <v>15</v>
+      </c>
+      <c r="N53" s="149"/>
+      <c r="O53" s="149"/>
+      <c r="P53" s="149"/>
+      <c r="Q53" s="149"/>
+      <c r="R53" s="149"/>
+      <c r="S53" s="152"/>
+    </row>
+    <row r="54" spans="1:19" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A54" s="128">
+        <v>52</v>
+      </c>
+      <c r="B54" s="175"/>
+      <c r="C54" s="130" t="s">
+        <v>331</v>
+      </c>
+      <c r="D54" s="129"/>
+      <c r="E54" s="4" t="s">
+        <v>162</v>
+      </c>
+      <c r="F54" s="4" t="s">
+        <v>332</v>
+      </c>
+      <c r="G54" s="129"/>
+      <c r="H54" s="129"/>
+      <c r="I54" s="129"/>
+      <c r="J54" s="129"/>
+      <c r="K54" s="129"/>
+      <c r="L54" s="131">
         <v>2</v>
       </c>
-      <c r="M53" s="165">
+      <c r="M54" s="160">
         <f t="shared" si="3"/>
         <v>10</v>
       </c>
-      <c r="N53" s="163"/>
-      <c r="O53" s="163"/>
-      <c r="P53" s="163"/>
-      <c r="Q53" s="163"/>
-      <c r="R53" s="163"/>
-      <c r="S53" s="166"/>
-    </row>
-    <row r="54" spans="1:19" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A54" s="141">
-        <v>52</v>
-      </c>
-      <c r="B54" s="167"/>
-      <c r="C54" s="143" t="s">
-        <v>331</v>
-      </c>
-      <c r="D54" s="142"/>
-      <c r="E54" s="4" t="s">
-        <v>162</v>
-      </c>
-      <c r="F54" s="4" t="s">
-        <v>332</v>
-      </c>
-      <c r="G54" s="142"/>
-      <c r="H54" s="142"/>
-      <c r="I54" s="142"/>
-      <c r="J54" s="142"/>
-      <c r="K54" s="142"/>
-      <c r="L54" s="144">
-        <v>2</v>
-      </c>
-      <c r="M54" s="176">
-        <f t="shared" si="3"/>
-        <v>10</v>
-      </c>
-      <c r="N54" s="142"/>
-      <c r="O54" s="142"/>
-      <c r="P54" s="142"/>
-      <c r="Q54" s="142"/>
-      <c r="R54" s="142"/>
-      <c r="S54" s="168"/>
+      <c r="N54" s="129"/>
+      <c r="O54" s="129"/>
+      <c r="P54" s="129"/>
+      <c r="Q54" s="129"/>
+      <c r="R54" s="129"/>
+      <c r="S54" s="153"/>
     </row>
     <row r="55" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A55" s="141">
+      <c r="A55" s="128">
         <v>53</v>
       </c>
-      <c r="B55" s="167"/>
-      <c r="C55" s="142"/>
-      <c r="D55" s="142"/>
-      <c r="E55" s="142"/>
-      <c r="F55" s="144" t="s">
+      <c r="B55" s="175"/>
+      <c r="C55" s="129"/>
+      <c r="D55" s="129"/>
+      <c r="E55" s="129"/>
+      <c r="F55" s="131" t="s">
         <v>333</v>
       </c>
-      <c r="G55" s="142"/>
-      <c r="H55" s="142"/>
-      <c r="I55" s="142"/>
-      <c r="J55" s="142"/>
-      <c r="K55" s="142"/>
-      <c r="L55" s="144">
+      <c r="G55" s="129"/>
+      <c r="H55" s="129"/>
+      <c r="I55" s="129"/>
+      <c r="J55" s="129"/>
+      <c r="K55" s="129"/>
+      <c r="L55" s="131">
         <v>1</v>
       </c>
-      <c r="M55" s="176">
+      <c r="M55" s="160">
         <f t="shared" si="3"/>
         <v>5</v>
       </c>
-      <c r="N55" s="142"/>
-      <c r="O55" s="142"/>
-      <c r="P55" s="142"/>
-      <c r="Q55" s="142"/>
-      <c r="R55" s="142"/>
-      <c r="S55" s="168"/>
+      <c r="N55" s="129"/>
+      <c r="O55" s="129"/>
+      <c r="P55" s="129"/>
+      <c r="Q55" s="129"/>
+      <c r="R55" s="129"/>
+      <c r="S55" s="153"/>
     </row>
-    <row r="56" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A56" s="175">
+    <row r="56" spans="1:19" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A56" s="159">
         <v>54</v>
       </c>
-      <c r="B56" s="169"/>
-      <c r="C56" s="170"/>
-      <c r="D56" s="170"/>
-      <c r="E56" s="170"/>
-      <c r="F56" s="171" t="s">
+      <c r="B56" s="176"/>
+      <c r="C56" s="177" t="s">
+        <v>339</v>
+      </c>
+      <c r="D56" s="154"/>
+      <c r="E56" s="4" t="s">
+        <v>162</v>
+      </c>
+      <c r="F56" s="155" t="s">
         <v>334</v>
       </c>
-      <c r="G56" s="170"/>
-      <c r="H56" s="170"/>
-      <c r="I56" s="170"/>
-      <c r="J56" s="170"/>
-      <c r="K56" s="170"/>
-      <c r="L56" s="172">
+      <c r="G56" s="154"/>
+      <c r="H56" s="154"/>
+      <c r="I56" s="154"/>
+      <c r="J56" s="154"/>
+      <c r="K56" s="154"/>
+      <c r="L56" s="156">
         <v>1</v>
       </c>
-      <c r="M56" s="173">
+      <c r="M56" s="157">
         <f t="shared" si="3"/>
         <v>5</v>
       </c>
-      <c r="N56" s="170"/>
-      <c r="O56" s="170"/>
-      <c r="P56" s="170"/>
-      <c r="Q56" s="170"/>
-      <c r="R56" s="170"/>
-      <c r="S56" s="174"/>
+      <c r="N56" s="154"/>
+      <c r="O56" s="154"/>
+      <c r="P56" s="154"/>
+      <c r="Q56" s="154"/>
+      <c r="R56" s="154"/>
+      <c r="S56" s="158"/>
     </row>
     <row r="57" spans="1:19" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="L57" s="129" t="s">
+      <c r="L57" s="164" t="s">
         <v>159</v>
       </c>
-      <c r="M57" s="129"/>
-      <c r="N57" s="129"/>
-      <c r="O57" s="129"/>
+      <c r="M57" s="164"/>
+      <c r="N57" s="164"/>
+      <c r="O57" s="164"/>
       <c r="P57" s="28"/>
       <c r="Q57" s="29"/>
       <c r="R57" s="30">
@@ -5730,12 +5740,12 @@
       </c>
     </row>
     <row r="58" spans="1:19" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="L58" s="130" t="s">
+      <c r="L58" s="165" t="s">
         <v>160</v>
       </c>
-      <c r="M58" s="130"/>
-      <c r="N58" s="130"/>
-      <c r="O58" s="130"/>
+      <c r="M58" s="165"/>
+      <c r="N58" s="165"/>
+      <c r="O58" s="165"/>
       <c r="P58" s="31">
         <f>SUM(P3:P57)</f>
         <v>41.213200000000001</v>

</xml_diff>

<commit_message>
Quote from Kevin in issue #9 has been added to LCSC BOM.
</commit_message>
<xml_diff>
--- a/Documents/Deliverables/BOM/LCSC_BOM.xlsx
+++ b/Documents/Deliverables/BOM/LCSC_BOM.xlsx
@@ -1,20 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="153222"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24701"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Github\FranciscoGimenez-HCDSHardware\Documents\Deliverables\BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark\FranciscoGimenez-HCDSHardware\Documents\Deliverables\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F15B62AE-B178-4321-A793-685FB3ABC51A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -985,12 +986,6 @@
     <t>U7, U8, U19</t>
   </si>
   <si>
-    <t>Aliexpress</t>
-  </si>
-  <si>
-    <t>Alibaba</t>
-  </si>
-  <si>
     <t>CAP CER 22UF 35V X5R 0805</t>
   </si>
   <si>
@@ -1064,19 +1059,25 @@
   </si>
   <si>
     <t>WS2812B DIY RGB LED Ring 37 to 241 Pixels WS2812 Round Modules SK6812 5050 Built-in RGB Addressable DC5V LED Circle Arduino Ring</t>
+  </si>
+  <si>
+    <t>Custom Supplier</t>
+  </si>
+  <si>
+    <t>Quote from Kevin</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="4">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
     <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.0000"/>
     <numFmt numFmtId="166" formatCode="_(&quot;$&quot;* #,##0.0000_);_(&quot;$&quot;* \(#,##0.0000\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="167" formatCode="_-[$$-409]* #,##0.00_ ;_-[$$-409]* \-#,##0.00\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
   </numFmts>
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="19" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1211,6 +1212,14 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <u/>
+      <sz val="10"/>
+      <color theme="4" tint="-0.249977111117893"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="6">
     <fill>
@@ -2110,9 +2119,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="3" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2226,6 +2232,9 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="14" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2274,8 +2283,8 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -2557,7 +2566,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:S58"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2574,7 +2583,7 @@
     <col min="11" max="11" width="10.7109375" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="19.42578125" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="18.28515625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="18.28515625" customWidth="1"/>
     <col min="15" max="15" width="11.42578125" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="12.140625" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="18.5703125" bestFit="1" customWidth="1"/>
@@ -2952,7 +2961,7 @@
       </c>
       <c r="S7" s="7"/>
     </row>
-    <row r="8" spans="1:19" s="125" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:19" s="124" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="27">
         <v>6</v>
       </c>
@@ -2966,7 +2975,7 @@
       <c r="E8" s="34" t="s">
         <v>162</v>
       </c>
-      <c r="F8" s="121" t="s">
+      <c r="F8" s="120" t="s">
         <v>30</v>
       </c>
       <c r="G8" s="1" t="s">
@@ -3073,29 +3082,29 @@
         <v>8</v>
       </c>
       <c r="B10" s="173"/>
-      <c r="C10" s="132" t="s">
+      <c r="C10" s="131" t="s">
+        <v>313</v>
+      </c>
+      <c r="D10" s="132" t="s">
+        <v>314</v>
+      </c>
+      <c r="E10" s="133" t="s">
         <v>315</v>
       </c>
-      <c r="D10" s="133" t="s">
+      <c r="F10" s="133" t="s">
         <v>316</v>
       </c>
-      <c r="E10" s="134" t="s">
-        <v>317</v>
-      </c>
-      <c r="F10" s="134" t="s">
-        <v>318</v>
-      </c>
-      <c r="G10" s="135" t="s">
-        <v>326</v>
+      <c r="G10" s="134" t="s">
+        <v>324</v>
       </c>
       <c r="H10" s="75" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="I10" s="82" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="J10" s="75" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="K10" s="77">
         <v>10</v>
@@ -3109,22 +3118,22 @@
       <c r="N10" s="116" t="s">
         <v>223</v>
       </c>
-      <c r="O10" s="136">
+      <c r="O10" s="135">
         <v>6.13E-2</v>
       </c>
       <c r="P10" s="85">
         <f>O10*K10</f>
         <v>0.61299999999999999</v>
       </c>
-      <c r="Q10" s="136">
+      <c r="Q10" s="135">
         <v>6.13E-2</v>
       </c>
-      <c r="R10" s="137">
+      <c r="R10" s="136">
         <f t="shared" si="0"/>
         <v>1.226</v>
       </c>
-      <c r="S10" s="138" t="s">
-        <v>337</v>
+      <c r="S10" s="137" t="s">
+        <v>335</v>
       </c>
     </row>
     <row r="11" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -3143,7 +3152,7 @@
       <c r="E11" s="14" t="s">
         <v>34</v>
       </c>
-      <c r="F11" s="122" t="s">
+      <c r="F11" s="121" t="s">
         <v>35</v>
       </c>
       <c r="G11" s="15" t="s">
@@ -3185,7 +3194,7 @@
         <v>1.2869999999999999</v>
       </c>
       <c r="S11" s="110" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
     </row>
     <row r="12" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -3259,7 +3268,7 @@
       <c r="E13" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="F13" s="121" t="s">
+      <c r="F13" s="120" t="s">
         <v>43</v>
       </c>
       <c r="G13" s="3" t="s">
@@ -3316,7 +3325,7 @@
       <c r="E14" s="8" t="s">
         <v>172</v>
       </c>
-      <c r="F14" s="123" t="s">
+      <c r="F14" s="122" t="s">
         <v>173</v>
       </c>
       <c r="G14" s="22" t="s">
@@ -3358,7 +3367,7 @@
         <f t="shared" si="0"/>
         <v>0.39149999999999996</v>
       </c>
-      <c r="S14" s="138" t="s">
+      <c r="S14" s="137" t="s">
         <v>265</v>
       </c>
     </row>
@@ -3402,7 +3411,7 @@
       <c r="M15" s="16">
         <v>20</v>
       </c>
-      <c r="N15" s="126" t="s">
+      <c r="N15" s="125" t="s">
         <v>223</v>
       </c>
       <c r="O15" s="18">
@@ -3516,7 +3525,7 @@
       <c r="M17" s="10">
         <v>20</v>
       </c>
-      <c r="N17" s="127" t="s">
+      <c r="N17" s="126" t="s">
         <v>223</v>
       </c>
       <c r="O17" s="13">
@@ -3533,7 +3542,7 @@
         <f t="shared" si="0"/>
         <v>0.39800000000000002</v>
       </c>
-      <c r="S17" s="118"/>
+      <c r="S17" s="117"/>
     </row>
     <row r="18" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="27">
@@ -3546,7 +3555,7 @@
         <v>45</v>
       </c>
       <c r="D18" s="49" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="E18" s="14" t="s">
         <v>162</v>
@@ -3557,7 +3566,7 @@
       <c r="G18" s="23" t="s">
         <v>148</v>
       </c>
-      <c r="H18" s="141" t="s">
+      <c r="H18" s="140" t="s">
         <v>274</v>
       </c>
       <c r="I18" s="45" t="s">
@@ -3576,24 +3585,24 @@
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
-      <c r="N18" s="119" t="s">
-        <v>313</v>
+      <c r="N18" s="118" t="s">
+        <v>338</v>
       </c>
       <c r="O18" s="18">
-        <v>1</v>
+        <v>2.9</v>
       </c>
       <c r="P18" s="19">
         <f>O18*L18</f>
-        <v>2</v>
+        <v>5.8</v>
       </c>
       <c r="Q18" s="18">
-        <v>1</v>
+        <v>2.9</v>
       </c>
       <c r="R18" s="79">
         <f t="shared" si="0"/>
-        <v>10</v>
-      </c>
-      <c r="S18" s="142" t="s">
+        <v>29</v>
+      </c>
+      <c r="S18" s="141" t="s">
         <v>275</v>
       </c>
     </row>
@@ -3649,11 +3658,11 @@
       <c r="Q19" s="13">
         <v>0.35360000000000003</v>
       </c>
-      <c r="R19" s="137">
+      <c r="R19" s="136">
         <f t="shared" si="0"/>
         <v>1.7680000000000002</v>
       </c>
-      <c r="S19" s="143"/>
+      <c r="S19" s="142"/>
     </row>
     <row r="20" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="27">
@@ -3674,7 +3683,7 @@
       <c r="F20" s="88" t="s">
         <v>53</v>
       </c>
-      <c r="G20" s="139" t="s">
+      <c r="G20" s="138" t="s">
         <v>39</v>
       </c>
       <c r="H20" s="99" t="s">
@@ -3713,7 +3722,7 @@
         <f t="shared" si="0"/>
         <v>0.28299999999999997</v>
       </c>
-      <c r="S20" s="140"/>
+      <c r="S20" s="139"/>
     </row>
     <row r="21" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="27">
@@ -3786,13 +3795,13 @@
       <c r="E22" s="92" t="s">
         <v>168</v>
       </c>
-      <c r="F22" s="144" t="s">
+      <c r="F22" s="143" t="s">
         <v>56</v>
       </c>
       <c r="G22" s="93" t="s">
         <v>57</v>
       </c>
-      <c r="H22" s="145" t="s">
+      <c r="H22" s="144" t="s">
         <v>276</v>
       </c>
       <c r="I22" s="100" t="s">
@@ -3848,7 +3857,7 @@
       <c r="E23" s="14" t="s">
         <v>59</v>
       </c>
-      <c r="F23" s="122" t="s">
+      <c r="F23" s="121" t="s">
         <v>60</v>
       </c>
       <c r="G23" s="23" t="s">
@@ -3957,7 +3966,7 @@
       </c>
       <c r="B25" s="167"/>
       <c r="C25" s="25" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="D25" s="50" t="s">
         <v>311</v>
@@ -3966,19 +3975,19 @@
         <v>59</v>
       </c>
       <c r="F25" s="4" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="G25" s="1" t="s">
         <v>64</v>
       </c>
       <c r="H25" s="6" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="I25" s="46" t="s">
         <v>161</v>
       </c>
       <c r="J25" s="4" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="K25" s="5">
         <v>100</v>
@@ -4080,7 +4089,7 @@
       <c r="E27" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="F27" s="121" t="s">
+      <c r="F27" s="120" t="s">
         <v>185</v>
       </c>
       <c r="G27" s="3" t="s">
@@ -4140,7 +4149,7 @@
       <c r="E28" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="F28" s="121" t="s">
+      <c r="F28" s="120" t="s">
         <v>66</v>
       </c>
       <c r="G28" s="3" t="s">
@@ -4258,7 +4267,7 @@
       <c r="E30" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="F30" s="121" t="s">
+      <c r="F30" s="120" t="s">
         <v>70</v>
       </c>
       <c r="G30" s="3" t="s">
@@ -4318,7 +4327,7 @@
       <c r="E31" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="F31" s="121" t="s">
+      <c r="F31" s="120" t="s">
         <v>72</v>
       </c>
       <c r="G31" s="3" t="s">
@@ -4378,7 +4387,7 @@
       <c r="E32" s="4" t="s">
         <v>182</v>
       </c>
-      <c r="F32" s="121" t="s">
+      <c r="F32" s="120" t="s">
         <v>166</v>
       </c>
       <c r="G32" s="44" t="s">
@@ -4438,7 +4447,7 @@
       <c r="E33" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="F33" s="121" t="s">
+      <c r="F33" s="120" t="s">
         <v>76</v>
       </c>
       <c r="G33" s="3" t="s">
@@ -4498,7 +4507,7 @@
       <c r="E34" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="F34" s="121" t="s">
+      <c r="F34" s="120" t="s">
         <v>79</v>
       </c>
       <c r="G34" s="3" t="s">
@@ -4558,7 +4567,7 @@
       <c r="E35" s="8" t="s">
         <v>59</v>
       </c>
-      <c r="F35" s="123" t="s">
+      <c r="F35" s="122" t="s">
         <v>82</v>
       </c>
       <c r="G35" s="21" t="s">
@@ -4567,7 +4576,7 @@
       <c r="H35" s="9" t="s">
         <v>241</v>
       </c>
-      <c r="I35" s="146" t="s">
+      <c r="I35" s="145" t="s">
         <v>240</v>
       </c>
       <c r="J35" s="8" t="s">
@@ -4589,18 +4598,18 @@
       <c r="O35" s="13">
         <v>1.8E-3</v>
       </c>
-      <c r="P35" s="137">
+      <c r="P35" s="136">
         <f t="shared" si="2"/>
         <v>0.18</v>
       </c>
       <c r="Q35" s="13">
         <v>1.8E-3</v>
       </c>
-      <c r="R35" s="137">
+      <c r="R35" s="136">
         <f t="shared" si="0"/>
         <v>3.5999999999999997E-2</v>
       </c>
-      <c r="S35" s="118" t="s">
+      <c r="S35" s="117" t="s">
         <v>167</v>
       </c>
     </row>
@@ -4608,7 +4617,7 @@
       <c r="A36" s="27">
         <v>34</v>
       </c>
-      <c r="B36" s="120" t="s">
+      <c r="B36" s="119" t="s">
         <v>83</v>
       </c>
       <c r="C36" s="95" t="s">
@@ -4724,7 +4733,7 @@
       </c>
       <c r="S37" s="108"/>
     </row>
-    <row r="38" spans="1:19" s="125" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:19" s="124" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A38" s="27">
         <v>36</v>
       </c>
@@ -4763,22 +4772,22 @@
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="N38" s="117" t="s">
-        <v>313</v>
+      <c r="N38" s="177" t="s">
+        <v>338</v>
       </c>
       <c r="O38" s="38">
-        <v>3.71</v>
+        <v>1.6</v>
       </c>
       <c r="P38" s="11">
         <f t="shared" si="2"/>
-        <v>3.71</v>
+        <v>1.6</v>
       </c>
       <c r="Q38" s="38">
-        <v>3.71</v>
+        <v>1.6</v>
       </c>
       <c r="R38" s="11">
         <f t="shared" si="0"/>
-        <v>18.55</v>
+        <v>8</v>
       </c>
       <c r="S38" s="106" t="s">
         <v>280</v>
@@ -4821,25 +4830,25 @@
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="N39" s="111" t="s">
-        <v>314</v>
+      <c r="N39" s="177" t="s">
+        <v>338</v>
       </c>
       <c r="O39" s="12">
-        <v>0.44700000000000001</v>
+        <v>1.5</v>
       </c>
       <c r="P39" s="11">
         <f>O39*L39</f>
-        <v>0.44700000000000001</v>
+        <v>1.5</v>
       </c>
       <c r="Q39" s="12">
-        <v>0.44700000000000001</v>
+        <v>1.5</v>
       </c>
       <c r="R39" s="11">
         <f t="shared" si="0"/>
-        <v>2.2349999999999999</v>
+        <v>7.5</v>
       </c>
       <c r="S39" s="109" t="s">
-        <v>275</v>
+        <v>339</v>
       </c>
     </row>
     <row r="40" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -5112,7 +5121,7 @@
         <v>5</v>
       </c>
       <c r="N44" s="111" t="s">
-        <v>314</v>
+        <v>338</v>
       </c>
       <c r="O44" s="12">
         <v>1</v>
@@ -5132,7 +5141,7 @@
         <v>278</v>
       </c>
     </row>
-    <row r="45" spans="1:19" s="125" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:19" s="124" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A45" s="27">
         <v>43</v>
       </c>
@@ -5149,7 +5158,7 @@
       <c r="F45" s="8" t="s">
         <v>108</v>
       </c>
-      <c r="G45" s="124" t="s">
+      <c r="G45" s="123" t="s">
         <v>156</v>
       </c>
       <c r="H45" s="9" t="s">
@@ -5171,22 +5180,22 @@
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="N45" s="116" t="s">
-        <v>313</v>
+      <c r="N45" s="177" t="s">
+        <v>338</v>
       </c>
       <c r="O45" s="13">
-        <v>4.3600000000000003</v>
+        <v>9.3000000000000007</v>
       </c>
       <c r="P45" s="85">
         <f t="shared" si="2"/>
-        <v>4.3600000000000003</v>
+        <v>9.3000000000000007</v>
       </c>
       <c r="Q45" s="13">
-        <v>4.3600000000000003</v>
+        <v>9.3000000000000007</v>
       </c>
       <c r="R45" s="80">
         <f t="shared" si="0"/>
-        <v>21.8</v>
+        <v>46.5</v>
       </c>
       <c r="S45" s="106" t="s">
         <v>280</v>
@@ -5508,7 +5517,7 @@
         <v>163</v>
       </c>
       <c r="J51" s="64" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
       <c r="K51" s="64"/>
       <c r="L51" s="65">
@@ -5562,7 +5571,7 @@
         <v>163</v>
       </c>
       <c r="J52" s="58" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="K52" s="58"/>
       <c r="L52" s="59">
@@ -5592,138 +5601,138 @@
       </c>
     </row>
     <row r="53" spans="1:19" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A53" s="128">
+      <c r="A53" s="127">
         <v>51</v>
       </c>
       <c r="B53" s="174" t="s">
-        <v>328</v>
-      </c>
-      <c r="C53" s="147" t="s">
-        <v>329</v>
-      </c>
-      <c r="D53" s="148"/>
+        <v>326</v>
+      </c>
+      <c r="C53" s="146" t="s">
+        <v>327</v>
+      </c>
+      <c r="D53" s="147"/>
       <c r="E53" s="14" t="s">
         <v>162</v>
       </c>
       <c r="F53" s="14" t="s">
-        <v>330</v>
-      </c>
-      <c r="G53" s="149"/>
-      <c r="H53" s="149"/>
-      <c r="I53" s="149"/>
-      <c r="J53" s="149"/>
-      <c r="K53" s="149"/>
-      <c r="L53" s="150">
+        <v>328</v>
+      </c>
+      <c r="G53" s="148"/>
+      <c r="H53" s="148"/>
+      <c r="I53" s="148"/>
+      <c r="J53" s="148"/>
+      <c r="K53" s="148"/>
+      <c r="L53" s="149">
         <v>3</v>
       </c>
-      <c r="M53" s="151">
+      <c r="M53" s="150">
         <f t="shared" si="3"/>
         <v>15</v>
       </c>
-      <c r="N53" s="149"/>
-      <c r="O53" s="149"/>
-      <c r="P53" s="149"/>
-      <c r="Q53" s="149"/>
-      <c r="R53" s="149"/>
-      <c r="S53" s="152"/>
+      <c r="N53" s="148"/>
+      <c r="O53" s="148"/>
+      <c r="P53" s="148"/>
+      <c r="Q53" s="148"/>
+      <c r="R53" s="148"/>
+      <c r="S53" s="151"/>
     </row>
     <row r="54" spans="1:19" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A54" s="128">
+      <c r="A54" s="127">
         <v>52</v>
       </c>
       <c r="B54" s="175"/>
-      <c r="C54" s="130" t="s">
-        <v>331</v>
-      </c>
-      <c r="D54" s="129"/>
+      <c r="C54" s="129" t="s">
+        <v>329</v>
+      </c>
+      <c r="D54" s="128"/>
       <c r="E54" s="4" t="s">
         <v>162</v>
       </c>
       <c r="F54" s="4" t="s">
-        <v>332</v>
-      </c>
-      <c r="G54" s="129"/>
-      <c r="H54" s="129"/>
-      <c r="I54" s="129"/>
-      <c r="J54" s="129"/>
-      <c r="K54" s="129"/>
-      <c r="L54" s="131">
+        <v>330</v>
+      </c>
+      <c r="G54" s="128"/>
+      <c r="H54" s="128"/>
+      <c r="I54" s="128"/>
+      <c r="J54" s="128"/>
+      <c r="K54" s="128"/>
+      <c r="L54" s="130">
         <v>2</v>
       </c>
-      <c r="M54" s="160">
+      <c r="M54" s="159">
         <f t="shared" si="3"/>
         <v>10</v>
       </c>
-      <c r="N54" s="129"/>
-      <c r="O54" s="129"/>
-      <c r="P54" s="129"/>
-      <c r="Q54" s="129"/>
-      <c r="R54" s="129"/>
-      <c r="S54" s="153"/>
+      <c r="N54" s="128"/>
+      <c r="O54" s="128"/>
+      <c r="P54" s="128"/>
+      <c r="Q54" s="128"/>
+      <c r="R54" s="128"/>
+      <c r="S54" s="152"/>
     </row>
     <row r="55" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A55" s="128">
+      <c r="A55" s="127">
         <v>53</v>
       </c>
       <c r="B55" s="175"/>
-      <c r="C55" s="129"/>
-      <c r="D55" s="129"/>
-      <c r="E55" s="129"/>
-      <c r="F55" s="131" t="s">
-        <v>333</v>
-      </c>
-      <c r="G55" s="129"/>
-      <c r="H55" s="129"/>
-      <c r="I55" s="129"/>
-      <c r="J55" s="129"/>
-      <c r="K55" s="129"/>
-      <c r="L55" s="131">
+      <c r="C55" s="128"/>
+      <c r="D55" s="128"/>
+      <c r="E55" s="128"/>
+      <c r="F55" s="130" t="s">
+        <v>331</v>
+      </c>
+      <c r="G55" s="128"/>
+      <c r="H55" s="128"/>
+      <c r="I55" s="128"/>
+      <c r="J55" s="128"/>
+      <c r="K55" s="128"/>
+      <c r="L55" s="130">
         <v>1</v>
       </c>
-      <c r="M55" s="160">
+      <c r="M55" s="159">
         <f t="shared" si="3"/>
         <v>5</v>
       </c>
-      <c r="N55" s="129"/>
-      <c r="O55" s="129"/>
-      <c r="P55" s="129"/>
-      <c r="Q55" s="129"/>
-      <c r="R55" s="129"/>
-      <c r="S55" s="153"/>
+      <c r="N55" s="128"/>
+      <c r="O55" s="128"/>
+      <c r="P55" s="128"/>
+      <c r="Q55" s="128"/>
+      <c r="R55" s="128"/>
+      <c r="S55" s="152"/>
     </row>
     <row r="56" spans="1:19" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A56" s="159">
+      <c r="A56" s="158">
         <v>54</v>
       </c>
       <c r="B56" s="176"/>
-      <c r="C56" s="177" t="s">
-        <v>339</v>
-      </c>
-      <c r="D56" s="154"/>
+      <c r="C56" s="160" t="s">
+        <v>337</v>
+      </c>
+      <c r="D56" s="153"/>
       <c r="E56" s="4" t="s">
         <v>162</v>
       </c>
-      <c r="F56" s="155" t="s">
-        <v>334</v>
-      </c>
-      <c r="G56" s="154"/>
-      <c r="H56" s="154"/>
-      <c r="I56" s="154"/>
-      <c r="J56" s="154"/>
-      <c r="K56" s="154"/>
-      <c r="L56" s="156">
+      <c r="F56" s="154" t="s">
+        <v>332</v>
+      </c>
+      <c r="G56" s="153"/>
+      <c r="H56" s="153"/>
+      <c r="I56" s="153"/>
+      <c r="J56" s="153"/>
+      <c r="K56" s="153"/>
+      <c r="L56" s="155">
         <v>1</v>
       </c>
-      <c r="M56" s="157">
+      <c r="M56" s="156">
         <f t="shared" si="3"/>
         <v>5</v>
       </c>
-      <c r="N56" s="154"/>
-      <c r="O56" s="154"/>
-      <c r="P56" s="154"/>
-      <c r="Q56" s="154"/>
-      <c r="R56" s="154"/>
-      <c r="S56" s="158"/>
+      <c r="N56" s="153"/>
+      <c r="O56" s="153"/>
+      <c r="P56" s="153"/>
+      <c r="Q56" s="153"/>
+      <c r="R56" s="153"/>
+      <c r="S56" s="157"/>
     </row>
     <row r="57" spans="1:19" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
       <c r="L57" s="164" t="s">
@@ -5736,7 +5745,7 @@
       <c r="Q57" s="29"/>
       <c r="R57" s="30">
         <f>SUM(R3:R56)</f>
-        <v>146.00119999999998</v>
+        <v>184.4162</v>
       </c>
     </row>
     <row r="58" spans="1:19" ht="18.75" x14ac:dyDescent="0.3">
@@ -5748,12 +5757,12 @@
       <c r="O58" s="165"/>
       <c r="P58" s="31">
         <f>SUM(P3:P57)</f>
-        <v>41.213200000000001</v>
+        <v>48.896200000000007</v>
       </c>
       <c r="Q58" s="32"/>
       <c r="R58" s="31">
         <f>R57/5</f>
-        <v>29.200239999999997</v>
+        <v>36.883240000000001</v>
       </c>
     </row>
   </sheetData>
@@ -5881,91 +5890,86 @@
     </cfRule>
   </conditionalFormatting>
   <hyperlinks>
-    <hyperlink ref="G3" r:id="rId1" display="https://lcsc.com/brand-detail/254.html"/>
-    <hyperlink ref="G4" r:id="rId2" display="https://lcsc.com/brand-detail/254.html"/>
-    <hyperlink ref="G5" r:id="rId3" display="https://lcsc.com/brand-detail/392.html"/>
-    <hyperlink ref="G6" r:id="rId4" display="https://lcsc.com/brand-detail/254.html"/>
-    <hyperlink ref="G7" r:id="rId5" display="https://lcsc.com/brand-detail/994.html"/>
-    <hyperlink ref="G12" r:id="rId6" display="https://lcsc.com/brand-detail/296.html"/>
-    <hyperlink ref="G22" r:id="rId7" display="https://lcsc.com/brand-detail/94.html"/>
-    <hyperlink ref="G24" r:id="rId8" display="https://lcsc.com/brand-detail/396.html"/>
-    <hyperlink ref="G41" r:id="rId9" display="https://lcsc.com/brand-detail/756.html"/>
-    <hyperlink ref="G42" r:id="rId10" display="https://lcsc.com/brand-detail/100.html"/>
-    <hyperlink ref="G47:G49" r:id="rId11" display="https://lcsc.com/brand-detail/853.html"/>
-    <hyperlink ref="G50" r:id="rId12" display="https://lcsc.com/brand-detail/109.html"/>
-    <hyperlink ref="G8" r:id="rId13" display="https://lcsc.com/brand-detail/994.html"/>
-    <hyperlink ref="G11" r:id="rId14" display="https://www.digikey.com/en/supplier-centers/central-semiconductor"/>
-    <hyperlink ref="G13" r:id="rId15" display="https://www.digikey.com/en/supplier-centers/sunled"/>
-    <hyperlink ref="G18" r:id="rId16" display="https://www.digikey.com/en/supplier-centers/wurth-electronics"/>
-    <hyperlink ref="G20" r:id="rId17" display="https://lcsc.com/brand-detail/296.html"/>
-    <hyperlink ref="G19" r:id="rId18" display="https://www.digikey.com/en/supplier-centers/tdk"/>
-    <hyperlink ref="G23" r:id="rId19" display="https://www.digikey.com/en/supplier-centers/te-connectivity-amp"/>
-    <hyperlink ref="G28" r:id="rId20" display="https://www.digikey.com/en/supplier-centers/rohm-semi"/>
-    <hyperlink ref="G29" r:id="rId21" display="https://www.digikey.com/en/supplier-centers/panasonic"/>
-    <hyperlink ref="G30" r:id="rId22" display="https://www.digikey.com/en/supplier-centers/vishay-dale"/>
-    <hyperlink ref="G31" r:id="rId23" display="https://www.digikey.com/en/supplier-centers/vishay-dale"/>
-    <hyperlink ref="G33" r:id="rId24" display="https://www.digikey.com/en/supplier-centers/vishay-dale"/>
-    <hyperlink ref="G34" r:id="rId25" display="https://www.digikey.com/en/supplier-centers/yageo"/>
-    <hyperlink ref="G35" r:id="rId26" display="https://www.digikey.com/en/supplier-centers/stackpole-electronics"/>
-    <hyperlink ref="G38" r:id="rId27" display="https://www.digikey.com/en/supplier-centers/texas-instruments"/>
-    <hyperlink ref="G39" r:id="rId28" display="https://www.digikey.com/en/supplier-centers/stmicroelectronics"/>
-    <hyperlink ref="G46" r:id="rId29" display="https://lcsc.com/brand-detail/853.html"/>
-    <hyperlink ref="G45" r:id="rId30" display="https://www.digikey.com/en/supplier-centers/analog-devices"/>
-    <hyperlink ref="G26" r:id="rId31" display="https://lcsc.com/brand-detail/396.html"/>
-    <hyperlink ref="G27" r:id="rId32" display="https://www.digikey.com/en/supplier-centers/te-connectivity-amp"/>
-    <hyperlink ref="G37" r:id="rId33" display="https://lcsc.com/brand-detail/877.html"/>
-    <hyperlink ref="N5" r:id="rId34"/>
-    <hyperlink ref="N7" r:id="rId35"/>
-    <hyperlink ref="N6" r:id="rId36"/>
-    <hyperlink ref="N3" r:id="rId37"/>
-    <hyperlink ref="N4" r:id="rId38"/>
-    <hyperlink ref="N8" r:id="rId39"/>
-    <hyperlink ref="N12" r:id="rId40"/>
-    <hyperlink ref="N13" r:id="rId41"/>
-    <hyperlink ref="N19" r:id="rId42"/>
-    <hyperlink ref="N20" r:id="rId43"/>
-    <hyperlink ref="N22" r:id="rId44"/>
-    <hyperlink ref="N24" r:id="rId45"/>
-    <hyperlink ref="N23" r:id="rId46"/>
-    <hyperlink ref="N30" r:id="rId47"/>
-    <hyperlink ref="N31" r:id="rId48"/>
-    <hyperlink ref="N33" r:id="rId49"/>
-    <hyperlink ref="N34" r:id="rId50"/>
-    <hyperlink ref="N35" r:id="rId51"/>
-    <hyperlink ref="N46" r:id="rId52"/>
-    <hyperlink ref="N47" r:id="rId53"/>
-    <hyperlink ref="N48" r:id="rId54"/>
-    <hyperlink ref="N50" r:id="rId55"/>
-    <hyperlink ref="N49" r:id="rId56"/>
-    <hyperlink ref="N42" r:id="rId57"/>
-    <hyperlink ref="N21" r:id="rId58"/>
-    <hyperlink ref="N26" r:id="rId59"/>
-    <hyperlink ref="N28" r:id="rId60"/>
-    <hyperlink ref="N29" r:id="rId61"/>
-    <hyperlink ref="N27" r:id="rId62"/>
-    <hyperlink ref="N32" r:id="rId63"/>
-    <hyperlink ref="N36" r:id="rId64"/>
-    <hyperlink ref="N37" r:id="rId65"/>
-    <hyperlink ref="N40" r:id="rId66"/>
-    <hyperlink ref="N41" r:id="rId67"/>
-    <hyperlink ref="N43" r:id="rId68"/>
-    <hyperlink ref="N9" r:id="rId69"/>
-    <hyperlink ref="N11" r:id="rId70"/>
-    <hyperlink ref="N14" r:id="rId71"/>
-    <hyperlink ref="N18" r:id="rId72"/>
-    <hyperlink ref="N39" r:id="rId73"/>
-    <hyperlink ref="N45" r:id="rId74" display="Arrow"/>
-    <hyperlink ref="N44" r:id="rId75"/>
-    <hyperlink ref="N15" r:id="rId76"/>
-    <hyperlink ref="N16" r:id="rId77"/>
-    <hyperlink ref="N17" r:id="rId78"/>
-    <hyperlink ref="N38" r:id="rId79"/>
-    <hyperlink ref="N10" r:id="rId80"/>
-    <hyperlink ref="G25" r:id="rId81" display="https://lcsc.com/brand-detail/396.html"/>
-    <hyperlink ref="N25" r:id="rId82"/>
+    <hyperlink ref="G3" r:id="rId1" display="https://lcsc.com/brand-detail/254.html" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="G4" r:id="rId2" display="https://lcsc.com/brand-detail/254.html" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
+    <hyperlink ref="G5" r:id="rId3" display="https://lcsc.com/brand-detail/392.html" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
+    <hyperlink ref="G6" r:id="rId4" display="https://lcsc.com/brand-detail/254.html" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
+    <hyperlink ref="G7" r:id="rId5" display="https://lcsc.com/brand-detail/994.html" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
+    <hyperlink ref="G12" r:id="rId6" display="https://lcsc.com/brand-detail/296.html" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
+    <hyperlink ref="G22" r:id="rId7" display="https://lcsc.com/brand-detail/94.html" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
+    <hyperlink ref="G24" r:id="rId8" display="https://lcsc.com/brand-detail/396.html" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
+    <hyperlink ref="G41" r:id="rId9" display="https://lcsc.com/brand-detail/756.html" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
+    <hyperlink ref="G42" r:id="rId10" display="https://lcsc.com/brand-detail/100.html" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
+    <hyperlink ref="G47:G49" r:id="rId11" display="https://lcsc.com/brand-detail/853.html" xr:uid="{00000000-0004-0000-0000-00000A000000}"/>
+    <hyperlink ref="G50" r:id="rId12" display="https://lcsc.com/brand-detail/109.html" xr:uid="{00000000-0004-0000-0000-00000B000000}"/>
+    <hyperlink ref="G8" r:id="rId13" display="https://lcsc.com/brand-detail/994.html" xr:uid="{00000000-0004-0000-0000-00000C000000}"/>
+    <hyperlink ref="G11" r:id="rId14" display="https://www.digikey.com/en/supplier-centers/central-semiconductor" xr:uid="{00000000-0004-0000-0000-00000D000000}"/>
+    <hyperlink ref="G13" r:id="rId15" display="https://www.digikey.com/en/supplier-centers/sunled" xr:uid="{00000000-0004-0000-0000-00000E000000}"/>
+    <hyperlink ref="G18" r:id="rId16" display="https://www.digikey.com/en/supplier-centers/wurth-electronics" xr:uid="{00000000-0004-0000-0000-00000F000000}"/>
+    <hyperlink ref="G20" r:id="rId17" display="https://lcsc.com/brand-detail/296.html" xr:uid="{00000000-0004-0000-0000-000010000000}"/>
+    <hyperlink ref="G19" r:id="rId18" display="https://www.digikey.com/en/supplier-centers/tdk" xr:uid="{00000000-0004-0000-0000-000011000000}"/>
+    <hyperlink ref="G23" r:id="rId19" display="https://www.digikey.com/en/supplier-centers/te-connectivity-amp" xr:uid="{00000000-0004-0000-0000-000012000000}"/>
+    <hyperlink ref="G28" r:id="rId20" display="https://www.digikey.com/en/supplier-centers/rohm-semi" xr:uid="{00000000-0004-0000-0000-000013000000}"/>
+    <hyperlink ref="G29" r:id="rId21" display="https://www.digikey.com/en/supplier-centers/panasonic" xr:uid="{00000000-0004-0000-0000-000014000000}"/>
+    <hyperlink ref="G30" r:id="rId22" display="https://www.digikey.com/en/supplier-centers/vishay-dale" xr:uid="{00000000-0004-0000-0000-000015000000}"/>
+    <hyperlink ref="G31" r:id="rId23" display="https://www.digikey.com/en/supplier-centers/vishay-dale" xr:uid="{00000000-0004-0000-0000-000016000000}"/>
+    <hyperlink ref="G33" r:id="rId24" display="https://www.digikey.com/en/supplier-centers/vishay-dale" xr:uid="{00000000-0004-0000-0000-000017000000}"/>
+    <hyperlink ref="G34" r:id="rId25" display="https://www.digikey.com/en/supplier-centers/yageo" xr:uid="{00000000-0004-0000-0000-000018000000}"/>
+    <hyperlink ref="G35" r:id="rId26" display="https://www.digikey.com/en/supplier-centers/stackpole-electronics" xr:uid="{00000000-0004-0000-0000-000019000000}"/>
+    <hyperlink ref="G38" r:id="rId27" display="https://www.digikey.com/en/supplier-centers/texas-instruments" xr:uid="{00000000-0004-0000-0000-00001A000000}"/>
+    <hyperlink ref="G39" r:id="rId28" display="https://www.digikey.com/en/supplier-centers/stmicroelectronics" xr:uid="{00000000-0004-0000-0000-00001B000000}"/>
+    <hyperlink ref="G46" r:id="rId29" display="https://lcsc.com/brand-detail/853.html" xr:uid="{00000000-0004-0000-0000-00001C000000}"/>
+    <hyperlink ref="G45" r:id="rId30" display="https://www.digikey.com/en/supplier-centers/analog-devices" xr:uid="{00000000-0004-0000-0000-00001D000000}"/>
+    <hyperlink ref="G26" r:id="rId31" display="https://lcsc.com/brand-detail/396.html" xr:uid="{00000000-0004-0000-0000-00001E000000}"/>
+    <hyperlink ref="G27" r:id="rId32" display="https://www.digikey.com/en/supplier-centers/te-connectivity-amp" xr:uid="{00000000-0004-0000-0000-00001F000000}"/>
+    <hyperlink ref="G37" r:id="rId33" display="https://lcsc.com/brand-detail/877.html" xr:uid="{00000000-0004-0000-0000-000020000000}"/>
+    <hyperlink ref="N5" r:id="rId34" xr:uid="{00000000-0004-0000-0000-000021000000}"/>
+    <hyperlink ref="N7" r:id="rId35" xr:uid="{00000000-0004-0000-0000-000022000000}"/>
+    <hyperlink ref="N6" r:id="rId36" xr:uid="{00000000-0004-0000-0000-000023000000}"/>
+    <hyperlink ref="N3" r:id="rId37" xr:uid="{00000000-0004-0000-0000-000024000000}"/>
+    <hyperlink ref="N4" r:id="rId38" xr:uid="{00000000-0004-0000-0000-000025000000}"/>
+    <hyperlink ref="N8" r:id="rId39" xr:uid="{00000000-0004-0000-0000-000026000000}"/>
+    <hyperlink ref="N12" r:id="rId40" xr:uid="{00000000-0004-0000-0000-000027000000}"/>
+    <hyperlink ref="N13" r:id="rId41" xr:uid="{00000000-0004-0000-0000-000028000000}"/>
+    <hyperlink ref="N19" r:id="rId42" xr:uid="{00000000-0004-0000-0000-000029000000}"/>
+    <hyperlink ref="N20" r:id="rId43" xr:uid="{00000000-0004-0000-0000-00002A000000}"/>
+    <hyperlink ref="N22" r:id="rId44" xr:uid="{00000000-0004-0000-0000-00002B000000}"/>
+    <hyperlink ref="N24" r:id="rId45" xr:uid="{00000000-0004-0000-0000-00002C000000}"/>
+    <hyperlink ref="N23" r:id="rId46" xr:uid="{00000000-0004-0000-0000-00002D000000}"/>
+    <hyperlink ref="N30" r:id="rId47" xr:uid="{00000000-0004-0000-0000-00002E000000}"/>
+    <hyperlink ref="N31" r:id="rId48" xr:uid="{00000000-0004-0000-0000-00002F000000}"/>
+    <hyperlink ref="N33" r:id="rId49" xr:uid="{00000000-0004-0000-0000-000030000000}"/>
+    <hyperlink ref="N34" r:id="rId50" xr:uid="{00000000-0004-0000-0000-000031000000}"/>
+    <hyperlink ref="N35" r:id="rId51" xr:uid="{00000000-0004-0000-0000-000032000000}"/>
+    <hyperlink ref="N46" r:id="rId52" xr:uid="{00000000-0004-0000-0000-000033000000}"/>
+    <hyperlink ref="N47" r:id="rId53" xr:uid="{00000000-0004-0000-0000-000034000000}"/>
+    <hyperlink ref="N48" r:id="rId54" xr:uid="{00000000-0004-0000-0000-000035000000}"/>
+    <hyperlink ref="N50" r:id="rId55" xr:uid="{00000000-0004-0000-0000-000036000000}"/>
+    <hyperlink ref="N49" r:id="rId56" xr:uid="{00000000-0004-0000-0000-000037000000}"/>
+    <hyperlink ref="N42" r:id="rId57" xr:uid="{00000000-0004-0000-0000-000038000000}"/>
+    <hyperlink ref="N21" r:id="rId58" xr:uid="{00000000-0004-0000-0000-000039000000}"/>
+    <hyperlink ref="N26" r:id="rId59" xr:uid="{00000000-0004-0000-0000-00003A000000}"/>
+    <hyperlink ref="N28" r:id="rId60" xr:uid="{00000000-0004-0000-0000-00003B000000}"/>
+    <hyperlink ref="N29" r:id="rId61" xr:uid="{00000000-0004-0000-0000-00003C000000}"/>
+    <hyperlink ref="N27" r:id="rId62" xr:uid="{00000000-0004-0000-0000-00003D000000}"/>
+    <hyperlink ref="N32" r:id="rId63" xr:uid="{00000000-0004-0000-0000-00003E000000}"/>
+    <hyperlink ref="N36" r:id="rId64" xr:uid="{00000000-0004-0000-0000-00003F000000}"/>
+    <hyperlink ref="N37" r:id="rId65" xr:uid="{00000000-0004-0000-0000-000040000000}"/>
+    <hyperlink ref="N40" r:id="rId66" xr:uid="{00000000-0004-0000-0000-000041000000}"/>
+    <hyperlink ref="N41" r:id="rId67" xr:uid="{00000000-0004-0000-0000-000042000000}"/>
+    <hyperlink ref="N43" r:id="rId68" xr:uid="{00000000-0004-0000-0000-000043000000}"/>
+    <hyperlink ref="N9" r:id="rId69" xr:uid="{00000000-0004-0000-0000-000044000000}"/>
+    <hyperlink ref="N11" r:id="rId70" xr:uid="{00000000-0004-0000-0000-000045000000}"/>
+    <hyperlink ref="N14" r:id="rId71" xr:uid="{00000000-0004-0000-0000-000046000000}"/>
+    <hyperlink ref="N15" r:id="rId72" xr:uid="{00000000-0004-0000-0000-00004B000000}"/>
+    <hyperlink ref="N16" r:id="rId73" xr:uid="{00000000-0004-0000-0000-00004C000000}"/>
+    <hyperlink ref="N17" r:id="rId74" xr:uid="{00000000-0004-0000-0000-00004D000000}"/>
+    <hyperlink ref="N10" r:id="rId75" xr:uid="{00000000-0004-0000-0000-00004F000000}"/>
+    <hyperlink ref="G25" r:id="rId76" display="https://lcsc.com/brand-detail/396.html" xr:uid="{00000000-0004-0000-0000-000050000000}"/>
+    <hyperlink ref="N25" r:id="rId77" xr:uid="{00000000-0004-0000-0000-000051000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId83"/>
+  <pageSetup orientation="portrait" r:id="rId78"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>

</xml_diff>

<commit_message>
Formating Issue ha BOM me Changes Required han
</commit_message>
<xml_diff>
--- a/Documents/Deliverables/BOM/LCSC_BOM.xlsx
+++ b/Documents/Deliverables/BOM/LCSC_BOM.xlsx
@@ -1,21 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24701"/>
-  <workbookPr/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+  <workbookPr defaultThemeVersion="153222"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark\FranciscoGimenez-HCDSHardware\Documents\Deliverables\BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Github\FranciscoGimenez-HCDSHardware\Documents\Deliverables\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F15B62AE-B178-4321-A793-685FB3ABC51A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -32,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="517" uniqueCount="340">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="533" uniqueCount="348">
   <si>
     <t>S. No.</t>
   </si>
@@ -704,9 +703,6 @@
     <t>VZH471M1ETR-1010</t>
   </si>
   <si>
-    <t>LCSC/MOQ</t>
-  </si>
-  <si>
     <t>LCSC Link</t>
   </si>
   <si>
@@ -1025,9 +1021,6 @@
     <t>C513764</t>
   </si>
   <si>
-    <t>Extra Components</t>
-  </si>
-  <si>
     <t>Mifare 13.56Mhz RC522 RFID Card Reader Module</t>
   </si>
   <si>
@@ -1065,12 +1058,42 @@
   </si>
   <si>
     <t>Quote from Kevin</t>
+  </si>
+  <si>
+    <t>Amazon</t>
+  </si>
+  <si>
+    <t>Power On/Off Switch</t>
+  </si>
+  <si>
+    <t>Battery</t>
+  </si>
+  <si>
+    <t>Adpter</t>
+  </si>
+  <si>
+    <t>12V USB-C Adapter</t>
+  </si>
+  <si>
+    <t>LifePO4; 7.2V; 6Ah battery.</t>
+  </si>
+  <si>
+    <t>Ulincos Momentary Push Button Switch U16F1 1NO1NC Black Metal Shell with Blue LED Ring Suitable for 16mm 5/8" Mounting Hole (Blue)</t>
+  </si>
+  <si>
+    <t>LCSC/MOQ(1 Board)</t>
+  </si>
+  <si>
+    <t>LCSC/MOQ(5 Board)</t>
+  </si>
+  <si>
+    <t>Peripherals</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="4">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
     <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.0000"/>
@@ -1253,7 +1276,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="41">
+  <borders count="40">
     <border>
       <left/>
       <right/>
@@ -1758,19 +1781,6 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -1779,7 +1789,7 @@
       <protection locked="0"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="178">
+  <cellXfs count="181">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2226,15 +2236,15 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="14" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2283,9 +2293,14 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="27" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -2566,8 +2581,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:S58"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:T61"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6.140625" bestFit="1" customWidth="1"/>
@@ -2580,18 +2595,19 @@
     <col min="8" max="8" width="16" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="17.5703125" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="6.140625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="10.7109375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="19.42578125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="18.28515625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="18.28515625" customWidth="1"/>
-    <col min="15" max="15" width="11.42578125" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="18.5703125" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="14" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="52.85546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="19" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="19" customWidth="1"/>
+    <col min="13" max="13" width="19.42578125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="18.28515625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="14.85546875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="18.5703125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="14" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="52.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:20" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="161" t="s">
         <v>157</v>
       </c>
@@ -2612,9 +2628,10 @@
       <c r="P1" s="162"/>
       <c r="Q1" s="162"/>
       <c r="R1" s="162"/>
-      <c r="S1" s="163"/>
+      <c r="S1" s="162"/>
+      <c r="T1" s="163"/>
     </row>
-    <row r="2" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="53" t="s">
         <v>0</v>
       </c>
@@ -2646,34 +2663,37 @@
         <v>8</v>
       </c>
       <c r="K2" s="54" t="s">
+        <v>345</v>
+      </c>
+      <c r="L2" s="54" t="s">
+        <v>346</v>
+      </c>
+      <c r="M2" s="54" t="s">
+        <v>9</v>
+      </c>
+      <c r="N2" s="54" t="s">
+        <v>263</v>
+      </c>
+      <c r="O2" s="54" t="s">
         <v>221</v>
       </c>
-      <c r="L2" s="54" t="s">
-        <v>9</v>
-      </c>
-      <c r="M2" s="54" t="s">
-        <v>264</v>
-      </c>
-      <c r="N2" s="54" t="s">
-        <v>222</v>
-      </c>
-      <c r="O2" s="54" t="s">
+      <c r="P2" s="54" t="s">
         <v>10</v>
       </c>
-      <c r="P2" s="54" t="s">
+      <c r="Q2" s="54" t="s">
         <v>11</v>
       </c>
-      <c r="Q2" s="54" t="s">
+      <c r="R2" s="54" t="s">
         <v>12</v>
       </c>
-      <c r="R2" s="54" t="s">
+      <c r="S2" s="54" t="s">
         <v>144</v>
       </c>
-      <c r="S2" s="54" t="s">
+      <c r="T2" s="54" t="s">
         <v>145</v>
       </c>
     </row>
-    <row r="3" spans="1:19" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:20" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="27">
         <v>1</v>
       </c>
@@ -2684,7 +2704,7 @@
         <v>13</v>
       </c>
       <c r="D3" s="84" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="E3" s="14" t="s">
         <v>14</v>
@@ -2707,32 +2727,35 @@
       <c r="K3" s="16">
         <v>50</v>
       </c>
-      <c r="L3" s="17">
+      <c r="L3" s="16">
+        <v>100</v>
+      </c>
+      <c r="M3" s="17">
         <v>13</v>
       </c>
-      <c r="M3" s="16">
+      <c r="N3" s="16">
         <v>100</v>
       </c>
-      <c r="N3" s="15" t="s">
-        <v>223</v>
-      </c>
-      <c r="O3" s="18">
+      <c r="O3" s="15" t="s">
+        <v>222</v>
+      </c>
+      <c r="P3" s="18">
         <v>6.8999999999999999E-3</v>
       </c>
-      <c r="P3" s="79">
-        <f>O3*K3</f>
+      <c r="Q3" s="79">
+        <f>P3*K3</f>
         <v>0.34499999999999997</v>
       </c>
-      <c r="Q3" s="18">
+      <c r="R3" s="18">
         <v>6.8999999999999999E-3</v>
       </c>
-      <c r="R3" s="79">
-        <f>Q3*M3</f>
+      <c r="S3" s="79">
+        <f>R3*N3</f>
         <v>0.69</v>
       </c>
-      <c r="S3" s="20"/>
+      <c r="T3" s="20"/>
     </row>
-    <row r="4" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="27">
         <v>2</v>
       </c>
@@ -2741,7 +2764,7 @@
         <v>17</v>
       </c>
       <c r="D4" s="50" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="E4" s="4" t="s">
         <v>14</v>
@@ -2764,32 +2787,33 @@
       <c r="K4" s="5">
         <v>50</v>
       </c>
-      <c r="L4" s="6">
+      <c r="L4" s="5"/>
+      <c r="M4" s="6">
         <v>7</v>
       </c>
-      <c r="M4" s="5">
+      <c r="N4" s="5">
         <v>50</v>
       </c>
-      <c r="N4" s="1" t="s">
-        <v>223</v>
-      </c>
-      <c r="O4" s="12">
+      <c r="O4" s="1" t="s">
+        <v>222</v>
+      </c>
+      <c r="P4" s="12">
         <v>6.4999999999999997E-3</v>
       </c>
-      <c r="P4" s="11">
-        <f>O4*K4</f>
+      <c r="Q4" s="11">
+        <f>P4*K4</f>
         <v>0.32500000000000001</v>
       </c>
-      <c r="Q4" s="12">
+      <c r="R4" s="12">
         <v>6.4999999999999997E-3</v>
       </c>
-      <c r="R4" s="11">
-        <f t="shared" ref="R4:R50" si="0">Q4*M4</f>
+      <c r="S4" s="11">
+        <f t="shared" ref="S4:S50" si="0">R4*N4</f>
         <v>0.32500000000000001</v>
       </c>
-      <c r="S4" s="7"/>
+      <c r="T4" s="7"/>
     </row>
-    <row r="5" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="27">
         <v>3</v>
       </c>
@@ -2798,7 +2822,7 @@
         <v>19</v>
       </c>
       <c r="D5" s="50" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="E5" s="4" t="s">
         <v>14</v>
@@ -2821,32 +2845,33 @@
       <c r="K5" s="5">
         <v>10</v>
       </c>
-      <c r="L5" s="6">
+      <c r="L5" s="5"/>
+      <c r="M5" s="6">
         <v>6</v>
       </c>
-      <c r="M5" s="5">
+      <c r="N5" s="5">
         <v>50</v>
       </c>
-      <c r="N5" s="1" t="s">
-        <v>223</v>
-      </c>
-      <c r="O5" s="12">
+      <c r="O5" s="1" t="s">
+        <v>222</v>
+      </c>
+      <c r="P5" s="12">
         <v>5.4699999999999999E-2</v>
       </c>
-      <c r="P5" s="11">
-        <f>O5*K5</f>
+      <c r="Q5" s="11">
+        <f>P5*K5</f>
         <v>0.54699999999999993</v>
       </c>
-      <c r="Q5" s="12">
+      <c r="R5" s="12">
         <v>5.1200000000000002E-2</v>
       </c>
-      <c r="R5" s="11">
+      <c r="S5" s="11">
         <f t="shared" si="0"/>
         <v>2.56</v>
       </c>
-      <c r="S5" s="7"/>
+      <c r="T5" s="7"/>
     </row>
-    <row r="6" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="27">
         <v>4</v>
       </c>
@@ -2878,33 +2903,34 @@
       <c r="K6" s="5">
         <v>20</v>
       </c>
-      <c r="L6" s="6">
+      <c r="L6" s="5"/>
+      <c r="M6" s="6">
         <v>2</v>
       </c>
-      <c r="M6" s="5">
-        <f t="shared" ref="M6:M45" si="1">L6*5</f>
+      <c r="N6" s="5">
+        <f t="shared" ref="N6:N45" si="1">M6*5</f>
         <v>10</v>
       </c>
-      <c r="N6" s="1" t="s">
-        <v>223</v>
-      </c>
-      <c r="O6" s="12">
+      <c r="O6" s="1" t="s">
+        <v>222</v>
+      </c>
+      <c r="P6" s="12">
         <v>2.5000000000000001E-2</v>
       </c>
-      <c r="P6" s="11">
-        <f>O6*K6</f>
+      <c r="Q6" s="11">
+        <f>P6*K6</f>
         <v>0.5</v>
       </c>
-      <c r="Q6" s="12">
+      <c r="R6" s="12">
         <v>2.5000000000000001E-2</v>
       </c>
-      <c r="R6" s="11">
+      <c r="S6" s="11">
         <f t="shared" si="0"/>
         <v>0.25</v>
       </c>
-      <c r="S6" s="7"/>
+      <c r="T6" s="7"/>
     </row>
-    <row r="7" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="27">
         <v>5</v>
       </c>
@@ -2913,7 +2939,7 @@
         <v>25</v>
       </c>
       <c r="D7" s="50" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="E7" s="4" t="s">
         <v>162</v>
@@ -2936,32 +2962,33 @@
       <c r="K7" s="5">
         <v>5</v>
       </c>
-      <c r="L7" s="6">
+      <c r="L7" s="5"/>
+      <c r="M7" s="6">
         <v>2</v>
       </c>
-      <c r="M7" s="5">
+      <c r="N7" s="5">
         <v>10</v>
       </c>
-      <c r="N7" s="1" t="s">
-        <v>223</v>
-      </c>
-      <c r="O7" s="12">
+      <c r="O7" s="1" t="s">
+        <v>222</v>
+      </c>
+      <c r="P7" s="12">
         <v>0.15359999999999999</v>
       </c>
-      <c r="P7" s="11">
-        <f t="shared" ref="P7:P50" si="2">O7*K7</f>
+      <c r="Q7" s="11">
+        <f t="shared" ref="Q7:Q50" si="2">P7*K7</f>
         <v>0.7679999999999999</v>
       </c>
-      <c r="Q7" s="12">
+      <c r="R7" s="12">
         <v>0.15359999999999999</v>
       </c>
-      <c r="R7" s="11">
+      <c r="S7" s="11">
         <f t="shared" si="0"/>
         <v>1.5359999999999998</v>
       </c>
-      <c r="S7" s="7"/>
+      <c r="T7" s="7"/>
     </row>
-    <row r="8" spans="1:19" s="124" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:20" s="124" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="27">
         <v>6</v>
       </c>
@@ -2993,150 +3020,153 @@
       <c r="K8" s="5">
         <v>1</v>
       </c>
-      <c r="L8" s="6">
+      <c r="L8" s="5"/>
+      <c r="M8" s="6">
         <v>2</v>
       </c>
-      <c r="M8" s="5">
+      <c r="N8" s="5">
         <v>12</v>
       </c>
-      <c r="N8" s="1" t="s">
-        <v>223</v>
-      </c>
-      <c r="O8" s="12">
+      <c r="O8" s="1" t="s">
+        <v>222</v>
+      </c>
+      <c r="P8" s="12">
         <v>0.2046</v>
       </c>
-      <c r="P8" s="11">
-        <f>O8*L8</f>
+      <c r="Q8" s="11">
+        <f>P8*M8</f>
         <v>0.40920000000000001</v>
       </c>
-      <c r="Q8" s="12">
+      <c r="R8" s="12">
         <v>0.16300000000000001</v>
       </c>
-      <c r="R8" s="11">
+      <c r="S8" s="11">
         <f t="shared" si="0"/>
         <v>1.956</v>
       </c>
-      <c r="S8" s="105" t="s">
-        <v>281</v>
+      <c r="T8" s="105" t="s">
+        <v>280</v>
       </c>
     </row>
-    <row r="9" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="27">
         <v>7</v>
       </c>
       <c r="B9" s="172"/>
       <c r="C9" s="112" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="D9" s="113" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="E9" s="114" t="s">
         <v>14</v>
       </c>
       <c r="F9" s="114" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="G9" s="115" t="s">
         <v>153</v>
       </c>
       <c r="H9" s="4" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="I9" s="46" t="s">
         <v>161</v>
       </c>
       <c r="J9" s="92" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="K9" s="5">
         <v>20</v>
       </c>
-      <c r="L9" s="6">
+      <c r="L9" s="5"/>
+      <c r="M9" s="6">
         <v>1</v>
       </c>
-      <c r="M9" s="5">
+      <c r="N9" s="5">
         <v>20</v>
       </c>
-      <c r="N9" s="1" t="s">
-        <v>223</v>
-      </c>
-      <c r="O9" s="12">
+      <c r="O9" s="1" t="s">
+        <v>222</v>
+      </c>
+      <c r="P9" s="12">
         <v>2.5399999999999999E-2</v>
       </c>
-      <c r="P9" s="11">
-        <f>O9*K9</f>
+      <c r="Q9" s="11">
+        <f>P9*K9</f>
         <v>0.50800000000000001</v>
       </c>
-      <c r="Q9" s="12">
+      <c r="R9" s="12">
         <v>2.5399999999999999E-2</v>
       </c>
-      <c r="R9" s="11">
+      <c r="S9" s="11">
         <f t="shared" si="0"/>
         <v>0.50800000000000001</v>
       </c>
-      <c r="S9" s="105"/>
+      <c r="T9" s="105"/>
     </row>
-    <row r="10" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="27">
         <v>8</v>
       </c>
       <c r="B10" s="173"/>
       <c r="C10" s="131" t="s">
+        <v>312</v>
+      </c>
+      <c r="D10" s="132" t="s">
         <v>313</v>
       </c>
-      <c r="D10" s="132" t="s">
+      <c r="E10" s="133" t="s">
         <v>314</v>
       </c>
-      <c r="E10" s="133" t="s">
+      <c r="F10" s="133" t="s">
         <v>315</v>
       </c>
-      <c r="F10" s="133" t="s">
-        <v>316</v>
-      </c>
       <c r="G10" s="134" t="s">
+        <v>323</v>
+      </c>
+      <c r="H10" s="75" t="s">
         <v>324</v>
       </c>
-      <c r="H10" s="75" t="s">
-        <v>325</v>
-      </c>
       <c r="I10" s="82" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="J10" s="75" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="K10" s="77">
         <v>10</v>
       </c>
-      <c r="L10" s="76">
+      <c r="L10" s="77"/>
+      <c r="M10" s="76">
         <v>2</v>
       </c>
-      <c r="M10" s="10">
+      <c r="N10" s="10">
         <v>20</v>
       </c>
-      <c r="N10" s="116" t="s">
-        <v>223</v>
-      </c>
-      <c r="O10" s="135">
+      <c r="O10" s="116" t="s">
+        <v>222</v>
+      </c>
+      <c r="P10" s="135">
         <v>6.13E-2</v>
       </c>
-      <c r="P10" s="85">
-        <f>O10*K10</f>
+      <c r="Q10" s="85">
+        <f>P10*K10</f>
         <v>0.61299999999999999</v>
       </c>
-      <c r="Q10" s="135">
+      <c r="R10" s="135">
         <v>6.13E-2</v>
       </c>
-      <c r="R10" s="136">
+      <c r="S10" s="136">
         <f t="shared" si="0"/>
         <v>1.226</v>
       </c>
-      <c r="S10" s="137" t="s">
-        <v>335</v>
+      <c r="T10" s="137" t="s">
+        <v>333</v>
       </c>
     </row>
-    <row r="11" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="27">
         <v>9</v>
       </c>
@@ -3159,10 +3189,10 @@
         <v>146</v>
       </c>
       <c r="H11" s="17" t="s">
+        <v>269</v>
+      </c>
+      <c r="I11" s="45" t="s">
         <v>270</v>
-      </c>
-      <c r="I11" s="45" t="s">
-        <v>271</v>
       </c>
       <c r="J11" s="14" t="s">
         <v>158</v>
@@ -3170,34 +3200,35 @@
       <c r="K11" s="16">
         <v>5</v>
       </c>
-      <c r="L11" s="17">
+      <c r="L11" s="16"/>
+      <c r="M11" s="17">
         <v>2</v>
       </c>
-      <c r="M11" s="16">
+      <c r="N11" s="16">
         <v>15</v>
       </c>
-      <c r="N11" s="15" t="s">
-        <v>223</v>
-      </c>
-      <c r="O11" s="18">
+      <c r="O11" s="15" t="s">
+        <v>222</v>
+      </c>
+      <c r="P11" s="18">
         <v>8.5800000000000001E-2</v>
       </c>
-      <c r="P11" s="79">
-        <f>O11*K11</f>
+      <c r="Q11" s="79">
+        <f>P11*K11</f>
         <v>0.42899999999999999</v>
       </c>
-      <c r="Q11" s="18">
+      <c r="R11" s="18">
         <v>8.5800000000000001E-2</v>
       </c>
-      <c r="R11" s="79">
+      <c r="S11" s="79">
         <f t="shared" si="0"/>
         <v>1.2869999999999999</v>
       </c>
-      <c r="S11" s="110" t="s">
-        <v>333</v>
+      <c r="T11" s="110" t="s">
+        <v>331</v>
       </c>
     </row>
-    <row r="12" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="27">
         <v>10</v>
       </c>
@@ -3218,7 +3249,7 @@
         <v>39</v>
       </c>
       <c r="H12" s="6" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="I12" s="46" t="s">
         <v>161</v>
@@ -3229,32 +3260,33 @@
       <c r="K12" s="5">
         <v>10</v>
       </c>
-      <c r="L12" s="6">
+      <c r="L12" s="5"/>
+      <c r="M12" s="6">
         <v>1</v>
       </c>
-      <c r="M12" s="5">
+      <c r="N12" s="5">
         <v>10</v>
       </c>
-      <c r="N12" s="1" t="s">
-        <v>223</v>
-      </c>
-      <c r="O12" s="12">
+      <c r="O12" s="1" t="s">
+        <v>222</v>
+      </c>
+      <c r="P12" s="12">
         <v>4.1799999999999997E-2</v>
       </c>
-      <c r="P12" s="11">
+      <c r="Q12" s="11">
         <f t="shared" si="2"/>
         <v>0.41799999999999998</v>
       </c>
-      <c r="Q12" s="12">
+      <c r="R12" s="12">
         <v>4.1799999999999997E-2</v>
       </c>
-      <c r="R12" s="11">
+      <c r="S12" s="11">
         <f t="shared" si="0"/>
         <v>0.41799999999999998</v>
       </c>
-      <c r="S12" s="7"/>
+      <c r="T12" s="7"/>
     </row>
-    <row r="13" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="27">
         <v>11</v>
       </c>
@@ -3275,10 +3307,10 @@
         <v>147</v>
       </c>
       <c r="H13" s="6" t="s">
+        <v>224</v>
+      </c>
+      <c r="I13" s="46" t="s">
         <v>225</v>
-      </c>
-      <c r="I13" s="46" t="s">
-        <v>226</v>
       </c>
       <c r="J13" s="4" t="s">
         <v>158</v>
@@ -3286,32 +3318,33 @@
       <c r="K13" s="5">
         <v>50</v>
       </c>
-      <c r="L13" s="6">
+      <c r="L13" s="5"/>
+      <c r="M13" s="6">
         <v>2</v>
       </c>
-      <c r="M13" s="5">
+      <c r="N13" s="5">
         <v>50</v>
       </c>
-      <c r="N13" s="1" t="s">
-        <v>223</v>
-      </c>
-      <c r="O13" s="12">
+      <c r="O13" s="1" t="s">
+        <v>222</v>
+      </c>
+      <c r="P13" s="12">
         <v>1.4800000000000001E-2</v>
       </c>
-      <c r="P13" s="11">
+      <c r="Q13" s="11">
         <f t="shared" si="2"/>
         <v>0.74</v>
       </c>
-      <c r="Q13" s="12">
+      <c r="R13" s="12">
         <v>1.4800000000000001E-2</v>
       </c>
-      <c r="R13" s="11">
+      <c r="S13" s="11">
         <f t="shared" si="0"/>
         <v>0.74</v>
       </c>
-      <c r="S13" s="7"/>
+      <c r="T13" s="7"/>
     </row>
-    <row r="14" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="27">
         <v>12</v>
       </c>
@@ -3332,10 +3365,10 @@
         <v>174</v>
       </c>
       <c r="H14" s="9" t="s">
+        <v>271</v>
+      </c>
+      <c r="I14" s="47" t="s">
         <v>272</v>
-      </c>
-      <c r="I14" s="47" t="s">
-        <v>273</v>
       </c>
       <c r="J14" s="8" t="s">
         <v>158</v>
@@ -3343,58 +3376,59 @@
       <c r="K14" s="75">
         <v>10</v>
       </c>
-      <c r="L14" s="76">
+      <c r="L14" s="75"/>
+      <c r="M14" s="76">
         <v>1</v>
       </c>
-      <c r="M14" s="77">
+      <c r="N14" s="77">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="N14" s="21" t="s">
-        <v>223</v>
-      </c>
-      <c r="O14" s="13">
+      <c r="O14" s="21" t="s">
+        <v>222</v>
+      </c>
+      <c r="P14" s="13">
         <v>7.8299999999999995E-2</v>
       </c>
-      <c r="P14" s="85">
+      <c r="Q14" s="85">
         <f t="shared" si="2"/>
         <v>0.78299999999999992</v>
       </c>
-      <c r="Q14" s="13">
+      <c r="R14" s="13">
         <v>7.8299999999999995E-2</v>
       </c>
-      <c r="R14" s="85">
+      <c r="S14" s="85">
         <f t="shared" si="0"/>
         <v>0.39149999999999996</v>
       </c>
-      <c r="S14" s="137" t="s">
-        <v>265</v>
+      <c r="T14" s="137" t="s">
+        <v>264</v>
       </c>
     </row>
-    <row r="15" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="27">
         <v>13</v>
       </c>
       <c r="B15" s="171" t="s">
+        <v>297</v>
+      </c>
+      <c r="C15" s="24" t="s">
+        <v>285</v>
+      </c>
+      <c r="D15" s="49" t="s">
+        <v>286</v>
+      </c>
+      <c r="E15" s="14" t="s">
+        <v>293</v>
+      </c>
+      <c r="F15" s="14" t="s">
+        <v>287</v>
+      </c>
+      <c r="G15" s="23" t="s">
+        <v>295</v>
+      </c>
+      <c r="H15" s="17" t="s">
         <v>298</v>
-      </c>
-      <c r="C15" s="24" t="s">
-        <v>286</v>
-      </c>
-      <c r="D15" s="49" t="s">
-        <v>287</v>
-      </c>
-      <c r="E15" s="14" t="s">
-        <v>294</v>
-      </c>
-      <c r="F15" s="14" t="s">
-        <v>288</v>
-      </c>
-      <c r="G15" s="23" t="s">
-        <v>296</v>
-      </c>
-      <c r="H15" s="17" t="s">
-        <v>299</v>
       </c>
       <c r="I15" s="45" t="s">
         <v>161</v>
@@ -3405,53 +3439,54 @@
       <c r="K15" s="14">
         <v>20</v>
       </c>
-      <c r="L15" s="17">
+      <c r="L15" s="14"/>
+      <c r="M15" s="17">
         <v>1</v>
       </c>
-      <c r="M15" s="16">
+      <c r="N15" s="16">
         <v>20</v>
       </c>
-      <c r="N15" s="125" t="s">
-        <v>223</v>
-      </c>
-      <c r="O15" s="18">
+      <c r="O15" s="125" t="s">
+        <v>222</v>
+      </c>
+      <c r="P15" s="18">
         <v>2.2800000000000001E-2</v>
       </c>
-      <c r="P15" s="79">
-        <f>O15*K15</f>
+      <c r="Q15" s="79">
+        <f>P15*K15</f>
         <v>0.45600000000000002</v>
       </c>
-      <c r="Q15" s="18">
+      <c r="R15" s="18">
         <v>2.2800000000000001E-2</v>
       </c>
-      <c r="R15" s="79">
+      <c r="S15" s="79">
         <f t="shared" si="0"/>
         <v>0.45600000000000002</v>
       </c>
-      <c r="S15" s="110"/>
+      <c r="T15" s="110"/>
     </row>
-    <row r="16" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="27">
         <v>14</v>
       </c>
       <c r="B16" s="172"/>
       <c r="C16" s="25" t="s">
+        <v>288</v>
+      </c>
+      <c r="D16" s="50" t="s">
         <v>289</v>
       </c>
-      <c r="D16" s="50" t="s">
+      <c r="E16" s="4" t="s">
+        <v>293</v>
+      </c>
+      <c r="F16" s="4" t="s">
         <v>290</v>
       </c>
-      <c r="E16" s="4" t="s">
-        <v>294</v>
-      </c>
-      <c r="F16" s="4" t="s">
-        <v>291</v>
-      </c>
       <c r="G16" s="3" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="H16" s="6" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="I16" s="46" t="s">
         <v>161</v>
@@ -3462,53 +3497,54 @@
       <c r="K16" s="4">
         <v>20</v>
       </c>
-      <c r="L16" s="6">
+      <c r="L16" s="4"/>
+      <c r="M16" s="6">
         <v>1</v>
       </c>
-      <c r="M16" s="5">
+      <c r="N16" s="5">
         <v>20</v>
       </c>
-      <c r="N16" s="111" t="s">
-        <v>223</v>
-      </c>
-      <c r="O16" s="12">
+      <c r="O16" s="111" t="s">
+        <v>222</v>
+      </c>
+      <c r="P16" s="12">
         <v>2.7900000000000001E-2</v>
       </c>
-      <c r="P16" s="83">
+      <c r="Q16" s="83">
         <f t="shared" si="2"/>
         <v>0.55800000000000005</v>
       </c>
-      <c r="Q16" s="12">
+      <c r="R16" s="12">
         <v>2.7900000000000001E-2</v>
       </c>
-      <c r="R16" s="11">
+      <c r="S16" s="11">
         <f t="shared" si="0"/>
         <v>0.55800000000000005</v>
       </c>
-      <c r="S16" s="105"/>
+      <c r="T16" s="105"/>
     </row>
-    <row r="17" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="27">
         <v>15</v>
       </c>
       <c r="B17" s="173"/>
       <c r="C17" s="26" t="s">
+        <v>291</v>
+      </c>
+      <c r="D17" s="52" t="s">
         <v>292</v>
       </c>
-      <c r="D17" s="52" t="s">
+      <c r="E17" s="8" t="s">
         <v>293</v>
       </c>
-      <c r="E17" s="8" t="s">
+      <c r="F17" s="8" t="s">
         <v>294</v>
       </c>
-      <c r="F17" s="8" t="s">
+      <c r="G17" s="22" t="s">
         <v>295</v>
       </c>
-      <c r="G17" s="22" t="s">
-        <v>296</v>
-      </c>
       <c r="H17" s="9" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="I17" s="47" t="s">
         <v>161</v>
@@ -3519,32 +3555,33 @@
       <c r="K17" s="8">
         <v>20</v>
       </c>
-      <c r="L17" s="9">
+      <c r="L17" s="8"/>
+      <c r="M17" s="9">
         <v>1</v>
       </c>
-      <c r="M17" s="10">
+      <c r="N17" s="10">
         <v>20</v>
       </c>
-      <c r="N17" s="126" t="s">
-        <v>223</v>
-      </c>
-      <c r="O17" s="13">
+      <c r="O17" s="126" t="s">
+        <v>222</v>
+      </c>
+      <c r="P17" s="13">
         <v>1.9900000000000001E-2</v>
       </c>
-      <c r="P17" s="85">
+      <c r="Q17" s="85">
         <f t="shared" si="2"/>
         <v>0.39800000000000002</v>
       </c>
-      <c r="Q17" s="13">
+      <c r="R17" s="13">
         <v>1.9900000000000001E-2</v>
       </c>
-      <c r="R17" s="85">
+      <c r="S17" s="85">
         <f t="shared" si="0"/>
         <v>0.39800000000000002</v>
       </c>
-      <c r="S17" s="117"/>
+      <c r="T17" s="117"/>
     </row>
-    <row r="18" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="27">
         <v>16</v>
       </c>
@@ -3555,7 +3592,7 @@
         <v>45</v>
       </c>
       <c r="D18" s="49" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="E18" s="14" t="s">
         <v>162</v>
@@ -3567,7 +3604,7 @@
         <v>148</v>
       </c>
       <c r="H18" s="140" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="I18" s="45" t="s">
         <v>161</v>
@@ -3578,35 +3615,36 @@
       <c r="K18" s="16">
         <v>5</v>
       </c>
-      <c r="L18" s="17">
+      <c r="L18" s="16"/>
+      <c r="M18" s="17">
         <v>2</v>
       </c>
-      <c r="M18" s="16">
+      <c r="N18" s="16">
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
-      <c r="N18" s="118" t="s">
-        <v>338</v>
-      </c>
-      <c r="O18" s="18">
+      <c r="O18" s="118" t="s">
+        <v>336</v>
+      </c>
+      <c r="P18" s="18">
         <v>2.9</v>
       </c>
-      <c r="P18" s="19">
-        <f>O18*L18</f>
+      <c r="Q18" s="19">
+        <f>P18*M18</f>
         <v>5.8</v>
       </c>
-      <c r="Q18" s="18">
+      <c r="R18" s="18">
         <v>2.9</v>
       </c>
-      <c r="R18" s="79">
+      <c r="S18" s="79">
         <f t="shared" si="0"/>
         <v>29</v>
       </c>
-      <c r="S18" s="141" t="s">
-        <v>275</v>
+      <c r="T18" s="141" t="s">
+        <v>274</v>
       </c>
     </row>
-    <row r="19" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="27">
         <v>17</v>
       </c>
@@ -3627,7 +3665,7 @@
         <v>149</v>
       </c>
       <c r="H19" s="9" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="I19" s="47" t="s">
         <v>161</v>
@@ -3638,33 +3676,34 @@
       <c r="K19" s="10">
         <v>1</v>
       </c>
-      <c r="L19" s="9">
+      <c r="L19" s="10"/>
+      <c r="M19" s="9">
         <v>1</v>
       </c>
-      <c r="M19" s="10">
+      <c r="N19" s="10">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="N19" s="21" t="s">
-        <v>223</v>
-      </c>
-      <c r="O19" s="13">
+      <c r="O19" s="21" t="s">
+        <v>222</v>
+      </c>
+      <c r="P19" s="13">
         <v>0.35360000000000003</v>
       </c>
-      <c r="P19" s="85">
+      <c r="Q19" s="85">
         <f t="shared" si="2"/>
         <v>0.35360000000000003</v>
       </c>
-      <c r="Q19" s="13">
+      <c r="R19" s="13">
         <v>0.35360000000000003</v>
       </c>
-      <c r="R19" s="136">
+      <c r="S19" s="136">
         <f t="shared" si="0"/>
         <v>1.7680000000000002</v>
       </c>
-      <c r="S19" s="142"/>
+      <c r="T19" s="142"/>
     </row>
-    <row r="20" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="27">
         <v>18</v>
       </c>
@@ -3687,7 +3726,7 @@
         <v>39</v>
       </c>
       <c r="H20" s="99" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="I20" s="100" t="s">
         <v>161</v>
@@ -3698,33 +3737,34 @@
       <c r="K20" s="101">
         <v>50</v>
       </c>
-      <c r="L20" s="99">
+      <c r="L20" s="101"/>
+      <c r="M20" s="99">
         <v>2</v>
       </c>
-      <c r="M20" s="101">
+      <c r="N20" s="101">
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
-      <c r="N20" s="102" t="s">
-        <v>223</v>
-      </c>
-      <c r="O20" s="89">
+      <c r="O20" s="102" t="s">
+        <v>222</v>
+      </c>
+      <c r="P20" s="89">
         <v>2.8299999999999999E-2</v>
       </c>
-      <c r="P20" s="83">
+      <c r="Q20" s="83">
         <f t="shared" si="2"/>
         <v>1.415</v>
       </c>
-      <c r="Q20" s="89">
+      <c r="R20" s="89">
         <v>2.8299999999999999E-2</v>
       </c>
-      <c r="R20" s="83">
+      <c r="S20" s="83">
         <f t="shared" si="0"/>
         <v>0.28299999999999997</v>
       </c>
-      <c r="S20" s="139"/>
+      <c r="T20" s="139"/>
     </row>
-    <row r="21" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="27">
         <v>19</v>
       </c>
@@ -3745,7 +3785,7 @@
         <v>57</v>
       </c>
       <c r="H21" s="6" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="I21" s="48" t="s">
         <v>161</v>
@@ -3756,32 +3796,33 @@
       <c r="K21" s="34">
         <v>1</v>
       </c>
-      <c r="L21" s="37">
+      <c r="L21" s="34"/>
+      <c r="M21" s="37">
         <v>1</v>
       </c>
-      <c r="M21" s="36">
+      <c r="N21" s="36">
         <v>6</v>
       </c>
-      <c r="N21" s="1" t="s">
-        <v>223</v>
-      </c>
-      <c r="O21" s="38">
+      <c r="O21" s="1" t="s">
+        <v>222</v>
+      </c>
+      <c r="P21" s="38">
         <v>0.2087</v>
       </c>
-      <c r="P21" s="11">
+      <c r="Q21" s="11">
         <f t="shared" si="2"/>
         <v>0.2087</v>
       </c>
-      <c r="Q21" s="38">
+      <c r="R21" s="38">
         <v>0.2087</v>
       </c>
-      <c r="R21" s="11">
+      <c r="S21" s="11">
         <f t="shared" si="0"/>
         <v>1.2522</v>
       </c>
-      <c r="S21" s="39"/>
+      <c r="T21" s="39"/>
     </row>
-    <row r="22" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="27">
         <v>20</v>
       </c>
@@ -3790,7 +3831,7 @@
         <v>54</v>
       </c>
       <c r="D22" s="91" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="E22" s="92" t="s">
         <v>168</v>
@@ -3802,10 +3843,10 @@
         <v>57</v>
       </c>
       <c r="H22" s="144" t="s">
+        <v>275</v>
+      </c>
+      <c r="I22" s="100" t="s">
         <v>276</v>
-      </c>
-      <c r="I22" s="100" t="s">
-        <v>277</v>
       </c>
       <c r="J22" s="97" t="s">
         <v>158</v>
@@ -3813,35 +3854,36 @@
       <c r="K22" s="101">
         <v>50</v>
       </c>
-      <c r="L22" s="99">
+      <c r="L22" s="101"/>
+      <c r="M22" s="99">
         <v>1</v>
       </c>
-      <c r="M22" s="101">
+      <c r="N22" s="101">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="N22" s="93" t="s">
-        <v>223</v>
-      </c>
-      <c r="O22" s="94">
+      <c r="O22" s="93" t="s">
+        <v>222</v>
+      </c>
+      <c r="P22" s="94">
         <v>2.0199999999999999E-2</v>
       </c>
-      <c r="P22" s="83">
+      <c r="Q22" s="83">
         <f t="shared" si="2"/>
         <v>1.01</v>
       </c>
-      <c r="Q22" s="94">
+      <c r="R22" s="94">
         <v>2.0199999999999999E-2</v>
       </c>
-      <c r="R22" s="83">
+      <c r="S22" s="83">
         <f t="shared" si="0"/>
         <v>0.10099999999999999</v>
       </c>
-      <c r="S22" s="109" t="s">
+      <c r="T22" s="109" t="s">
         <v>167</v>
       </c>
     </row>
-    <row r="23" spans="1:19" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:20" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="27">
         <v>21</v>
       </c>
@@ -3852,7 +3894,7 @@
         <v>58</v>
       </c>
       <c r="D23" s="49" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="E23" s="14" t="s">
         <v>59</v>
@@ -3864,10 +3906,10 @@
         <v>150</v>
       </c>
       <c r="H23" s="17" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="I23" s="17" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="J23" s="14" t="s">
         <v>133</v>
@@ -3875,34 +3917,35 @@
       <c r="K23" s="16">
         <v>10</v>
       </c>
-      <c r="L23" s="17">
+      <c r="L23" s="16"/>
+      <c r="M23" s="17">
         <v>7</v>
       </c>
-      <c r="M23" s="16">
+      <c r="N23" s="16">
         <v>40</v>
       </c>
-      <c r="N23" s="15" t="s">
-        <v>223</v>
-      </c>
-      <c r="O23" s="18">
+      <c r="O23" s="15" t="s">
+        <v>222</v>
+      </c>
+      <c r="P23" s="18">
         <v>5.91E-2</v>
       </c>
-      <c r="P23" s="79">
+      <c r="Q23" s="79">
         <f t="shared" si="2"/>
         <v>0.59099999999999997</v>
       </c>
-      <c r="Q23" s="18">
+      <c r="R23" s="18">
         <v>5.91E-2</v>
       </c>
-      <c r="R23" s="79">
+      <c r="S23" s="79">
         <f t="shared" si="0"/>
         <v>2.3639999999999999</v>
       </c>
-      <c r="S23" s="110" t="s">
+      <c r="T23" s="110" t="s">
         <v>167</v>
       </c>
     </row>
-    <row r="24" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="27">
         <v>22</v>
       </c>
@@ -3923,7 +3966,7 @@
         <v>64</v>
       </c>
       <c r="H24" s="6" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="I24" s="46" t="s">
         <v>161</v>
@@ -3934,90 +3977,92 @@
       <c r="K24" s="5">
         <v>100</v>
       </c>
-      <c r="L24" s="6">
+      <c r="L24" s="5"/>
+      <c r="M24" s="6">
         <v>1</v>
       </c>
-      <c r="M24" s="5">
+      <c r="N24" s="5">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="N24" s="1" t="s">
-        <v>223</v>
-      </c>
-      <c r="O24" s="12">
+      <c r="O24" s="1" t="s">
+        <v>222</v>
+      </c>
+      <c r="P24" s="12">
         <v>1.6000000000000001E-3</v>
       </c>
-      <c r="P24" s="11">
+      <c r="Q24" s="11">
         <f t="shared" si="2"/>
         <v>0.16</v>
       </c>
-      <c r="Q24" s="12">
+      <c r="R24" s="12">
         <v>1.6000000000000001E-3</v>
       </c>
-      <c r="R24" s="11">
+      <c r="S24" s="11">
         <f t="shared" si="0"/>
         <v>8.0000000000000002E-3</v>
       </c>
-      <c r="S24" s="7"/>
+      <c r="T24" s="7"/>
     </row>
-    <row r="25" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="27">
         <v>23</v>
       </c>
       <c r="B25" s="167"/>
       <c r="C25" s="25" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="D25" s="50" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="E25" s="4" t="s">
         <v>59</v>
       </c>
       <c r="F25" s="4" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="G25" s="1" t="s">
         <v>64</v>
       </c>
       <c r="H25" s="6" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="I25" s="46" t="s">
         <v>161</v>
       </c>
       <c r="J25" s="4" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="K25" s="5">
         <v>100</v>
       </c>
-      <c r="L25" s="6">
+      <c r="L25" s="5"/>
+      <c r="M25" s="6">
         <v>1</v>
       </c>
-      <c r="M25" s="5">
+      <c r="N25" s="5">
         <v>5</v>
       </c>
-      <c r="N25" s="111" t="s">
-        <v>223</v>
-      </c>
-      <c r="O25" s="12">
+      <c r="O25" s="111" t="s">
+        <v>222</v>
+      </c>
+      <c r="P25" s="12">
         <v>1.1999999999999999E-3</v>
       </c>
-      <c r="P25" s="11">
+      <c r="Q25" s="11">
         <f t="shared" si="2"/>
         <v>0.12</v>
       </c>
-      <c r="Q25" s="12">
+      <c r="R25" s="12">
         <v>1.1999999999999999E-3</v>
       </c>
-      <c r="R25" s="11">
+      <c r="S25" s="11">
         <f t="shared" si="0"/>
         <v>5.9999999999999993E-3</v>
       </c>
-      <c r="S25" s="7"/>
+      <c r="T25" s="7"/>
     </row>
-    <row r="26" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" s="27">
         <v>24</v>
       </c>
@@ -4026,7 +4071,7 @@
         <v>178</v>
       </c>
       <c r="D26" s="50" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="E26" s="4" t="s">
         <v>59</v>
@@ -4038,7 +4083,7 @@
         <v>64</v>
       </c>
       <c r="H26" s="6" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="I26" s="46" t="s">
         <v>161</v>
@@ -4049,33 +4094,34 @@
       <c r="K26" s="34">
         <v>100</v>
       </c>
-      <c r="L26" s="37">
+      <c r="L26" s="34"/>
+      <c r="M26" s="37">
         <v>1</v>
       </c>
-      <c r="M26" s="36">
+      <c r="N26" s="36">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="N26" s="35" t="s">
-        <v>223</v>
-      </c>
-      <c r="O26" s="38">
+      <c r="O26" s="35" t="s">
+        <v>222</v>
+      </c>
+      <c r="P26" s="38">
         <v>2E-3</v>
       </c>
-      <c r="P26" s="11">
+      <c r="Q26" s="11">
         <f t="shared" si="2"/>
         <v>0.2</v>
       </c>
-      <c r="Q26" s="38">
+      <c r="R26" s="38">
         <v>2E-3</v>
       </c>
-      <c r="R26" s="11">
+      <c r="S26" s="11">
         <f t="shared" si="0"/>
         <v>0.01</v>
       </c>
-      <c r="S26" s="42"/>
+      <c r="T26" s="42"/>
     </row>
-    <row r="27" spans="1:19" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:20" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="27">
         <v>25</v>
       </c>
@@ -4084,7 +4130,7 @@
         <v>184</v>
       </c>
       <c r="D27" s="50" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="E27" s="4" t="s">
         <v>59</v>
@@ -4096,10 +4142,10 @@
         <v>150</v>
       </c>
       <c r="H27" s="6" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="I27" s="46" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="J27" s="4" t="s">
         <v>186</v>
@@ -4107,35 +4153,36 @@
       <c r="K27" s="4">
         <v>20</v>
       </c>
-      <c r="L27" s="6">
+      <c r="L27" s="4"/>
+      <c r="M27" s="6">
         <v>3</v>
       </c>
-      <c r="M27" s="5">
+      <c r="N27" s="5">
         <f t="shared" si="1"/>
         <v>15</v>
       </c>
-      <c r="N27" s="1" t="s">
-        <v>223</v>
-      </c>
-      <c r="O27" s="12">
+      <c r="O27" s="1" t="s">
+        <v>222</v>
+      </c>
+      <c r="P27" s="12">
         <v>3.7600000000000001E-2</v>
       </c>
-      <c r="P27" s="11">
+      <c r="Q27" s="11">
         <f t="shared" si="2"/>
         <v>0.752</v>
       </c>
-      <c r="Q27" s="12">
+      <c r="R27" s="12">
         <v>3.7600000000000001E-2</v>
       </c>
-      <c r="R27" s="11">
+      <c r="S27" s="11">
         <f t="shared" si="0"/>
         <v>0.56400000000000006</v>
       </c>
-      <c r="S27" s="105" t="s">
+      <c r="T27" s="105" t="s">
         <v>167</v>
       </c>
     </row>
-    <row r="28" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="27">
         <v>26</v>
       </c>
@@ -4144,7 +4191,7 @@
         <v>65</v>
       </c>
       <c r="D28" s="50" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="E28" s="4" t="s">
         <v>59</v>
@@ -4156,10 +4203,10 @@
         <v>152</v>
       </c>
       <c r="H28" s="6" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="I28" s="46" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="J28" s="4" t="s">
         <v>135</v>
@@ -4167,35 +4214,36 @@
       <c r="K28" s="4">
         <v>100</v>
       </c>
-      <c r="L28" s="6">
+      <c r="L28" s="4"/>
+      <c r="M28" s="6">
         <v>1</v>
       </c>
-      <c r="M28" s="5">
+      <c r="N28" s="5">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="N28" s="1" t="s">
-        <v>223</v>
-      </c>
-      <c r="O28" s="12">
+      <c r="O28" s="1" t="s">
+        <v>222</v>
+      </c>
+      <c r="P28" s="12">
         <v>2.3999999999999998E-3</v>
       </c>
-      <c r="P28" s="11">
+      <c r="Q28" s="11">
         <f t="shared" si="2"/>
         <v>0.24</v>
       </c>
-      <c r="Q28" s="12">
+      <c r="R28" s="12">
         <v>2.3999999999999998E-3</v>
       </c>
-      <c r="R28" s="11">
+      <c r="S28" s="11">
         <f t="shared" si="0"/>
         <v>1.1999999999999999E-2</v>
       </c>
-      <c r="S28" s="105" t="s">
+      <c r="T28" s="105" t="s">
         <v>167</v>
       </c>
     </row>
-    <row r="29" spans="1:19" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:20" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A29" s="27">
         <v>27</v>
       </c>
@@ -4204,7 +4252,7 @@
         <v>67</v>
       </c>
       <c r="D29" s="50" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="E29" s="4" t="s">
         <v>59</v>
@@ -4216,9 +4264,9 @@
         <v>154</v>
       </c>
       <c r="H29" s="6" t="s">
-        <v>253</v>
-      </c>
-      <c r="I29" s="46" t="s">
+        <v>252</v>
+      </c>
+      <c r="I29" s="177" t="s">
         <v>161</v>
       </c>
       <c r="J29" s="4" t="s">
@@ -4227,33 +4275,34 @@
       <c r="K29" s="4">
         <v>20</v>
       </c>
-      <c r="L29" s="6">
+      <c r="L29" s="4"/>
+      <c r="M29" s="6">
         <v>1</v>
       </c>
-      <c r="M29" s="5">
+      <c r="N29" s="5">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="N29" s="1" t="s">
-        <v>223</v>
-      </c>
-      <c r="O29" s="12">
+      <c r="O29" s="1" t="s">
+        <v>222</v>
+      </c>
+      <c r="P29" s="12">
         <v>2.2100000000000002E-2</v>
       </c>
-      <c r="P29" s="11">
+      <c r="Q29" s="11">
         <f t="shared" si="2"/>
         <v>0.44200000000000006</v>
       </c>
-      <c r="Q29" s="12">
+      <c r="R29" s="12">
         <v>2.2100000000000002E-2</v>
       </c>
-      <c r="R29" s="11">
+      <c r="S29" s="11">
         <f t="shared" si="0"/>
         <v>0.11050000000000001</v>
       </c>
-      <c r="S29" s="7"/>
+      <c r="T29" s="7"/>
     </row>
-    <row r="30" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="27">
         <v>28</v>
       </c>
@@ -4262,7 +4311,7 @@
         <v>69</v>
       </c>
       <c r="D30" s="50" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="E30" s="4" t="s">
         <v>59</v>
@@ -4274,10 +4323,10 @@
         <v>155</v>
       </c>
       <c r="H30" s="6" t="s">
+        <v>237</v>
+      </c>
+      <c r="I30" s="6" t="s">
         <v>238</v>
-      </c>
-      <c r="I30" s="6" t="s">
-        <v>239</v>
       </c>
       <c r="J30" s="4" t="s">
         <v>137</v>
@@ -4285,35 +4334,36 @@
       <c r="K30" s="5">
         <v>20</v>
       </c>
-      <c r="L30" s="6">
+      <c r="L30" s="5"/>
+      <c r="M30" s="6">
         <v>4</v>
       </c>
-      <c r="M30" s="5">
+      <c r="N30" s="5">
         <f t="shared" si="1"/>
         <v>20</v>
       </c>
-      <c r="N30" s="1" t="s">
-        <v>223</v>
-      </c>
-      <c r="O30" s="12">
+      <c r="O30" s="1" t="s">
+        <v>222</v>
+      </c>
+      <c r="P30" s="12">
         <v>3.7600000000000001E-2</v>
       </c>
-      <c r="P30" s="11">
+      <c r="Q30" s="11">
         <f t="shared" si="2"/>
         <v>0.752</v>
       </c>
-      <c r="Q30" s="12">
+      <c r="R30" s="12">
         <v>3.7600000000000001E-2</v>
       </c>
-      <c r="R30" s="11">
+      <c r="S30" s="11">
         <f t="shared" si="0"/>
         <v>0.752</v>
       </c>
-      <c r="S30" s="105" t="s">
+      <c r="T30" s="105" t="s">
         <v>167</v>
       </c>
     </row>
-    <row r="31" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="27">
         <v>29</v>
       </c>
@@ -4334,10 +4384,10 @@
         <v>155</v>
       </c>
       <c r="H31" s="6" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="I31" s="6" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="J31" s="4" t="s">
         <v>138</v>
@@ -4345,35 +4395,36 @@
       <c r="K31" s="5">
         <v>100</v>
       </c>
-      <c r="L31" s="6">
+      <c r="L31" s="5"/>
+      <c r="M31" s="6">
         <v>1</v>
       </c>
-      <c r="M31" s="5">
+      <c r="N31" s="5">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="N31" s="1" t="s">
-        <v>223</v>
-      </c>
-      <c r="O31" s="12">
+      <c r="O31" s="1" t="s">
+        <v>222</v>
+      </c>
+      <c r="P31" s="12">
         <v>1.1999999999999999E-3</v>
       </c>
-      <c r="P31" s="11">
+      <c r="Q31" s="11">
         <f t="shared" si="2"/>
         <v>0.12</v>
       </c>
-      <c r="Q31" s="12">
+      <c r="R31" s="12">
         <v>1.1999999999999999E-3</v>
       </c>
-      <c r="R31" s="11">
+      <c r="S31" s="11">
         <f t="shared" si="0"/>
         <v>5.9999999999999993E-3</v>
       </c>
-      <c r="S31" s="105" t="s">
+      <c r="T31" s="105" t="s">
         <v>167</v>
       </c>
     </row>
-    <row r="32" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="27">
         <v>30</v>
       </c>
@@ -4394,10 +4445,10 @@
         <v>183</v>
       </c>
       <c r="H32" s="6" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="I32" s="46" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="J32" s="4" t="s">
         <v>139</v>
@@ -4405,35 +4456,36 @@
       <c r="K32" s="4">
         <v>10</v>
       </c>
-      <c r="L32" s="37">
+      <c r="L32" s="4"/>
+      <c r="M32" s="37">
         <v>1</v>
       </c>
-      <c r="M32" s="36">
+      <c r="N32" s="36">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="N32" s="1" t="s">
-        <v>223</v>
-      </c>
-      <c r="O32" s="38">
+      <c r="O32" s="1" t="s">
+        <v>222</v>
+      </c>
+      <c r="P32" s="38">
         <v>4.19E-2</v>
       </c>
-      <c r="P32" s="11">
+      <c r="Q32" s="11">
         <f t="shared" si="2"/>
         <v>0.41899999999999998</v>
       </c>
-      <c r="Q32" s="38">
+      <c r="R32" s="38">
         <v>4.19E-2</v>
       </c>
-      <c r="R32" s="11">
+      <c r="S32" s="11">
         <f t="shared" si="0"/>
         <v>0.20949999999999999</v>
       </c>
-      <c r="S32" s="105" t="s">
+      <c r="T32" s="105" t="s">
         <v>167</v>
       </c>
     </row>
-    <row r="33" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A33" s="27">
         <v>31</v>
       </c>
@@ -4454,10 +4506,10 @@
         <v>155</v>
       </c>
       <c r="H33" s="6" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="I33" s="6" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="J33" s="4" t="s">
         <v>140</v>
@@ -4465,35 +4517,36 @@
       <c r="K33" s="5">
         <v>100</v>
       </c>
-      <c r="L33" s="6">
+      <c r="L33" s="5"/>
+      <c r="M33" s="6">
         <v>1</v>
       </c>
-      <c r="M33" s="5">
+      <c r="N33" s="5">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="N33" s="1" t="s">
-        <v>223</v>
-      </c>
-      <c r="O33" s="12">
+      <c r="O33" s="1" t="s">
+        <v>222</v>
+      </c>
+      <c r="P33" s="12">
         <v>1.4E-3</v>
       </c>
-      <c r="P33" s="11">
+      <c r="Q33" s="11">
         <f t="shared" si="2"/>
         <v>0.13999999999999999</v>
       </c>
-      <c r="Q33" s="12">
+      <c r="R33" s="12">
         <v>1.4E-3</v>
       </c>
-      <c r="R33" s="11">
+      <c r="S33" s="11">
         <f t="shared" si="0"/>
         <v>7.0000000000000001E-3</v>
       </c>
-      <c r="S33" s="105" t="s">
+      <c r="T33" s="105" t="s">
         <v>167</v>
       </c>
     </row>
-    <row r="34" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A34" s="27">
         <v>32</v>
       </c>
@@ -4514,10 +4567,10 @@
         <v>153</v>
       </c>
       <c r="H34" s="6" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="I34" s="73" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="J34" s="4" t="s">
         <v>141</v>
@@ -4525,35 +4578,36 @@
       <c r="K34" s="5">
         <v>100</v>
       </c>
-      <c r="L34" s="6">
+      <c r="L34" s="5"/>
+      <c r="M34" s="6">
         <v>1</v>
       </c>
-      <c r="M34" s="5">
+      <c r="N34" s="5">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="N34" s="1" t="s">
-        <v>223</v>
-      </c>
-      <c r="O34" s="12">
+      <c r="O34" s="1" t="s">
+        <v>222</v>
+      </c>
+      <c r="P34" s="12">
         <v>1.4E-3</v>
       </c>
-      <c r="P34" s="11">
+      <c r="Q34" s="11">
         <f t="shared" si="2"/>
         <v>0.13999999999999999</v>
       </c>
-      <c r="Q34" s="12">
+      <c r="R34" s="12">
         <v>1.4E-3</v>
       </c>
-      <c r="R34" s="11">
+      <c r="S34" s="11">
         <f t="shared" si="0"/>
         <v>7.0000000000000001E-3</v>
       </c>
-      <c r="S34" s="105" t="s">
+      <c r="T34" s="105" t="s">
         <v>167</v>
       </c>
     </row>
-    <row r="35" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A35" s="27">
         <v>33</v>
       </c>
@@ -4574,10 +4628,10 @@
         <v>151</v>
       </c>
       <c r="H35" s="9" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="I35" s="145" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="J35" s="8" t="s">
         <v>142</v>
@@ -4585,35 +4639,36 @@
       <c r="K35" s="10">
         <v>100</v>
       </c>
-      <c r="L35" s="9">
+      <c r="L35" s="10"/>
+      <c r="M35" s="9">
         <v>4</v>
       </c>
-      <c r="M35" s="10">
+      <c r="N35" s="10">
         <f t="shared" si="1"/>
         <v>20</v>
       </c>
-      <c r="N35" s="21" t="s">
-        <v>223</v>
-      </c>
-      <c r="O35" s="13">
+      <c r="O35" s="21" t="s">
+        <v>222</v>
+      </c>
+      <c r="P35" s="13">
         <v>1.8E-3</v>
       </c>
-      <c r="P35" s="136">
+      <c r="Q35" s="136">
         <f t="shared" si="2"/>
         <v>0.18</v>
       </c>
-      <c r="Q35" s="13">
+      <c r="R35" s="13">
         <v>1.8E-3</v>
       </c>
-      <c r="R35" s="136">
+      <c r="S35" s="136">
         <f t="shared" si="0"/>
         <v>3.5999999999999997E-2</v>
       </c>
-      <c r="S35" s="117" t="s">
+      <c r="T35" s="117" t="s">
         <v>167</v>
       </c>
     </row>
-    <row r="36" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A36" s="27">
         <v>34</v>
       </c>
@@ -4636,9 +4691,9 @@
         <v>189</v>
       </c>
       <c r="H36" s="99" t="s">
-        <v>258</v>
-      </c>
-      <c r="I36" s="100" t="s">
+        <v>257</v>
+      </c>
+      <c r="I36" s="178" t="s">
         <v>161</v>
       </c>
       <c r="J36" s="97" t="s">
@@ -4647,33 +4702,34 @@
       <c r="K36" s="97">
         <v>1</v>
       </c>
-      <c r="L36" s="99">
+      <c r="L36" s="97"/>
+      <c r="M36" s="99">
         <v>1</v>
       </c>
-      <c r="M36" s="101">
+      <c r="N36" s="101">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="N36" s="102" t="s">
-        <v>223</v>
-      </c>
-      <c r="O36" s="103">
+      <c r="O36" s="102" t="s">
+        <v>222</v>
+      </c>
+      <c r="P36" s="103">
         <v>0.25850000000000001</v>
       </c>
-      <c r="P36" s="83">
+      <c r="Q36" s="83">
         <f t="shared" si="2"/>
         <v>0.25850000000000001</v>
       </c>
-      <c r="Q36" s="103">
+      <c r="R36" s="103">
         <v>0.25850000000000001</v>
       </c>
-      <c r="R36" s="80">
+      <c r="S36" s="80">
         <f t="shared" si="0"/>
         <v>1.2925</v>
       </c>
-      <c r="S36" s="107"/>
+      <c r="T36" s="107"/>
     </row>
-    <row r="37" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A37" s="27">
         <v>35</v>
       </c>
@@ -4696,9 +4752,9 @@
         <v>89</v>
       </c>
       <c r="H37" s="17" t="s">
-        <v>259</v>
-      </c>
-      <c r="I37" s="49" t="s">
+        <v>258</v>
+      </c>
+      <c r="I37" s="84" t="s">
         <v>161</v>
       </c>
       <c r="J37" s="49" t="s">
@@ -4707,33 +4763,34 @@
       <c r="K37" s="49">
         <v>1</v>
       </c>
-      <c r="L37" s="70">
+      <c r="L37" s="49"/>
+      <c r="M37" s="70">
         <v>1</v>
       </c>
-      <c r="M37" s="70">
+      <c r="N37" s="70">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="N37" s="104" t="s">
-        <v>223</v>
-      </c>
-      <c r="O37" s="71">
+      <c r="O37" s="104" t="s">
+        <v>222</v>
+      </c>
+      <c r="P37" s="71">
         <v>4.0141</v>
       </c>
-      <c r="P37" s="79">
+      <c r="Q37" s="79">
         <f t="shared" si="2"/>
         <v>4.0141</v>
       </c>
-      <c r="Q37" s="71">
+      <c r="R37" s="71">
         <v>4.0141</v>
       </c>
-      <c r="R37" s="79">
+      <c r="S37" s="79">
         <f t="shared" si="0"/>
         <v>20.070499999999999</v>
       </c>
-      <c r="S37" s="108"/>
+      <c r="T37" s="108"/>
     </row>
-    <row r="38" spans="1:19" s="124" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:20" s="124" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A38" s="27">
         <v>36</v>
       </c>
@@ -4756,7 +4813,7 @@
       <c r="H38" s="6" t="s">
         <v>158</v>
       </c>
-      <c r="I38" s="46" t="s">
+      <c r="I38" s="177" t="s">
         <v>161</v>
       </c>
       <c r="J38" s="34" t="s">
@@ -4765,35 +4822,36 @@
       <c r="K38" s="34">
         <v>1</v>
       </c>
-      <c r="L38" s="37">
+      <c r="L38" s="34"/>
+      <c r="M38" s="37">
         <v>1</v>
       </c>
-      <c r="M38" s="36">
+      <c r="N38" s="36">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="N38" s="177" t="s">
-        <v>338</v>
-      </c>
-      <c r="O38" s="38">
+      <c r="O38" s="160" t="s">
+        <v>336</v>
+      </c>
+      <c r="P38" s="38">
         <v>1.6</v>
       </c>
-      <c r="P38" s="11">
+      <c r="Q38" s="11">
         <f t="shared" si="2"/>
         <v>1.6</v>
       </c>
-      <c r="Q38" s="38">
+      <c r="R38" s="38">
         <v>1.6</v>
       </c>
-      <c r="R38" s="11">
+      <c r="S38" s="11">
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
-      <c r="S38" s="106" t="s">
-        <v>280</v>
+      <c r="T38" s="106" t="s">
+        <v>279</v>
       </c>
     </row>
-    <row r="39" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A39" s="27">
         <v>37</v>
       </c>
@@ -4814,7 +4872,7 @@
         <v>106</v>
       </c>
       <c r="H39" s="3"/>
-      <c r="I39" s="46" t="s">
+      <c r="I39" s="177" t="s">
         <v>161</v>
       </c>
       <c r="J39" s="4" t="s">
@@ -4823,35 +4881,36 @@
       <c r="K39" s="4">
         <v>1</v>
       </c>
-      <c r="L39" s="6">
+      <c r="L39" s="4"/>
+      <c r="M39" s="6">
         <v>1</v>
       </c>
-      <c r="M39" s="5">
+      <c r="N39" s="5">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="N39" s="177" t="s">
-        <v>338</v>
-      </c>
-      <c r="O39" s="12">
+      <c r="O39" s="160" t="s">
+        <v>336</v>
+      </c>
+      <c r="P39" s="12">
         <v>1.5</v>
       </c>
-      <c r="P39" s="11">
-        <f>O39*L39</f>
+      <c r="Q39" s="11">
+        <f>P39*M39</f>
         <v>1.5</v>
       </c>
-      <c r="Q39" s="12">
+      <c r="R39" s="12">
         <v>1.5</v>
       </c>
-      <c r="R39" s="11">
+      <c r="S39" s="11">
         <f t="shared" si="0"/>
         <v>7.5</v>
       </c>
-      <c r="S39" s="109" t="s">
-        <v>339</v>
+      <c r="T39" s="109" t="s">
+        <v>337</v>
       </c>
     </row>
-    <row r="40" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A40" s="27">
         <v>38</v>
       </c>
@@ -4872,9 +4931,9 @@
         <v>194</v>
       </c>
       <c r="H40" s="6" t="s">
-        <v>260</v>
-      </c>
-      <c r="I40" s="46" t="s">
+        <v>259</v>
+      </c>
+      <c r="I40" s="177" t="s">
         <v>161</v>
       </c>
       <c r="J40" s="4" t="s">
@@ -4883,33 +4942,34 @@
       <c r="K40" s="4">
         <v>1</v>
       </c>
-      <c r="L40" s="6">
+      <c r="L40" s="4"/>
+      <c r="M40" s="6">
         <v>1</v>
       </c>
-      <c r="M40" s="5">
+      <c r="N40" s="5">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="N40" s="1" t="s">
-        <v>223</v>
-      </c>
-      <c r="O40" s="12">
+      <c r="O40" s="1" t="s">
+        <v>222</v>
+      </c>
+      <c r="P40" s="12">
         <v>3.0926999999999998</v>
       </c>
-      <c r="P40" s="11">
+      <c r="Q40" s="11">
         <f t="shared" si="2"/>
         <v>3.0926999999999998</v>
       </c>
-      <c r="Q40" s="12">
+      <c r="R40" s="12">
         <v>3.0926999999999998</v>
       </c>
-      <c r="R40" s="11">
+      <c r="S40" s="11">
         <f t="shared" si="0"/>
         <v>15.4635</v>
       </c>
-      <c r="S40" s="105"/>
+      <c r="T40" s="105"/>
     </row>
-    <row r="41" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A41" s="27">
         <v>39</v>
       </c>
@@ -4921,7 +4981,7 @@
         <v>100</v>
       </c>
       <c r="E41" s="81" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="F41" s="34" t="s">
         <v>101</v>
@@ -4930,9 +4990,9 @@
         <v>102</v>
       </c>
       <c r="H41" s="6" t="s">
-        <v>261</v>
-      </c>
-      <c r="I41" s="46" t="s">
+        <v>260</v>
+      </c>
+      <c r="I41" s="177" t="s">
         <v>161</v>
       </c>
       <c r="J41" s="34" t="s">
@@ -4941,33 +5001,34 @@
       <c r="K41" s="34">
         <v>1</v>
       </c>
-      <c r="L41" s="37">
+      <c r="L41" s="34"/>
+      <c r="M41" s="37">
         <v>1</v>
       </c>
-      <c r="M41" s="36">
+      <c r="N41" s="36">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="N41" s="35" t="s">
-        <v>223</v>
-      </c>
-      <c r="O41" s="38">
+      <c r="O41" s="35" t="s">
+        <v>222</v>
+      </c>
+      <c r="P41" s="38">
         <v>0.76100000000000001</v>
       </c>
-      <c r="P41" s="11">
+      <c r="Q41" s="11">
         <f t="shared" si="2"/>
         <v>0.76100000000000001</v>
       </c>
-      <c r="Q41" s="38">
+      <c r="R41" s="38">
         <v>0.76100000000000001</v>
       </c>
-      <c r="R41" s="11">
+      <c r="S41" s="11">
         <f t="shared" si="0"/>
         <v>3.8050000000000002</v>
       </c>
-      <c r="S41" s="106"/>
+      <c r="T41" s="106"/>
     </row>
-    <row r="42" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A42" s="27">
         <v>40</v>
       </c>
@@ -4976,7 +5037,7 @@
         <v>103</v>
       </c>
       <c r="D42" s="51" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="E42" s="4" t="s">
         <v>104</v>
@@ -4988,9 +5049,9 @@
         <v>98</v>
       </c>
       <c r="H42" s="6" t="s">
-        <v>248</v>
-      </c>
-      <c r="I42" s="46" t="s">
+        <v>247</v>
+      </c>
+      <c r="I42" s="177" t="s">
         <v>161</v>
       </c>
       <c r="J42" s="4" t="s">
@@ -4999,33 +5060,34 @@
       <c r="K42" s="4">
         <v>1</v>
       </c>
-      <c r="L42" s="6">
+      <c r="L42" s="4"/>
+      <c r="M42" s="6">
         <v>3</v>
       </c>
-      <c r="M42" s="5">
+      <c r="N42" s="5">
         <f t="shared" si="1"/>
         <v>15</v>
       </c>
-      <c r="N42" s="1" t="s">
-        <v>223</v>
-      </c>
-      <c r="O42" s="12">
+      <c r="O42" s="1" t="s">
+        <v>222</v>
+      </c>
+      <c r="P42" s="12">
         <v>0.2137</v>
       </c>
-      <c r="P42" s="11">
-        <f>O42*L42</f>
+      <c r="Q42" s="11">
+        <f>P42*M42</f>
         <v>0.6411</v>
       </c>
-      <c r="Q42" s="12">
+      <c r="R42" s="12">
         <v>0.16619999999999999</v>
       </c>
-      <c r="R42" s="11">
+      <c r="S42" s="11">
         <f t="shared" si="0"/>
         <v>2.4929999999999999</v>
       </c>
-      <c r="S42" s="105"/>
+      <c r="T42" s="105"/>
     </row>
-    <row r="43" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A43" s="27">
         <v>41</v>
       </c>
@@ -5046,9 +5108,9 @@
         <v>203</v>
       </c>
       <c r="H43" s="6" t="s">
-        <v>263</v>
-      </c>
-      <c r="I43" s="46" t="s">
+        <v>262</v>
+      </c>
+      <c r="I43" s="177" t="s">
         <v>161</v>
       </c>
       <c r="J43" s="34" t="s">
@@ -5057,33 +5119,34 @@
       <c r="K43" s="34">
         <v>1</v>
       </c>
-      <c r="L43" s="37">
+      <c r="L43" s="34"/>
+      <c r="M43" s="37">
         <v>1</v>
       </c>
-      <c r="M43" s="36">
+      <c r="N43" s="36">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="N43" s="35" t="s">
-        <v>223</v>
-      </c>
-      <c r="O43" s="38">
+      <c r="O43" s="35" t="s">
+        <v>222</v>
+      </c>
+      <c r="P43" s="38">
         <v>0.61140000000000005</v>
       </c>
-      <c r="P43" s="11">
+      <c r="Q43" s="11">
         <f t="shared" si="2"/>
         <v>0.61140000000000005</v>
       </c>
-      <c r="Q43" s="38">
+      <c r="R43" s="38">
         <v>0.61140000000000005</v>
       </c>
-      <c r="R43" s="11">
+      <c r="S43" s="11">
         <f t="shared" si="0"/>
         <v>3.0570000000000004</v>
       </c>
-      <c r="S43" s="106"/>
+      <c r="T43" s="106"/>
     </row>
-    <row r="44" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A44" s="27">
         <v>42</v>
       </c>
@@ -5113,35 +5176,36 @@
       <c r="K44" s="4">
         <v>1</v>
       </c>
-      <c r="L44" s="6">
+      <c r="L44" s="4"/>
+      <c r="M44" s="6">
         <v>1</v>
       </c>
-      <c r="M44" s="5">
+      <c r="N44" s="5">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="N44" s="111" t="s">
-        <v>338</v>
-      </c>
-      <c r="O44" s="12">
+      <c r="O44" s="111" t="s">
+        <v>336</v>
+      </c>
+      <c r="P44" s="12">
         <v>1</v>
       </c>
-      <c r="P44" s="11">
-        <f>O44*K44</f>
+      <c r="Q44" s="11">
+        <f>P44*K44</f>
         <v>1</v>
       </c>
-      <c r="Q44" s="12">
+      <c r="R44" s="12">
         <v>1</v>
       </c>
-      <c r="R44" s="11">
+      <c r="S44" s="11">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="S44" s="106" t="s">
-        <v>278</v>
+      <c r="T44" s="106" t="s">
+        <v>277</v>
       </c>
     </row>
-    <row r="45" spans="1:19" s="124" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:20" s="124" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A45" s="27">
         <v>43</v>
       </c>
@@ -5173,35 +5237,36 @@
       <c r="K45" s="8">
         <v>1</v>
       </c>
-      <c r="L45" s="9">
+      <c r="L45" s="8"/>
+      <c r="M45" s="9">
         <v>1</v>
       </c>
-      <c r="M45" s="10">
+      <c r="N45" s="10">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="N45" s="177" t="s">
-        <v>338</v>
-      </c>
-      <c r="O45" s="13">
+      <c r="O45" s="160" t="s">
+        <v>336</v>
+      </c>
+      <c r="P45" s="13">
         <v>9.3000000000000007</v>
       </c>
-      <c r="P45" s="85">
+      <c r="Q45" s="85">
         <f t="shared" si="2"/>
         <v>9.3000000000000007</v>
       </c>
-      <c r="Q45" s="13">
+      <c r="R45" s="13">
         <v>9.3000000000000007</v>
       </c>
-      <c r="R45" s="80">
+      <c r="S45" s="80">
         <f t="shared" si="0"/>
         <v>46.5</v>
       </c>
-      <c r="S45" s="106" t="s">
-        <v>280</v>
+      <c r="T45" s="106" t="s">
+        <v>279</v>
       </c>
     </row>
-    <row r="46" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A46" s="27">
         <v>44</v>
       </c>
@@ -5212,7 +5277,7 @@
         <v>205</v>
       </c>
       <c r="D46" s="49" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="E46" s="14" t="s">
         <v>162</v>
@@ -5224,7 +5289,7 @@
         <v>111</v>
       </c>
       <c r="H46" s="78" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="I46" s="45" t="s">
         <v>161</v>
@@ -5235,33 +5300,34 @@
       <c r="K46" s="16">
         <v>20</v>
       </c>
-      <c r="L46" s="17">
+      <c r="L46" s="16"/>
+      <c r="M46" s="17">
         <v>8</v>
       </c>
-      <c r="M46" s="16">
-        <f t="shared" ref="M46:M56" si="3">L46*5</f>
+      <c r="N46" s="16">
+        <f t="shared" ref="N46:N59" si="3">M46*5</f>
         <v>40</v>
       </c>
-      <c r="N46" s="15" t="s">
-        <v>223</v>
-      </c>
-      <c r="O46" s="18">
+      <c r="O46" s="15" t="s">
+        <v>222</v>
+      </c>
+      <c r="P46" s="18">
         <v>3.1E-2</v>
       </c>
-      <c r="P46" s="79">
+      <c r="Q46" s="79">
         <f t="shared" si="2"/>
         <v>0.62</v>
       </c>
-      <c r="Q46" s="18">
+      <c r="R46" s="18">
         <v>3.1E-2</v>
       </c>
-      <c r="R46" s="79">
+      <c r="S46" s="79">
         <f t="shared" si="0"/>
         <v>1.24</v>
       </c>
-      <c r="S46" s="110"/>
+      <c r="T46" s="110"/>
     </row>
-    <row r="47" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A47" s="27">
         <v>45</v>
       </c>
@@ -5282,7 +5348,7 @@
         <v>111</v>
       </c>
       <c r="H47" s="73" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="I47" s="46" t="s">
         <v>161</v>
@@ -5293,33 +5359,34 @@
       <c r="K47" s="5">
         <v>1</v>
       </c>
-      <c r="L47" s="6">
+      <c r="L47" s="5"/>
+      <c r="M47" s="6">
         <v>3</v>
       </c>
-      <c r="M47" s="5">
+      <c r="N47" s="5">
         <f t="shared" si="3"/>
         <v>15</v>
       </c>
-      <c r="N47" s="1" t="s">
-        <v>223</v>
-      </c>
-      <c r="O47" s="12">
+      <c r="O47" s="1" t="s">
+        <v>222</v>
+      </c>
+      <c r="P47" s="12">
         <v>0.1608</v>
       </c>
-      <c r="P47" s="11">
-        <f>O47*L47</f>
+      <c r="Q47" s="11">
+        <f>P47*M47</f>
         <v>0.4824</v>
       </c>
-      <c r="Q47" s="12">
+      <c r="R47" s="12">
         <v>0.12540000000000001</v>
       </c>
-      <c r="R47" s="11">
+      <c r="S47" s="11">
         <f t="shared" si="0"/>
         <v>1.8810000000000002</v>
       </c>
-      <c r="S47" s="105"/>
+      <c r="T47" s="105"/>
     </row>
-    <row r="48" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A48" s="27">
         <v>46</v>
       </c>
@@ -5340,7 +5407,7 @@
         <v>111</v>
       </c>
       <c r="H48" s="6" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="I48" s="46" t="s">
         <v>161</v>
@@ -5351,32 +5418,33 @@
       <c r="K48" s="5">
         <v>10</v>
       </c>
-      <c r="L48" s="6">
+      <c r="L48" s="5"/>
+      <c r="M48" s="6">
         <v>5</v>
       </c>
-      <c r="M48" s="5">
+      <c r="N48" s="5">
         <v>30</v>
       </c>
-      <c r="N48" s="1" t="s">
-        <v>247</v>
-      </c>
-      <c r="O48" s="12">
+      <c r="O48" s="1" t="s">
+        <v>246</v>
+      </c>
+      <c r="P48" s="12">
         <v>4.53E-2</v>
       </c>
-      <c r="P48" s="11">
+      <c r="Q48" s="11">
         <f t="shared" si="2"/>
         <v>0.45300000000000001</v>
       </c>
-      <c r="Q48" s="12">
+      <c r="R48" s="12">
         <v>4.53E-2</v>
       </c>
-      <c r="R48" s="11">
+      <c r="S48" s="11">
         <f t="shared" si="0"/>
         <v>1.359</v>
       </c>
-      <c r="S48" s="105"/>
+      <c r="T48" s="105"/>
     </row>
-    <row r="49" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A49" s="27">
         <v>47</v>
       </c>
@@ -5397,7 +5465,7 @@
         <v>111</v>
       </c>
       <c r="H49" s="73" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="I49" s="46" t="s">
         <v>161</v>
@@ -5408,33 +5476,34 @@
       <c r="K49" s="5">
         <v>5</v>
       </c>
-      <c r="L49" s="6">
+      <c r="L49" s="5"/>
+      <c r="M49" s="6">
         <v>2</v>
       </c>
-      <c r="M49" s="5">
+      <c r="N49" s="5">
         <f t="shared" si="3"/>
         <v>10</v>
       </c>
-      <c r="N49" s="1" t="s">
-        <v>223</v>
-      </c>
-      <c r="O49" s="12">
+      <c r="O49" s="1" t="s">
+        <v>222</v>
+      </c>
+      <c r="P49" s="12">
         <v>0.1099</v>
       </c>
-      <c r="P49" s="11">
-        <f>O49*K49</f>
+      <c r="Q49" s="11">
+        <f>P49*K49</f>
         <v>0.54949999999999999</v>
       </c>
-      <c r="Q49" s="12">
+      <c r="R49" s="12">
         <v>0.1099</v>
       </c>
-      <c r="R49" s="11">
+      <c r="S49" s="11">
         <f t="shared" si="0"/>
         <v>1.099</v>
       </c>
-      <c r="S49" s="105"/>
+      <c r="T49" s="105"/>
     </row>
-    <row r="50" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A50" s="27">
         <v>48</v>
       </c>
@@ -5455,7 +5524,7 @@
         <v>123</v>
       </c>
       <c r="H50" s="6" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="I50" s="46" t="s">
         <v>161</v>
@@ -5466,33 +5535,34 @@
       <c r="K50" s="5">
         <v>1</v>
       </c>
-      <c r="L50" s="6">
+      <c r="L50" s="5"/>
+      <c r="M50" s="6">
         <v>1</v>
       </c>
-      <c r="M50" s="5">
+      <c r="N50" s="5">
         <f t="shared" si="3"/>
         <v>5</v>
       </c>
-      <c r="N50" s="1" t="s">
-        <v>223</v>
-      </c>
-      <c r="O50" s="12">
+      <c r="O50" s="1" t="s">
+        <v>222</v>
+      </c>
+      <c r="P50" s="12">
         <v>3.1720000000000002</v>
       </c>
-      <c r="P50" s="80">
+      <c r="Q50" s="80">
         <f t="shared" si="2"/>
         <v>3.1720000000000002</v>
       </c>
-      <c r="Q50" s="12">
+      <c r="R50" s="12">
         <v>3.1720000000000002</v>
       </c>
-      <c r="R50" s="80">
+      <c r="S50" s="80">
         <f t="shared" si="0"/>
         <v>15.860000000000001</v>
       </c>
-      <c r="S50" s="105"/>
+      <c r="T50" s="105"/>
     </row>
-    <row r="51" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A51" s="27">
         <v>49</v>
       </c>
@@ -5517,20 +5587,18 @@
         <v>163</v>
       </c>
       <c r="J51" s="64" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="K51" s="64"/>
-      <c r="L51" s="65">
+      <c r="L51" s="64"/>
+      <c r="M51" s="65">
         <v>1</v>
       </c>
-      <c r="M51" s="65">
+      <c r="N51" s="65">
         <f t="shared" si="3"/>
         <v>5</v>
       </c>
-      <c r="N51" s="64" t="s">
-        <v>163</v>
-      </c>
-      <c r="O51" s="66" t="s">
+      <c r="O51" s="64" t="s">
         <v>163</v>
       </c>
       <c r="P51" s="66" t="s">
@@ -5542,11 +5610,14 @@
       <c r="R51" s="66" t="s">
         <v>163</v>
       </c>
-      <c r="S51" s="67" t="s">
+      <c r="S51" s="66" t="s">
+        <v>163</v>
+      </c>
+      <c r="T51" s="67" t="s">
         <v>164</v>
       </c>
     </row>
-    <row r="52" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A52" s="27">
         <v>50</v>
       </c>
@@ -5555,7 +5626,7 @@
         <v>124</v>
       </c>
       <c r="D52" s="56" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="E52" s="56" t="s">
         <v>162</v>
@@ -5571,20 +5642,18 @@
         <v>163</v>
       </c>
       <c r="J52" s="58" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="K52" s="58"/>
-      <c r="L52" s="59">
+      <c r="L52" s="58"/>
+      <c r="M52" s="59">
         <v>4</v>
       </c>
-      <c r="M52" s="59">
+      <c r="N52" s="59">
         <f t="shared" si="3"/>
         <v>20</v>
       </c>
-      <c r="N52" s="58" t="s">
-        <v>163</v>
-      </c>
-      <c r="O52" s="60" t="s">
+      <c r="O52" s="58" t="s">
         <v>163</v>
       </c>
       <c r="P52" s="60" t="s">
@@ -5596,180 +5665,304 @@
       <c r="R52" s="60" t="s">
         <v>163</v>
       </c>
-      <c r="S52" s="61" t="s">
+      <c r="S52" s="60" t="s">
+        <v>163</v>
+      </c>
+      <c r="T52" s="61" t="s">
         <v>164</v>
       </c>
     </row>
-    <row r="53" spans="1:19" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:20" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A53" s="127">
         <v>51</v>
       </c>
       <c r="B53" s="174" t="s">
-        <v>326</v>
+        <v>347</v>
       </c>
       <c r="C53" s="146" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="D53" s="147"/>
       <c r="E53" s="14" t="s">
         <v>162</v>
       </c>
       <c r="F53" s="14" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="G53" s="148"/>
       <c r="H53" s="148"/>
       <c r="I53" s="148"/>
       <c r="J53" s="148"/>
       <c r="K53" s="148"/>
-      <c r="L53" s="149">
-        <v>3</v>
-      </c>
-      <c r="M53" s="150">
+      <c r="L53" s="179"/>
+      <c r="M53" s="149">
+        <v>2</v>
+      </c>
+      <c r="N53" s="150">
         <f t="shared" si="3"/>
-        <v>15</v>
-      </c>
-      <c r="N53" s="148"/>
-      <c r="O53" s="148"/>
+        <v>10</v>
+      </c>
+      <c r="O53" s="118" t="s">
+        <v>338</v>
+      </c>
       <c r="P53" s="148"/>
       <c r="Q53" s="148"/>
       <c r="R53" s="148"/>
-      <c r="S53" s="151"/>
+      <c r="S53" s="148"/>
+      <c r="T53" s="151"/>
     </row>
-    <row r="54" spans="1:19" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:20" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A54" s="127">
         <v>52</v>
       </c>
       <c r="B54" s="175"/>
       <c r="C54" s="129" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="D54" s="128"/>
       <c r="E54" s="4" t="s">
         <v>162</v>
       </c>
       <c r="F54" s="4" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="G54" s="128"/>
       <c r="H54" s="128"/>
       <c r="I54" s="128"/>
       <c r="J54" s="128"/>
       <c r="K54" s="128"/>
-      <c r="L54" s="130">
+      <c r="L54" s="128"/>
+      <c r="M54" s="130">
         <v>2</v>
       </c>
-      <c r="M54" s="159">
+      <c r="N54" s="158">
         <f t="shared" si="3"/>
         <v>10</v>
       </c>
-      <c r="N54" s="128"/>
-      <c r="O54" s="128"/>
+      <c r="O54" s="111" t="s">
+        <v>338</v>
+      </c>
       <c r="P54" s="128"/>
       <c r="Q54" s="128"/>
       <c r="R54" s="128"/>
-      <c r="S54" s="152"/>
+      <c r="S54" s="128"/>
+      <c r="T54" s="152"/>
     </row>
-    <row r="55" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:20" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A55" s="127">
         <v>53</v>
       </c>
       <c r="B55" s="175"/>
-      <c r="C55" s="128"/>
+      <c r="C55" s="129" t="s">
+        <v>344</v>
+      </c>
       <c r="D55" s="128"/>
-      <c r="E55" s="128"/>
-      <c r="F55" s="130" t="s">
-        <v>331</v>
+      <c r="E55" s="4" t="s">
+        <v>162</v>
+      </c>
+      <c r="F55" s="4" t="s">
+        <v>339</v>
       </c>
       <c r="G55" s="128"/>
       <c r="H55" s="128"/>
       <c r="I55" s="128"/>
       <c r="J55" s="128"/>
       <c r="K55" s="128"/>
-      <c r="L55" s="130">
+      <c r="L55" s="128"/>
+      <c r="M55" s="130">
         <v>1</v>
       </c>
-      <c r="M55" s="159">
+      <c r="N55" s="158">
         <f t="shared" si="3"/>
         <v>5</v>
       </c>
-      <c r="N55" s="128"/>
-      <c r="O55" s="128"/>
+      <c r="O55" s="111" t="s">
+        <v>338</v>
+      </c>
       <c r="P55" s="128"/>
       <c r="Q55" s="128"/>
       <c r="R55" s="128"/>
-      <c r="S55" s="152"/>
+      <c r="S55" s="128"/>
+      <c r="T55" s="152"/>
     </row>
-    <row r="56" spans="1:19" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A56" s="158">
+    <row r="56" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A56" s="127">
         <v>54</v>
       </c>
-      <c r="B56" s="176"/>
-      <c r="C56" s="160" t="s">
-        <v>337</v>
-      </c>
-      <c r="D56" s="153"/>
+      <c r="B56" s="175"/>
+      <c r="C56" s="129" t="s">
+        <v>343</v>
+      </c>
+      <c r="D56" s="128"/>
       <c r="E56" s="4" t="s">
         <v>162</v>
       </c>
-      <c r="F56" s="154" t="s">
-        <v>332</v>
-      </c>
-      <c r="G56" s="153"/>
-      <c r="H56" s="153"/>
-      <c r="I56" s="153"/>
-      <c r="J56" s="153"/>
-      <c r="K56" s="153"/>
-      <c r="L56" s="155">
+      <c r="F56" s="4" t="s">
+        <v>340</v>
+      </c>
+      <c r="G56" s="128"/>
+      <c r="H56" s="128"/>
+      <c r="I56" s="128"/>
+      <c r="J56" s="128"/>
+      <c r="K56" s="128"/>
+      <c r="L56" s="128"/>
+      <c r="M56" s="130">
         <v>1</v>
       </c>
-      <c r="M56" s="156">
+      <c r="N56" s="158">
         <f t="shared" si="3"/>
         <v>5</v>
       </c>
-      <c r="N56" s="153"/>
-      <c r="O56" s="153"/>
-      <c r="P56" s="153"/>
-      <c r="Q56" s="153"/>
-      <c r="R56" s="153"/>
-      <c r="S56" s="157"/>
+      <c r="O56" s="111"/>
+      <c r="P56" s="128"/>
+      <c r="Q56" s="128"/>
+      <c r="R56" s="128"/>
+      <c r="S56" s="128"/>
+      <c r="T56" s="152"/>
     </row>
-    <row r="57" spans="1:19" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="L57" s="164" t="s">
+    <row r="57" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A57" s="127">
+        <v>55</v>
+      </c>
+      <c r="B57" s="175"/>
+      <c r="C57" s="129" t="s">
+        <v>342</v>
+      </c>
+      <c r="D57" s="128"/>
+      <c r="E57" s="4" t="s">
+        <v>162</v>
+      </c>
+      <c r="F57" s="4" t="s">
+        <v>341</v>
+      </c>
+      <c r="G57" s="128"/>
+      <c r="H57" s="128"/>
+      <c r="I57" s="128"/>
+      <c r="J57" s="128"/>
+      <c r="K57" s="128"/>
+      <c r="L57" s="128"/>
+      <c r="M57" s="130">
+        <v>1</v>
+      </c>
+      <c r="N57" s="158">
+        <f t="shared" si="3"/>
+        <v>5</v>
+      </c>
+      <c r="O57" s="111" t="s">
+        <v>338</v>
+      </c>
+      <c r="P57" s="128"/>
+      <c r="Q57" s="128"/>
+      <c r="R57" s="128"/>
+      <c r="S57" s="128"/>
+      <c r="T57" s="152"/>
+    </row>
+    <row r="58" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A58" s="127">
+        <v>56</v>
+      </c>
+      <c r="B58" s="175"/>
+      <c r="C58" s="128"/>
+      <c r="D58" s="128"/>
+      <c r="E58" s="4" t="s">
+        <v>162</v>
+      </c>
+      <c r="F58" s="130" t="s">
+        <v>329</v>
+      </c>
+      <c r="G58" s="128"/>
+      <c r="H58" s="128"/>
+      <c r="I58" s="128"/>
+      <c r="J58" s="128"/>
+      <c r="K58" s="128"/>
+      <c r="L58" s="128"/>
+      <c r="M58" s="130">
+        <v>1</v>
+      </c>
+      <c r="N58" s="158">
+        <f t="shared" si="3"/>
+        <v>5</v>
+      </c>
+      <c r="O58" s="128"/>
+      <c r="P58" s="128"/>
+      <c r="Q58" s="128"/>
+      <c r="R58" s="128"/>
+      <c r="S58" s="128"/>
+      <c r="T58" s="152"/>
+    </row>
+    <row r="59" spans="1:20" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A59" s="127">
+        <v>57</v>
+      </c>
+      <c r="B59" s="176"/>
+      <c r="C59" s="159" t="s">
+        <v>335</v>
+      </c>
+      <c r="D59" s="153"/>
+      <c r="E59" s="4" t="s">
+        <v>162</v>
+      </c>
+      <c r="F59" s="154" t="s">
+        <v>330</v>
+      </c>
+      <c r="G59" s="153"/>
+      <c r="H59" s="153"/>
+      <c r="I59" s="153"/>
+      <c r="J59" s="153"/>
+      <c r="K59" s="153"/>
+      <c r="L59" s="180"/>
+      <c r="M59" s="155">
+        <v>2</v>
+      </c>
+      <c r="N59" s="156">
+        <f t="shared" si="3"/>
+        <v>10</v>
+      </c>
+      <c r="O59" s="116" t="s">
+        <v>338</v>
+      </c>
+      <c r="P59" s="153"/>
+      <c r="Q59" s="153"/>
+      <c r="R59" s="153"/>
+      <c r="S59" s="153"/>
+      <c r="T59" s="157"/>
+    </row>
+    <row r="60" spans="1:20" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="M60" s="164" t="s">
         <v>159</v>
       </c>
-      <c r="M57" s="164"/>
-      <c r="N57" s="164"/>
-      <c r="O57" s="164"/>
-      <c r="P57" s="28"/>
-      <c r="Q57" s="29"/>
-      <c r="R57" s="30">
-        <f>SUM(R3:R56)</f>
+      <c r="N60" s="164"/>
+      <c r="O60" s="164"/>
+      <c r="P60" s="164"/>
+      <c r="Q60" s="28"/>
+      <c r="R60" s="29"/>
+      <c r="S60" s="30">
+        <f>SUM(S3:S59)</f>
         <v>184.4162</v>
       </c>
     </row>
-    <row r="58" spans="1:19" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="L58" s="165" t="s">
+    <row r="61" spans="1:20" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="M61" s="165" t="s">
         <v>160</v>
       </c>
-      <c r="M58" s="165"/>
-      <c r="N58" s="165"/>
-      <c r="O58" s="165"/>
-      <c r="P58" s="31">
-        <f>SUM(P3:P57)</f>
+      <c r="N61" s="165"/>
+      <c r="O61" s="165"/>
+      <c r="P61" s="165"/>
+      <c r="Q61" s="31">
+        <f>SUM(Q3:Q60)</f>
         <v>48.896200000000007</v>
       </c>
-      <c r="Q58" s="32"/>
-      <c r="R58" s="31">
-        <f>R57/5</f>
+      <c r="R61" s="32"/>
+      <c r="S61" s="31">
+        <f>S60/5</f>
         <v>36.883240000000001</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="12">
-    <mergeCell ref="A1:S1"/>
-    <mergeCell ref="L57:O57"/>
-    <mergeCell ref="L58:O58"/>
+    <mergeCell ref="A1:T1"/>
+    <mergeCell ref="M60:P60"/>
+    <mergeCell ref="M61:P61"/>
     <mergeCell ref="B37:B45"/>
     <mergeCell ref="B46:B52"/>
     <mergeCell ref="B18:B19"/>
@@ -5778,10 +5971,10 @@
     <mergeCell ref="B11:B14"/>
     <mergeCell ref="B15:B17"/>
     <mergeCell ref="B3:B10"/>
-    <mergeCell ref="B53:B56"/>
+    <mergeCell ref="B53:B59"/>
   </mergeCells>
   <phoneticPr fontId="17" type="noConversion"/>
-  <conditionalFormatting sqref="P58">
+  <conditionalFormatting sqref="Q61">
     <cfRule type="dataBar" priority="5">
       <dataBar>
         <cfvo type="min"/>
@@ -5795,7 +5988,7 @@
       </extLst>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="R57:R58">
+  <conditionalFormatting sqref="S60:S61">
     <cfRule type="dataBar" priority="4">
       <dataBar>
         <cfvo type="min"/>
@@ -5809,7 +6002,7 @@
       </extLst>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="S52">
+  <conditionalFormatting sqref="T52">
     <cfRule type="dataBar" priority="20">
       <dataBar>
         <cfvo type="min"/>
@@ -5823,7 +6016,7 @@
       </extLst>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L3:M50 L52:M56">
+  <conditionalFormatting sqref="M3:N50 M52:N59">
     <cfRule type="colorScale" priority="21">
       <colorScale>
         <cfvo type="min"/>
@@ -5835,7 +6028,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L51:M51">
+  <conditionalFormatting sqref="M51:N51">
     <cfRule type="colorScale" priority="3">
       <colorScale>
         <cfvo type="min"/>
@@ -5847,7 +6040,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="S51">
+  <conditionalFormatting sqref="T51">
     <cfRule type="dataBar" priority="1">
       <dataBar>
         <cfvo type="min"/>
@@ -5861,7 +6054,7 @@
       </extLst>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P3:P50">
+  <conditionalFormatting sqref="Q3:Q50">
     <cfRule type="dataBar" priority="42">
       <dataBar>
         <cfvo type="min"/>
@@ -5875,7 +6068,7 @@
       </extLst>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="R3:R50">
+  <conditionalFormatting sqref="S3:S50">
     <cfRule type="dataBar" priority="44">
       <dataBar>
         <cfvo type="min"/>
@@ -5890,86 +6083,91 @@
     </cfRule>
   </conditionalFormatting>
   <hyperlinks>
-    <hyperlink ref="G3" r:id="rId1" display="https://lcsc.com/brand-detail/254.html" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
-    <hyperlink ref="G4" r:id="rId2" display="https://lcsc.com/brand-detail/254.html" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
-    <hyperlink ref="G5" r:id="rId3" display="https://lcsc.com/brand-detail/392.html" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
-    <hyperlink ref="G6" r:id="rId4" display="https://lcsc.com/brand-detail/254.html" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
-    <hyperlink ref="G7" r:id="rId5" display="https://lcsc.com/brand-detail/994.html" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
-    <hyperlink ref="G12" r:id="rId6" display="https://lcsc.com/brand-detail/296.html" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
-    <hyperlink ref="G22" r:id="rId7" display="https://lcsc.com/brand-detail/94.html" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
-    <hyperlink ref="G24" r:id="rId8" display="https://lcsc.com/brand-detail/396.html" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
-    <hyperlink ref="G41" r:id="rId9" display="https://lcsc.com/brand-detail/756.html" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
-    <hyperlink ref="G42" r:id="rId10" display="https://lcsc.com/brand-detail/100.html" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
-    <hyperlink ref="G47:G49" r:id="rId11" display="https://lcsc.com/brand-detail/853.html" xr:uid="{00000000-0004-0000-0000-00000A000000}"/>
-    <hyperlink ref="G50" r:id="rId12" display="https://lcsc.com/brand-detail/109.html" xr:uid="{00000000-0004-0000-0000-00000B000000}"/>
-    <hyperlink ref="G8" r:id="rId13" display="https://lcsc.com/brand-detail/994.html" xr:uid="{00000000-0004-0000-0000-00000C000000}"/>
-    <hyperlink ref="G11" r:id="rId14" display="https://www.digikey.com/en/supplier-centers/central-semiconductor" xr:uid="{00000000-0004-0000-0000-00000D000000}"/>
-    <hyperlink ref="G13" r:id="rId15" display="https://www.digikey.com/en/supplier-centers/sunled" xr:uid="{00000000-0004-0000-0000-00000E000000}"/>
-    <hyperlink ref="G18" r:id="rId16" display="https://www.digikey.com/en/supplier-centers/wurth-electronics" xr:uid="{00000000-0004-0000-0000-00000F000000}"/>
-    <hyperlink ref="G20" r:id="rId17" display="https://lcsc.com/brand-detail/296.html" xr:uid="{00000000-0004-0000-0000-000010000000}"/>
-    <hyperlink ref="G19" r:id="rId18" display="https://www.digikey.com/en/supplier-centers/tdk" xr:uid="{00000000-0004-0000-0000-000011000000}"/>
-    <hyperlink ref="G23" r:id="rId19" display="https://www.digikey.com/en/supplier-centers/te-connectivity-amp" xr:uid="{00000000-0004-0000-0000-000012000000}"/>
-    <hyperlink ref="G28" r:id="rId20" display="https://www.digikey.com/en/supplier-centers/rohm-semi" xr:uid="{00000000-0004-0000-0000-000013000000}"/>
-    <hyperlink ref="G29" r:id="rId21" display="https://www.digikey.com/en/supplier-centers/panasonic" xr:uid="{00000000-0004-0000-0000-000014000000}"/>
-    <hyperlink ref="G30" r:id="rId22" display="https://www.digikey.com/en/supplier-centers/vishay-dale" xr:uid="{00000000-0004-0000-0000-000015000000}"/>
-    <hyperlink ref="G31" r:id="rId23" display="https://www.digikey.com/en/supplier-centers/vishay-dale" xr:uid="{00000000-0004-0000-0000-000016000000}"/>
-    <hyperlink ref="G33" r:id="rId24" display="https://www.digikey.com/en/supplier-centers/vishay-dale" xr:uid="{00000000-0004-0000-0000-000017000000}"/>
-    <hyperlink ref="G34" r:id="rId25" display="https://www.digikey.com/en/supplier-centers/yageo" xr:uid="{00000000-0004-0000-0000-000018000000}"/>
-    <hyperlink ref="G35" r:id="rId26" display="https://www.digikey.com/en/supplier-centers/stackpole-electronics" xr:uid="{00000000-0004-0000-0000-000019000000}"/>
-    <hyperlink ref="G38" r:id="rId27" display="https://www.digikey.com/en/supplier-centers/texas-instruments" xr:uid="{00000000-0004-0000-0000-00001A000000}"/>
-    <hyperlink ref="G39" r:id="rId28" display="https://www.digikey.com/en/supplier-centers/stmicroelectronics" xr:uid="{00000000-0004-0000-0000-00001B000000}"/>
-    <hyperlink ref="G46" r:id="rId29" display="https://lcsc.com/brand-detail/853.html" xr:uid="{00000000-0004-0000-0000-00001C000000}"/>
-    <hyperlink ref="G45" r:id="rId30" display="https://www.digikey.com/en/supplier-centers/analog-devices" xr:uid="{00000000-0004-0000-0000-00001D000000}"/>
-    <hyperlink ref="G26" r:id="rId31" display="https://lcsc.com/brand-detail/396.html" xr:uid="{00000000-0004-0000-0000-00001E000000}"/>
-    <hyperlink ref="G27" r:id="rId32" display="https://www.digikey.com/en/supplier-centers/te-connectivity-amp" xr:uid="{00000000-0004-0000-0000-00001F000000}"/>
-    <hyperlink ref="G37" r:id="rId33" display="https://lcsc.com/brand-detail/877.html" xr:uid="{00000000-0004-0000-0000-000020000000}"/>
-    <hyperlink ref="N5" r:id="rId34" xr:uid="{00000000-0004-0000-0000-000021000000}"/>
-    <hyperlink ref="N7" r:id="rId35" xr:uid="{00000000-0004-0000-0000-000022000000}"/>
-    <hyperlink ref="N6" r:id="rId36" xr:uid="{00000000-0004-0000-0000-000023000000}"/>
-    <hyperlink ref="N3" r:id="rId37" xr:uid="{00000000-0004-0000-0000-000024000000}"/>
-    <hyperlink ref="N4" r:id="rId38" xr:uid="{00000000-0004-0000-0000-000025000000}"/>
-    <hyperlink ref="N8" r:id="rId39" xr:uid="{00000000-0004-0000-0000-000026000000}"/>
-    <hyperlink ref="N12" r:id="rId40" xr:uid="{00000000-0004-0000-0000-000027000000}"/>
-    <hyperlink ref="N13" r:id="rId41" xr:uid="{00000000-0004-0000-0000-000028000000}"/>
-    <hyperlink ref="N19" r:id="rId42" xr:uid="{00000000-0004-0000-0000-000029000000}"/>
-    <hyperlink ref="N20" r:id="rId43" xr:uid="{00000000-0004-0000-0000-00002A000000}"/>
-    <hyperlink ref="N22" r:id="rId44" xr:uid="{00000000-0004-0000-0000-00002B000000}"/>
-    <hyperlink ref="N24" r:id="rId45" xr:uid="{00000000-0004-0000-0000-00002C000000}"/>
-    <hyperlink ref="N23" r:id="rId46" xr:uid="{00000000-0004-0000-0000-00002D000000}"/>
-    <hyperlink ref="N30" r:id="rId47" xr:uid="{00000000-0004-0000-0000-00002E000000}"/>
-    <hyperlink ref="N31" r:id="rId48" xr:uid="{00000000-0004-0000-0000-00002F000000}"/>
-    <hyperlink ref="N33" r:id="rId49" xr:uid="{00000000-0004-0000-0000-000030000000}"/>
-    <hyperlink ref="N34" r:id="rId50" xr:uid="{00000000-0004-0000-0000-000031000000}"/>
-    <hyperlink ref="N35" r:id="rId51" xr:uid="{00000000-0004-0000-0000-000032000000}"/>
-    <hyperlink ref="N46" r:id="rId52" xr:uid="{00000000-0004-0000-0000-000033000000}"/>
-    <hyperlink ref="N47" r:id="rId53" xr:uid="{00000000-0004-0000-0000-000034000000}"/>
-    <hyperlink ref="N48" r:id="rId54" xr:uid="{00000000-0004-0000-0000-000035000000}"/>
-    <hyperlink ref="N50" r:id="rId55" xr:uid="{00000000-0004-0000-0000-000036000000}"/>
-    <hyperlink ref="N49" r:id="rId56" xr:uid="{00000000-0004-0000-0000-000037000000}"/>
-    <hyperlink ref="N42" r:id="rId57" xr:uid="{00000000-0004-0000-0000-000038000000}"/>
-    <hyperlink ref="N21" r:id="rId58" xr:uid="{00000000-0004-0000-0000-000039000000}"/>
-    <hyperlink ref="N26" r:id="rId59" xr:uid="{00000000-0004-0000-0000-00003A000000}"/>
-    <hyperlink ref="N28" r:id="rId60" xr:uid="{00000000-0004-0000-0000-00003B000000}"/>
-    <hyperlink ref="N29" r:id="rId61" xr:uid="{00000000-0004-0000-0000-00003C000000}"/>
-    <hyperlink ref="N27" r:id="rId62" xr:uid="{00000000-0004-0000-0000-00003D000000}"/>
-    <hyperlink ref="N32" r:id="rId63" xr:uid="{00000000-0004-0000-0000-00003E000000}"/>
-    <hyperlink ref="N36" r:id="rId64" xr:uid="{00000000-0004-0000-0000-00003F000000}"/>
-    <hyperlink ref="N37" r:id="rId65" xr:uid="{00000000-0004-0000-0000-000040000000}"/>
-    <hyperlink ref="N40" r:id="rId66" xr:uid="{00000000-0004-0000-0000-000041000000}"/>
-    <hyperlink ref="N41" r:id="rId67" xr:uid="{00000000-0004-0000-0000-000042000000}"/>
-    <hyperlink ref="N43" r:id="rId68" xr:uid="{00000000-0004-0000-0000-000043000000}"/>
-    <hyperlink ref="N9" r:id="rId69" xr:uid="{00000000-0004-0000-0000-000044000000}"/>
-    <hyperlink ref="N11" r:id="rId70" xr:uid="{00000000-0004-0000-0000-000045000000}"/>
-    <hyperlink ref="N14" r:id="rId71" xr:uid="{00000000-0004-0000-0000-000046000000}"/>
-    <hyperlink ref="N15" r:id="rId72" xr:uid="{00000000-0004-0000-0000-00004B000000}"/>
-    <hyperlink ref="N16" r:id="rId73" xr:uid="{00000000-0004-0000-0000-00004C000000}"/>
-    <hyperlink ref="N17" r:id="rId74" xr:uid="{00000000-0004-0000-0000-00004D000000}"/>
-    <hyperlink ref="N10" r:id="rId75" xr:uid="{00000000-0004-0000-0000-00004F000000}"/>
-    <hyperlink ref="G25" r:id="rId76" display="https://lcsc.com/brand-detail/396.html" xr:uid="{00000000-0004-0000-0000-000050000000}"/>
-    <hyperlink ref="N25" r:id="rId77" xr:uid="{00000000-0004-0000-0000-000051000000}"/>
+    <hyperlink ref="G3" r:id="rId1" display="https://lcsc.com/brand-detail/254.html"/>
+    <hyperlink ref="G4" r:id="rId2" display="https://lcsc.com/brand-detail/254.html"/>
+    <hyperlink ref="G5" r:id="rId3" display="https://lcsc.com/brand-detail/392.html"/>
+    <hyperlink ref="G6" r:id="rId4" display="https://lcsc.com/brand-detail/254.html"/>
+    <hyperlink ref="G7" r:id="rId5" display="https://lcsc.com/brand-detail/994.html"/>
+    <hyperlink ref="G12" r:id="rId6" display="https://lcsc.com/brand-detail/296.html"/>
+    <hyperlink ref="G22" r:id="rId7" display="https://lcsc.com/brand-detail/94.html"/>
+    <hyperlink ref="G24" r:id="rId8" display="https://lcsc.com/brand-detail/396.html"/>
+    <hyperlink ref="G41" r:id="rId9" display="https://lcsc.com/brand-detail/756.html"/>
+    <hyperlink ref="G42" r:id="rId10" display="https://lcsc.com/brand-detail/100.html"/>
+    <hyperlink ref="G47:G49" r:id="rId11" display="https://lcsc.com/brand-detail/853.html"/>
+    <hyperlink ref="G50" r:id="rId12" display="https://lcsc.com/brand-detail/109.html"/>
+    <hyperlink ref="G8" r:id="rId13" display="https://lcsc.com/brand-detail/994.html"/>
+    <hyperlink ref="G11" r:id="rId14" display="https://www.digikey.com/en/supplier-centers/central-semiconductor"/>
+    <hyperlink ref="G13" r:id="rId15" display="https://www.digikey.com/en/supplier-centers/sunled"/>
+    <hyperlink ref="G18" r:id="rId16" display="https://www.digikey.com/en/supplier-centers/wurth-electronics"/>
+    <hyperlink ref="G20" r:id="rId17" display="https://lcsc.com/brand-detail/296.html"/>
+    <hyperlink ref="G19" r:id="rId18" display="https://www.digikey.com/en/supplier-centers/tdk"/>
+    <hyperlink ref="G23" r:id="rId19" display="https://www.digikey.com/en/supplier-centers/te-connectivity-amp"/>
+    <hyperlink ref="G28" r:id="rId20" display="https://www.digikey.com/en/supplier-centers/rohm-semi"/>
+    <hyperlink ref="G29" r:id="rId21" display="https://www.digikey.com/en/supplier-centers/panasonic"/>
+    <hyperlink ref="G30" r:id="rId22" display="https://www.digikey.com/en/supplier-centers/vishay-dale"/>
+    <hyperlink ref="G31" r:id="rId23" display="https://www.digikey.com/en/supplier-centers/vishay-dale"/>
+    <hyperlink ref="G33" r:id="rId24" display="https://www.digikey.com/en/supplier-centers/vishay-dale"/>
+    <hyperlink ref="G34" r:id="rId25" display="https://www.digikey.com/en/supplier-centers/yageo"/>
+    <hyperlink ref="G35" r:id="rId26" display="https://www.digikey.com/en/supplier-centers/stackpole-electronics"/>
+    <hyperlink ref="G38" r:id="rId27" display="https://www.digikey.com/en/supplier-centers/texas-instruments"/>
+    <hyperlink ref="G39" r:id="rId28" display="https://www.digikey.com/en/supplier-centers/stmicroelectronics"/>
+    <hyperlink ref="G46" r:id="rId29" display="https://lcsc.com/brand-detail/853.html"/>
+    <hyperlink ref="G45" r:id="rId30" display="https://www.digikey.com/en/supplier-centers/analog-devices"/>
+    <hyperlink ref="G26" r:id="rId31" display="https://lcsc.com/brand-detail/396.html"/>
+    <hyperlink ref="G27" r:id="rId32" display="https://www.digikey.com/en/supplier-centers/te-connectivity-amp"/>
+    <hyperlink ref="G37" r:id="rId33" display="https://lcsc.com/brand-detail/877.html"/>
+    <hyperlink ref="O5" r:id="rId34"/>
+    <hyperlink ref="O7" r:id="rId35"/>
+    <hyperlink ref="O6" r:id="rId36"/>
+    <hyperlink ref="O3" r:id="rId37"/>
+    <hyperlink ref="O4" r:id="rId38"/>
+    <hyperlink ref="O8" r:id="rId39"/>
+    <hyperlink ref="O12" r:id="rId40"/>
+    <hyperlink ref="O13" r:id="rId41"/>
+    <hyperlink ref="O19" r:id="rId42"/>
+    <hyperlink ref="O20" r:id="rId43"/>
+    <hyperlink ref="O22" r:id="rId44"/>
+    <hyperlink ref="O24" r:id="rId45"/>
+    <hyperlink ref="O23" r:id="rId46"/>
+    <hyperlink ref="O30" r:id="rId47"/>
+    <hyperlink ref="O31" r:id="rId48"/>
+    <hyperlink ref="O33" r:id="rId49"/>
+    <hyperlink ref="O34" r:id="rId50"/>
+    <hyperlink ref="O35" r:id="rId51"/>
+    <hyperlink ref="O46" r:id="rId52"/>
+    <hyperlink ref="O47" r:id="rId53"/>
+    <hyperlink ref="O48" r:id="rId54"/>
+    <hyperlink ref="O50" r:id="rId55"/>
+    <hyperlink ref="O49" r:id="rId56"/>
+    <hyperlink ref="O42" r:id="rId57"/>
+    <hyperlink ref="O21" r:id="rId58"/>
+    <hyperlink ref="O26" r:id="rId59"/>
+    <hyperlink ref="O28" r:id="rId60"/>
+    <hyperlink ref="O29" r:id="rId61"/>
+    <hyperlink ref="O27" r:id="rId62"/>
+    <hyperlink ref="O32" r:id="rId63"/>
+    <hyperlink ref="O36" r:id="rId64"/>
+    <hyperlink ref="O37" r:id="rId65"/>
+    <hyperlink ref="O40" r:id="rId66"/>
+    <hyperlink ref="O41" r:id="rId67"/>
+    <hyperlink ref="O43" r:id="rId68"/>
+    <hyperlink ref="O9" r:id="rId69"/>
+    <hyperlink ref="O11" r:id="rId70"/>
+    <hyperlink ref="O14" r:id="rId71"/>
+    <hyperlink ref="O15" r:id="rId72"/>
+    <hyperlink ref="O16" r:id="rId73"/>
+    <hyperlink ref="O17" r:id="rId74"/>
+    <hyperlink ref="O10" r:id="rId75"/>
+    <hyperlink ref="G25" r:id="rId76" display="https://lcsc.com/brand-detail/396.html"/>
+    <hyperlink ref="O25" r:id="rId77"/>
+    <hyperlink ref="O53" r:id="rId78"/>
+    <hyperlink ref="O59" r:id="rId79"/>
+    <hyperlink ref="O54" r:id="rId80" location="customerReviews"/>
+    <hyperlink ref="O55" r:id="rId81"/>
+    <hyperlink ref="O57" r:id="rId82"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId78"/>
+  <pageSetup orientation="portrait" r:id="rId83"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
@@ -5984,7 +6182,7 @@
               <x14:axisColor rgb="FF000000"/>
             </x14:dataBar>
           </x14:cfRule>
-          <xm:sqref>P58</xm:sqref>
+          <xm:sqref>Q61</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
           <x14:cfRule type="dataBar" id="{36ECBF5D-EFFC-4768-AC2E-9F5CCB8EA1CF}">
@@ -5997,7 +6195,7 @@
               <x14:axisColor rgb="FF000000"/>
             </x14:dataBar>
           </x14:cfRule>
-          <xm:sqref>R57:R58</xm:sqref>
+          <xm:sqref>S60:S61</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
           <x14:cfRule type="dataBar" id="{8043E1D2-A386-4972-9379-8F1175F4CD55}">
@@ -6010,7 +6208,7 @@
               <x14:axisColor rgb="FF000000"/>
             </x14:dataBar>
           </x14:cfRule>
-          <xm:sqref>S52</xm:sqref>
+          <xm:sqref>T52</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
           <x14:cfRule type="dataBar" id="{568B2A70-A44C-42B7-B5F8-9C8E28B37608}">
@@ -6023,7 +6221,7 @@
               <x14:axisColor rgb="FF000000"/>
             </x14:dataBar>
           </x14:cfRule>
-          <xm:sqref>S51</xm:sqref>
+          <xm:sqref>T51</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
           <x14:cfRule type="dataBar" id="{B802BE45-AE6E-4AFB-92D7-CAE7DD159284}">
@@ -6036,7 +6234,7 @@
               <x14:axisColor rgb="FF000000"/>
             </x14:dataBar>
           </x14:cfRule>
-          <xm:sqref>P3:P50</xm:sqref>
+          <xm:sqref>Q3:Q50</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
           <x14:cfRule type="dataBar" id="{423AC320-90C5-4685-9B12-A5EE24B441D5}">
@@ -6049,7 +6247,7 @@
               <x14:axisColor rgb="FF000000"/>
             </x14:dataBar>
           </x14:cfRule>
-          <xm:sqref>R3:R50</xm:sqref>
+          <xm:sqref>S3:S50</xm:sqref>
         </x14:conditionalFormatting>
       </x14:conditionalFormattings>
     </ext>

</xml_diff>

<commit_message>
#28 header footprint review ho gaye han Or BOM me b add kr diye han
</commit_message>
<xml_diff>
--- a/Documents/Deliverables/BOM/LCSC_BOM.xlsx
+++ b/Documents/Deliverables/BOM/LCSC_BOM.xlsx
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="518" uniqueCount="336">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="546" uniqueCount="348">
   <si>
     <t>S. No.</t>
   </si>
@@ -360,9 +360,6 @@
     <t>CONN HEADER VERT 4POS 2.5MM</t>
   </si>
   <si>
-    <t>J2, J12, J17</t>
-  </si>
-  <si>
     <t>B4B-XH-A(LF)(SN)</t>
   </si>
   <si>
@@ -373,9 +370,6 @@
   </si>
   <si>
     <t>CONN HEADER VERT 7POS 2.5MM</t>
-  </si>
-  <si>
-    <t>J14, J15</t>
   </si>
   <si>
     <t>B7B-XH-A(LF)(SN)</t>
@@ -643,9 +637,6 @@
 </t>
   </si>
   <si>
-    <t>J10, J11, J13, J20, J30</t>
-  </si>
-  <si>
     <t>Capacitors</t>
   </si>
   <si>
@@ -891,9 +882,6 @@
     <t>C98224</t>
   </si>
   <si>
-    <t>J3, J24, J25, J26, J27, J28, J29</t>
-  </si>
-  <si>
     <t>P1, P2, P3, P4, P5, P6</t>
   </si>
   <si>
@@ -1051,6 +1039,54 @@
   </si>
   <si>
     <t>LED4, LED5</t>
+  </si>
+  <si>
+    <t>J3, J24, J25, J28, J29</t>
+  </si>
+  <si>
+    <t>J4</t>
+  </si>
+  <si>
+    <t>J14</t>
+  </si>
+  <si>
+    <t>J30</t>
+  </si>
+  <si>
+    <t>7 POS 2.54mm female header</t>
+  </si>
+  <si>
+    <t>J1, J15</t>
+  </si>
+  <si>
+    <t>HDR_F_1X7</t>
+  </si>
+  <si>
+    <t>4 POS 2.54mm female header</t>
+  </si>
+  <si>
+    <t>J2</t>
+  </si>
+  <si>
+    <t>HDR_F_1X4</t>
+  </si>
+  <si>
+    <t>3 POS 2.54mm female header</t>
+  </si>
+  <si>
+    <t>J10, J11, J12, J13, J20</t>
+  </si>
+  <si>
+    <t>HDR_F_1X3</t>
+  </si>
+  <si>
+    <t>------</t>
+  </si>
+  <si>
+    <t>Aliexpress</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aliexprss Shipping Charges </t>
   </si>
 </sst>
 </file>
@@ -2184,45 +2220,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="25" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2282,15 +2279,6 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="32" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2346,6 +2334,54 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -2628,7 +2664,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:T61"/>
+  <dimension ref="A1:T66"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6.140625" bestFit="1" customWidth="1"/>
@@ -2654,28 +2690,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:20" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="146" t="s">
-        <v>152</v>
-      </c>
-      <c r="B1" s="147"/>
-      <c r="C1" s="147"/>
-      <c r="D1" s="147"/>
-      <c r="E1" s="147"/>
-      <c r="F1" s="147"/>
-      <c r="G1" s="147"/>
-      <c r="H1" s="147"/>
-      <c r="I1" s="147"/>
-      <c r="J1" s="147"/>
-      <c r="K1" s="147"/>
-      <c r="L1" s="147"/>
-      <c r="M1" s="147"/>
-      <c r="N1" s="147"/>
-      <c r="O1" s="147"/>
-      <c r="P1" s="147"/>
-      <c r="Q1" s="147"/>
-      <c r="R1" s="147"/>
-      <c r="S1" s="147"/>
-      <c r="T1" s="148"/>
+      <c r="A1" s="185" t="s">
+        <v>150</v>
+      </c>
+      <c r="B1" s="186"/>
+      <c r="C1" s="186"/>
+      <c r="D1" s="186"/>
+      <c r="E1" s="186"/>
+      <c r="F1" s="186"/>
+      <c r="G1" s="186"/>
+      <c r="H1" s="186"/>
+      <c r="I1" s="186"/>
+      <c r="J1" s="186"/>
+      <c r="K1" s="186"/>
+      <c r="L1" s="186"/>
+      <c r="M1" s="186"/>
+      <c r="N1" s="186"/>
+      <c r="O1" s="186"/>
+      <c r="P1" s="186"/>
+      <c r="Q1" s="186"/>
+      <c r="R1" s="186"/>
+      <c r="S1" s="186"/>
+      <c r="T1" s="187"/>
     </row>
     <row r="2" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="52" t="s">
@@ -2700,7 +2736,7 @@
         <v>6</v>
       </c>
       <c r="H2" s="53" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="I2" s="53" t="s">
         <v>7</v>
@@ -2709,19 +2745,19 @@
         <v>8</v>
       </c>
       <c r="K2" s="53" t="s">
-        <v>323</v>
+        <v>319</v>
       </c>
       <c r="L2" s="53" t="s">
-        <v>324</v>
+        <v>320</v>
       </c>
       <c r="M2" s="53" t="s">
         <v>9</v>
       </c>
       <c r="N2" s="53" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="O2" s="53" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="P2" s="53" t="s">
         <v>10</v>
@@ -2733,24 +2769,24 @@
         <v>12</v>
       </c>
       <c r="S2" s="53" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="T2" s="53" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
     </row>
     <row r="3" spans="1:20" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="27">
         <v>1</v>
       </c>
-      <c r="B3" s="156" t="s">
-        <v>202</v>
+      <c r="B3" s="196" t="s">
+        <v>199</v>
       </c>
       <c r="C3" s="71" t="s">
         <v>13</v>
       </c>
       <c r="D3" s="83" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="E3" s="14" t="s">
         <v>14</v>
@@ -2762,13 +2798,13 @@
         <v>16</v>
       </c>
       <c r="H3" s="73" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="I3" s="44" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="J3" s="14" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="K3" s="16">
         <v>50</v>
@@ -2779,12 +2815,12 @@
       <c r="M3" s="17">
         <v>13</v>
       </c>
-      <c r="N3" s="173">
+      <c r="N3" s="160">
         <f>M3*5</f>
         <v>65</v>
       </c>
       <c r="O3" s="15" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="P3" s="18">
         <v>6.1000000000000004E-3</v>
@@ -2806,12 +2842,12 @@
       <c r="A4" s="27">
         <v>2</v>
       </c>
-      <c r="B4" s="157"/>
+      <c r="B4" s="195"/>
       <c r="C4" s="25" t="s">
         <v>17</v>
       </c>
       <c r="D4" s="49" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="E4" s="4" t="s">
         <v>14</v>
@@ -2823,13 +2859,13 @@
         <v>16</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="I4" s="45" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="J4" s="4" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="K4" s="5">
         <v>50</v>
@@ -2841,11 +2877,11 @@
         <v>7</v>
       </c>
       <c r="N4" s="5">
-        <f t="shared" ref="N4:N59" si="0">M4*5</f>
+        <f t="shared" ref="N4:N62" si="0">M4*5</f>
         <v>35</v>
       </c>
       <c r="O4" s="1" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="P4" s="12">
         <v>3.7000000000000002E-3</v>
@@ -2867,12 +2903,12 @@
       <c r="A5" s="27">
         <v>3</v>
       </c>
-      <c r="B5" s="157"/>
+      <c r="B5" s="195"/>
       <c r="C5" s="25" t="s">
         <v>19</v>
       </c>
       <c r="D5" s="49" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="E5" s="4" t="s">
         <v>14</v>
@@ -2884,13 +2920,13 @@
         <v>21</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="I5" s="45" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="J5" s="4" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="K5" s="5">
         <v>20</v>
@@ -2906,7 +2942,7 @@
         <v>30</v>
       </c>
       <c r="O5" s="1" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="P5" s="12">
         <v>3.1199999999999999E-2</v>
@@ -2928,7 +2964,7 @@
       <c r="A6" s="27">
         <v>4</v>
       </c>
-      <c r="B6" s="157"/>
+      <c r="B6" s="195"/>
       <c r="C6" s="25" t="s">
         <v>22</v>
       </c>
@@ -2945,13 +2981,13 @@
         <v>16</v>
       </c>
       <c r="H6" s="4" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="I6" s="45" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="J6" s="4" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="K6" s="5">
         <v>20</v>
@@ -2967,7 +3003,7 @@
         <v>10</v>
       </c>
       <c r="O6" s="1" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="P6" s="12">
         <v>1.8100000000000002E-2</v>
@@ -2980,7 +3016,7 @@
         <v>1.8100000000000002E-2</v>
       </c>
       <c r="S6" s="11">
-        <f t="shared" ref="S6:S50" si="1">R6*L6</f>
+        <f t="shared" ref="S6:S53" si="1">R6*L6</f>
         <v>0.36200000000000004</v>
       </c>
       <c r="T6" s="7"/>
@@ -2989,30 +3025,30 @@
       <c r="A7" s="27">
         <v>5</v>
       </c>
-      <c r="B7" s="157"/>
+      <c r="B7" s="195"/>
       <c r="C7" s="25" t="s">
-        <v>327</v>
+        <v>323</v>
       </c>
       <c r="D7" s="49" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="F7" s="4" t="s">
+        <v>325</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="H7" s="4" t="s">
         <v>329</v>
       </c>
-      <c r="G7" s="1" t="s">
-        <v>148</v>
-      </c>
-      <c r="H7" s="4" t="s">
-        <v>333</v>
-      </c>
       <c r="I7" s="45" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="J7" s="4" t="s">
-        <v>328</v>
+        <v>324</v>
       </c>
       <c r="K7" s="5">
         <v>50</v>
@@ -3028,13 +3064,13 @@
         <v>10</v>
       </c>
       <c r="O7" s="1" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="P7" s="12">
         <v>8.8000000000000005E-3</v>
       </c>
       <c r="Q7" s="11">
-        <f t="shared" ref="Q7:Q50" si="2">P7*K7</f>
+        <f t="shared" ref="Q7:Q53" si="2">P7*K7</f>
         <v>0.44</v>
       </c>
       <c r="R7" s="12">
@@ -3050,7 +3086,7 @@
       <c r="A8" s="27">
         <v>6</v>
       </c>
-      <c r="B8" s="157"/>
+      <c r="B8" s="195"/>
       <c r="C8" s="33" t="s">
         <v>26</v>
       </c>
@@ -3058,7 +3094,7 @@
         <v>27</v>
       </c>
       <c r="E8" s="34" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="F8" s="4" t="s">
         <v>28</v>
@@ -3067,11 +3103,11 @@
         <v>25</v>
       </c>
       <c r="H8" s="4" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="I8" s="5"/>
       <c r="J8" s="4" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="K8" s="5"/>
       <c r="L8" s="5"/>
@@ -3099,30 +3135,30 @@
       <c r="A9" s="27">
         <v>7</v>
       </c>
-      <c r="B9" s="157"/>
+      <c r="B9" s="195"/>
       <c r="C9" s="106" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
       <c r="D9" s="107" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
       <c r="E9" s="108" t="s">
         <v>14</v>
       </c>
       <c r="F9" s="108" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="H9" s="4" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="I9" s="45" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="J9" s="91" t="s">
-        <v>254</v>
+        <v>251</v>
       </c>
       <c r="K9" s="5">
         <v>20</v>
@@ -3138,7 +3174,7 @@
         <v>5</v>
       </c>
       <c r="O9" s="1" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="P9" s="12">
         <v>2.0500000000000001E-2</v>
@@ -3160,30 +3196,30 @@
       <c r="A10" s="27">
         <v>8</v>
       </c>
-      <c r="B10" s="158"/>
+      <c r="B10" s="197"/>
       <c r="C10" s="120" t="s">
-        <v>292</v>
+        <v>288</v>
       </c>
       <c r="D10" s="121" t="s">
-        <v>293</v>
+        <v>289</v>
       </c>
       <c r="E10" s="122" t="s">
+        <v>290</v>
+      </c>
+      <c r="F10" s="122" t="s">
+        <v>291</v>
+      </c>
+      <c r="G10" s="123" t="s">
+        <v>299</v>
+      </c>
+      <c r="H10" s="74" t="s">
+        <v>300</v>
+      </c>
+      <c r="I10" s="81" t="s">
+        <v>307</v>
+      </c>
+      <c r="J10" s="74" t="s">
         <v>294</v>
-      </c>
-      <c r="F10" s="122" t="s">
-        <v>295</v>
-      </c>
-      <c r="G10" s="123" t="s">
-        <v>303</v>
-      </c>
-      <c r="H10" s="74" t="s">
-        <v>304</v>
-      </c>
-      <c r="I10" s="81" t="s">
-        <v>311</v>
-      </c>
-      <c r="J10" s="74" t="s">
-        <v>298</v>
       </c>
       <c r="K10" s="76">
         <v>10</v>
@@ -3199,7 +3235,7 @@
         <v>10</v>
       </c>
       <c r="O10" s="21" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="P10" s="124">
         <v>5.8700000000000002E-2</v>
@@ -3216,14 +3252,14 @@
         <v>1.1739999999999999</v>
       </c>
       <c r="T10" s="126" t="s">
-        <v>312</v>
+        <v>308</v>
       </c>
     </row>
     <row r="11" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="27">
         <v>9</v>
       </c>
-      <c r="B11" s="157" t="s">
+      <c r="B11" s="195" t="s">
         <v>29</v>
       </c>
       <c r="C11" s="85" t="s">
@@ -3235,27 +3271,27 @@
       <c r="E11" s="87" t="s">
         <v>32</v>
       </c>
-      <c r="F11" s="187" t="s">
+      <c r="F11" s="171" t="s">
         <v>33</v>
       </c>
-      <c r="G11" s="159" t="s">
-        <v>141</v>
-      </c>
-      <c r="H11" s="160"/>
-      <c r="I11" s="183"/>
+      <c r="G11" s="146" t="s">
+        <v>139</v>
+      </c>
+      <c r="H11" s="147"/>
+      <c r="I11" s="167"/>
       <c r="J11" s="87" t="s">
-        <v>153</v>
-      </c>
-      <c r="K11" s="174"/>
-      <c r="L11" s="174"/>
-      <c r="M11" s="160">
+        <v>151</v>
+      </c>
+      <c r="K11" s="161"/>
+      <c r="L11" s="161"/>
+      <c r="M11" s="147">
         <v>2</v>
       </c>
-      <c r="N11" s="174">
+      <c r="N11" s="161">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="O11" s="159"/>
+      <c r="O11" s="146"/>
       <c r="P11" s="88"/>
       <c r="Q11" s="82">
         <f>P11*K11</f>
@@ -3266,15 +3302,15 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="T11" s="188"/>
+      <c r="T11" s="172"/>
     </row>
     <row r="12" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="27">
         <v>10</v>
       </c>
-      <c r="B12" s="157"/>
+      <c r="B12" s="195"/>
       <c r="C12" s="25" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="D12" s="49" t="s">
         <v>34</v>
@@ -3289,13 +3325,13 @@
         <v>37</v>
       </c>
       <c r="H12" s="6" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="I12" s="45" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="J12" s="4" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="K12" s="5">
         <v>10</v>
@@ -3311,7 +3347,7 @@
         <v>5</v>
       </c>
       <c r="O12" s="1" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="P12" s="12">
         <v>5.3699999999999998E-2</v>
@@ -3333,30 +3369,30 @@
       <c r="A13" s="27">
         <v>11</v>
       </c>
-      <c r="B13" s="157"/>
+      <c r="B13" s="195"/>
       <c r="C13" s="89" t="s">
+        <v>163</v>
+      </c>
+      <c r="D13" s="90" t="s">
+        <v>164</v>
+      </c>
+      <c r="E13" s="91" t="s">
         <v>165</v>
       </c>
-      <c r="D13" s="90" t="s">
+      <c r="F13" s="132" t="s">
         <v>166</v>
       </c>
-      <c r="E13" s="91" t="s">
+      <c r="G13" s="163" t="s">
         <v>167</v>
       </c>
-      <c r="F13" s="132" t="s">
-        <v>168</v>
-      </c>
-      <c r="G13" s="176" t="s">
-        <v>169</v>
-      </c>
-      <c r="H13" s="177" t="s">
-        <v>255</v>
-      </c>
-      <c r="I13" s="178" t="s">
-        <v>256</v>
+      <c r="H13" s="164" t="s">
+        <v>252</v>
+      </c>
+      <c r="I13" s="165" t="s">
+        <v>253</v>
       </c>
       <c r="J13" s="91" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="K13" s="94">
         <v>5</v>
@@ -3367,12 +3403,12 @@
       <c r="M13" s="95">
         <v>1</v>
       </c>
-      <c r="N13" s="182">
+      <c r="N13" s="166">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
       <c r="O13" s="92" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="P13" s="93">
         <v>9.6500000000000002E-2</v>
@@ -3389,39 +3425,39 @@
         <v>0.96500000000000008</v>
       </c>
       <c r="T13" s="101" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
     </row>
     <row r="14" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="27">
         <v>12</v>
       </c>
-      <c r="B14" s="179" t="s">
-        <v>278</v>
+      <c r="B14" s="198" t="s">
+        <v>275</v>
       </c>
       <c r="C14" s="24" t="s">
-        <v>266</v>
+        <v>263</v>
       </c>
       <c r="D14" s="48" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
       <c r="E14" s="14" t="s">
-        <v>274</v>
+        <v>271</v>
       </c>
       <c r="F14" s="14" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
       <c r="G14" s="23" t="s">
+        <v>273</v>
+      </c>
+      <c r="H14" s="17" t="s">
         <v>276</v>
       </c>
-      <c r="H14" s="17" t="s">
-        <v>279</v>
-      </c>
       <c r="I14" s="44" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="J14" s="14" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="K14" s="14">
         <v>20</v>
@@ -3437,7 +3473,7 @@
         <v>5</v>
       </c>
       <c r="O14" s="117" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="P14" s="18">
         <v>0.02</v>
@@ -3459,30 +3495,30 @@
       <c r="A15" s="27">
         <v>13</v>
       </c>
-      <c r="B15" s="180"/>
+      <c r="B15" s="199"/>
       <c r="C15" s="89" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
       <c r="D15" s="90" t="s">
-        <v>270</v>
+        <v>267</v>
       </c>
       <c r="E15" s="91" t="s">
+        <v>271</v>
+      </c>
+      <c r="F15" s="91" t="s">
+        <v>268</v>
+      </c>
+      <c r="G15" s="163" t="s">
         <v>274</v>
       </c>
-      <c r="F15" s="91" t="s">
-        <v>271</v>
-      </c>
-      <c r="G15" s="176" t="s">
+      <c r="H15" s="164" t="s">
         <v>277</v>
       </c>
-      <c r="H15" s="177" t="s">
-        <v>280</v>
-      </c>
-      <c r="I15" s="178" t="s">
-        <v>156</v>
+      <c r="I15" s="165" t="s">
+        <v>154</v>
       </c>
       <c r="J15" s="91" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="K15" s="91">
         <v>20</v>
@@ -3490,15 +3526,15 @@
       <c r="L15" s="91">
         <v>20</v>
       </c>
-      <c r="M15" s="177">
+      <c r="M15" s="164">
         <v>1</v>
       </c>
-      <c r="N15" s="182">
+      <c r="N15" s="166">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="O15" s="175" t="s">
-        <v>215</v>
+      <c r="O15" s="162" t="s">
+        <v>212</v>
       </c>
       <c r="P15" s="93">
         <v>3.1E-2</v>
@@ -3520,30 +3556,30 @@
       <c r="A16" s="27">
         <v>14</v>
       </c>
-      <c r="B16" s="180"/>
+      <c r="B16" s="199"/>
       <c r="C16" s="25" t="s">
+        <v>269</v>
+      </c>
+      <c r="D16" s="49" t="s">
+        <v>270</v>
+      </c>
+      <c r="E16" s="4" t="s">
+        <v>271</v>
+      </c>
+      <c r="F16" s="4" t="s">
         <v>272</v>
       </c>
-      <c r="D16" s="49" t="s">
+      <c r="G16" s="3" t="s">
         <v>273</v>
       </c>
-      <c r="E16" s="4" t="s">
-        <v>274</v>
-      </c>
-      <c r="F16" s="4" t="s">
-        <v>275</v>
-      </c>
-      <c r="G16" s="3" t="s">
-        <v>276</v>
-      </c>
       <c r="H16" s="6" t="s">
-        <v>281</v>
+        <v>278</v>
       </c>
       <c r="I16" s="45" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="J16" s="4" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="K16" s="4">
         <v>20</v>
@@ -3559,7 +3595,7 @@
         <v>5</v>
       </c>
       <c r="O16" s="105" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="P16" s="12">
         <v>1.8499999999999999E-2</v>
@@ -3581,30 +3617,30 @@
       <c r="A17" s="27">
         <v>15</v>
       </c>
-      <c r="B17" s="181"/>
-      <c r="C17" s="189" t="s">
+      <c r="B17" s="200"/>
+      <c r="C17" s="173" t="s">
         <v>38</v>
       </c>
-      <c r="D17" s="190" t="s">
-        <v>335</v>
+      <c r="D17" s="174" t="s">
+        <v>331</v>
       </c>
       <c r="E17" s="74" t="s">
         <v>39</v>
       </c>
-      <c r="F17" s="192" t="s">
+      <c r="F17" s="176" t="s">
         <v>40</v>
       </c>
-      <c r="G17" s="193" t="s">
-        <v>142</v>
+      <c r="G17" s="177" t="s">
+        <v>140</v>
       </c>
       <c r="H17" s="75" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="I17" s="81" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="J17" s="74" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="K17" s="76">
         <v>50</v>
@@ -3619,8 +3655,8 @@
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="O17" s="191" t="s">
-        <v>215</v>
+      <c r="O17" s="175" t="s">
+        <v>212</v>
       </c>
       <c r="P17" s="124">
         <v>1.4E-2</v>
@@ -3642,32 +3678,32 @@
       <c r="A18" s="27">
         <v>16</v>
       </c>
-      <c r="B18" s="151" t="s">
+      <c r="B18" s="190" t="s">
         <v>41</v>
       </c>
       <c r="C18" s="24" t="s">
         <v>42</v>
       </c>
       <c r="D18" s="48" t="s">
-        <v>299</v>
+        <v>295</v>
       </c>
       <c r="E18" s="14" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="F18" s="14" t="s">
         <v>43</v>
       </c>
       <c r="G18" s="23" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="H18" s="129" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
       <c r="I18" s="44" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="J18" s="14" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="K18" s="16">
         <v>4</v>
@@ -3683,7 +3719,7 @@
         <v>10</v>
       </c>
       <c r="O18" s="111" t="s">
-        <v>315</v>
+        <v>311</v>
       </c>
       <c r="P18" s="18">
         <v>2.9</v>
@@ -3700,14 +3736,14 @@
         <v>37.699999999999996</v>
       </c>
       <c r="T18" s="130" t="s">
-        <v>258</v>
+        <v>255</v>
       </c>
     </row>
     <row r="19" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="27">
         <v>17</v>
       </c>
-      <c r="B19" s="153"/>
+      <c r="B19" s="192"/>
       <c r="C19" s="26" t="s">
         <v>44</v>
       </c>
@@ -3715,22 +3751,22 @@
         <v>45</v>
       </c>
       <c r="E19" s="8" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="F19" s="8" t="s">
         <v>46</v>
       </c>
       <c r="G19" s="22" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="H19" s="9" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="I19" s="46" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="J19" s="8" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="K19" s="10">
         <v>2</v>
@@ -3746,7 +3782,7 @@
         <v>5</v>
       </c>
       <c r="O19" s="21" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="P19" s="13">
         <v>0.34520000000000001</v>
@@ -3768,7 +3804,7 @@
       <c r="A20" s="27">
         <v>18</v>
       </c>
-      <c r="B20" s="155" t="s">
+      <c r="B20" s="194" t="s">
         <v>47</v>
       </c>
       <c r="C20" s="85" t="s">
@@ -3778,7 +3814,7 @@
         <v>49</v>
       </c>
       <c r="E20" s="87" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="F20" s="87" t="s">
         <v>50</v>
@@ -3787,13 +3823,13 @@
         <v>37</v>
       </c>
       <c r="H20" s="95" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="I20" s="96" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="J20" s="94" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="K20" s="97">
         <v>20</v>
@@ -3804,12 +3840,12 @@
       <c r="M20" s="95">
         <v>2</v>
       </c>
-      <c r="N20" s="174">
+      <c r="N20" s="161">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
       <c r="O20" s="98" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="P20" s="88">
         <v>3.49E-2</v>
@@ -3831,28 +3867,28 @@
       <c r="A21" s="27">
         <v>19</v>
       </c>
-      <c r="B21" s="152"/>
+      <c r="B21" s="191"/>
       <c r="C21" s="25" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="D21" s="49" t="s">
         <v>52</v>
       </c>
       <c r="E21" s="4" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="F21" s="4" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="G21" s="35" t="s">
         <v>54</v>
       </c>
       <c r="H21" s="6"/>
       <c r="I21" s="47" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="J21" s="34" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="K21" s="34"/>
       <c r="L21" s="34"/>
@@ -3880,15 +3916,15 @@
       <c r="A22" s="27">
         <v>20</v>
       </c>
-      <c r="B22" s="153"/>
+      <c r="B22" s="192"/>
       <c r="C22" s="26" t="s">
         <v>51</v>
       </c>
       <c r="D22" s="51" t="s">
-        <v>284</v>
+        <v>280</v>
       </c>
       <c r="E22" s="8" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="F22" s="8" t="s">
         <v>53</v>
@@ -3896,14 +3932,14 @@
       <c r="G22" s="21" t="s">
         <v>54</v>
       </c>
-      <c r="H22" s="194" t="s">
-        <v>334</v>
+      <c r="H22" s="178" t="s">
+        <v>330</v>
       </c>
       <c r="I22" s="81" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="J22" s="74" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="K22" s="76">
         <v>10</v>
@@ -3919,7 +3955,7 @@
         <v>5</v>
       </c>
       <c r="O22" s="109" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="P22" s="13">
         <v>5.74E-2</v>
@@ -3941,14 +3977,14 @@
       <c r="A23" s="27">
         <v>21</v>
       </c>
-      <c r="B23" s="151" t="s">
-        <v>203</v>
+      <c r="B23" s="190" t="s">
+        <v>200</v>
       </c>
       <c r="C23" s="40" t="s">
         <v>55</v>
       </c>
       <c r="D23" s="48" t="s">
-        <v>287</v>
+        <v>283</v>
       </c>
       <c r="E23" s="14" t="s">
         <v>56</v>
@@ -3957,16 +3993,16 @@
         <v>57</v>
       </c>
       <c r="G23" s="23" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="H23" s="17" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
       <c r="I23" s="17" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="J23" s="14" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="K23" s="16">
         <v>10</v>
@@ -3982,7 +4018,7 @@
         <v>35</v>
       </c>
       <c r="O23" s="15" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="P23" s="18">
         <v>5.5399999999999998E-2</v>
@@ -3999,19 +4035,19 @@
         <v>2.2159999999999997</v>
       </c>
       <c r="T23" s="104" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
     </row>
     <row r="24" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="27">
         <v>22</v>
       </c>
-      <c r="B24" s="152"/>
+      <c r="B24" s="191"/>
       <c r="C24" s="25" t="s">
         <v>58</v>
       </c>
       <c r="D24" s="49" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="E24" s="4" t="s">
         <v>56</v>
@@ -4023,13 +4059,13 @@
         <v>61</v>
       </c>
       <c r="H24" s="6" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="I24" s="45" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="J24" s="4" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="K24" s="5">
         <v>100</v>
@@ -4045,7 +4081,7 @@
         <v>5</v>
       </c>
       <c r="O24" s="1" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="P24" s="12">
         <v>1.8E-3</v>
@@ -4067,30 +4103,30 @@
       <c r="A25" s="27">
         <v>23</v>
       </c>
-      <c r="B25" s="152"/>
+      <c r="B25" s="191"/>
       <c r="C25" s="25" t="s">
-        <v>301</v>
+        <v>297</v>
       </c>
       <c r="D25" s="49" t="s">
-        <v>291</v>
+        <v>287</v>
       </c>
       <c r="E25" s="4" t="s">
         <v>56</v>
       </c>
       <c r="F25" s="4" t="s">
-        <v>302</v>
+        <v>298</v>
       </c>
       <c r="G25" s="1" t="s">
         <v>61</v>
       </c>
       <c r="H25" s="6" t="s">
-        <v>313</v>
+        <v>309</v>
       </c>
       <c r="I25" s="45" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="J25" s="4" t="s">
-        <v>300</v>
+        <v>296</v>
       </c>
       <c r="K25" s="5">
         <v>100</v>
@@ -4106,7 +4142,7 @@
         <v>5</v>
       </c>
       <c r="O25" s="105" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="P25" s="12">
         <v>1.1999999999999999E-3</v>
@@ -4128,30 +4164,30 @@
       <c r="A26" s="27">
         <v>24</v>
       </c>
-      <c r="B26" s="152"/>
+      <c r="B26" s="191"/>
       <c r="C26" s="25" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="D26" s="49" t="s">
-        <v>290</v>
+        <v>286</v>
       </c>
       <c r="E26" s="4" t="s">
         <v>56</v>
       </c>
       <c r="F26" s="4" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="G26" s="1" t="s">
         <v>61</v>
       </c>
       <c r="H26" s="6" t="s">
-        <v>240</v>
+        <v>237</v>
       </c>
       <c r="I26" s="45" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="J26" s="34" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="K26" s="34">
         <v>100</v>
@@ -4167,7 +4203,7 @@
         <v>5</v>
       </c>
       <c r="O26" s="35" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="P26" s="37">
         <v>1.5E-3</v>
@@ -4189,30 +4225,30 @@
       <c r="A27" s="27">
         <v>25</v>
       </c>
-      <c r="B27" s="152"/>
+      <c r="B27" s="191"/>
       <c r="C27" s="42" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="D27" s="49" t="s">
-        <v>288</v>
+        <v>284</v>
       </c>
       <c r="E27" s="4" t="s">
         <v>56</v>
       </c>
       <c r="F27" s="112" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="G27" s="3" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="H27" s="6" t="s">
-        <v>245</v>
+        <v>242</v>
       </c>
       <c r="I27" s="45" t="s">
-        <v>244</v>
+        <v>241</v>
       </c>
       <c r="J27" s="4" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="K27" s="4">
         <v>20</v>
@@ -4228,7 +4264,7 @@
         <v>15</v>
       </c>
       <c r="O27" s="1" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="P27" s="12">
         <v>1.95E-2</v>
@@ -4245,19 +4281,19 @@
         <v>0.39</v>
       </c>
       <c r="T27" s="99" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
     </row>
     <row r="28" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="27">
         <v>26</v>
       </c>
-      <c r="B28" s="152"/>
+      <c r="B28" s="191"/>
       <c r="C28" s="25" t="s">
         <v>62</v>
       </c>
       <c r="D28" s="49" t="s">
-        <v>286</v>
+        <v>282</v>
       </c>
       <c r="E28" s="4" t="s">
         <v>56</v>
@@ -4266,16 +4302,16 @@
         <v>63</v>
       </c>
       <c r="G28" s="3" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="H28" s="6" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
       <c r="I28" s="45" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="J28" s="4" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="K28" s="4">
         <v>100</v>
@@ -4291,7 +4327,7 @@
         <v>5</v>
       </c>
       <c r="O28" s="1" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="P28" s="12">
         <v>1.4E-3</v>
@@ -4308,19 +4344,19 @@
         <v>0.13999999999999999</v>
       </c>
       <c r="T28" s="99" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
     </row>
     <row r="29" spans="1:20" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A29" s="27">
         <v>27</v>
       </c>
-      <c r="B29" s="152"/>
+      <c r="B29" s="191"/>
       <c r="C29" s="42" t="s">
         <v>64</v>
       </c>
       <c r="D29" s="49" t="s">
-        <v>289</v>
+        <v>285</v>
       </c>
       <c r="E29" s="4" t="s">
         <v>56</v>
@@ -4329,16 +4365,16 @@
         <v>65</v>
       </c>
       <c r="G29" s="3" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="H29" s="6" t="s">
-        <v>243</v>
+        <v>240</v>
       </c>
       <c r="I29" s="143" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="J29" s="4" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="K29" s="4">
         <v>20</v>
@@ -4354,7 +4390,7 @@
         <v>5</v>
       </c>
       <c r="O29" s="1" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="P29" s="12">
         <v>1.35E-2</v>
@@ -4376,12 +4412,12 @@
       <c r="A30" s="27">
         <v>28</v>
       </c>
-      <c r="B30" s="152"/>
+      <c r="B30" s="191"/>
       <c r="C30" s="25" t="s">
         <v>66</v>
       </c>
       <c r="D30" s="49" t="s">
-        <v>285</v>
+        <v>281</v>
       </c>
       <c r="E30" s="4" t="s">
         <v>56</v>
@@ -4390,16 +4426,16 @@
         <v>67</v>
       </c>
       <c r="G30" s="3" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="H30" s="6" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="I30" s="6" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="J30" s="4" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="K30" s="5">
         <v>20</v>
@@ -4415,7 +4451,7 @@
         <v>20</v>
       </c>
       <c r="O30" s="1" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="P30" s="12">
         <v>2.0400000000000001E-2</v>
@@ -4432,14 +4468,14 @@
         <v>0.81600000000000006</v>
       </c>
       <c r="T30" s="99" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
     </row>
     <row r="31" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="27">
         <v>29</v>
       </c>
-      <c r="B31" s="152"/>
+      <c r="B31" s="191"/>
       <c r="C31" s="25" t="s">
         <v>68</v>
       </c>
@@ -4453,16 +4489,16 @@
         <v>69</v>
       </c>
       <c r="G31" s="3" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="H31" s="6" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="I31" s="6" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="J31" s="4" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="K31" s="5">
         <v>100</v>
@@ -4478,7 +4514,7 @@
         <v>5</v>
       </c>
       <c r="O31" s="1" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="P31" s="12">
         <v>1.4E-3</v>
@@ -4495,33 +4531,33 @@
         <v>0.13999999999999999</v>
       </c>
       <c r="T31" s="99" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
     </row>
     <row r="32" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="27">
         <v>30</v>
       </c>
-      <c r="B32" s="152"/>
+      <c r="B32" s="191"/>
       <c r="C32" s="25" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="D32" s="49" t="s">
         <v>70</v>
       </c>
       <c r="E32" s="4" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="F32" s="4" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="G32" s="43" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="H32" s="6"/>
       <c r="I32" s="45"/>
       <c r="J32" s="4" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="K32" s="4"/>
       <c r="L32" s="4"/>
@@ -4544,14 +4580,14 @@
         <v>0</v>
       </c>
       <c r="T32" s="99" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
     </row>
     <row r="33" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A33" s="27">
         <v>31</v>
       </c>
-      <c r="B33" s="152"/>
+      <c r="B33" s="191"/>
       <c r="C33" s="25" t="s">
         <v>71</v>
       </c>
@@ -4565,16 +4601,16 @@
         <v>73</v>
       </c>
       <c r="G33" s="3" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="H33" s="6" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="I33" s="6" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="J33" s="4" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="K33" s="5">
         <v>100</v>
@@ -4590,7 +4626,7 @@
         <v>5</v>
       </c>
       <c r="O33" s="1" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="P33" s="12">
         <v>1.5E-3</v>
@@ -4607,14 +4643,14 @@
         <v>0.15</v>
       </c>
       <c r="T33" s="99" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
     </row>
     <row r="34" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A34" s="27">
         <v>32</v>
       </c>
-      <c r="B34" s="152"/>
+      <c r="B34" s="191"/>
       <c r="C34" s="25" t="s">
         <v>74</v>
       </c>
@@ -4628,16 +4664,16 @@
         <v>76</v>
       </c>
       <c r="G34" s="3" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="H34" s="6" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="I34" s="72" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="J34" s="4" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="K34" s="5">
         <v>100</v>
@@ -4653,7 +4689,7 @@
         <v>5</v>
       </c>
       <c r="O34" s="1" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="P34" s="12">
         <v>1.5E-3</v>
@@ -4670,14 +4706,14 @@
         <v>0.15</v>
       </c>
       <c r="T34" s="99" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
     </row>
     <row r="35" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A35" s="27">
         <v>33</v>
       </c>
-      <c r="B35" s="153"/>
+      <c r="B35" s="192"/>
       <c r="C35" s="26" t="s">
         <v>77</v>
       </c>
@@ -4691,16 +4727,16 @@
         <v>79</v>
       </c>
       <c r="G35" s="21" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="H35" s="9" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="I35" s="133" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="J35" s="8" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="K35" s="10">
         <v>100</v>
@@ -4716,7 +4752,7 @@
         <v>20</v>
       </c>
       <c r="O35" s="21" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="P35" s="13">
         <v>1.1999999999999999E-3</v>
@@ -4733,77 +4769,77 @@
         <v>0.12</v>
       </c>
       <c r="T35" s="110" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
     </row>
     <row r="36" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A36" s="27">
         <v>34</v>
       </c>
-      <c r="B36" s="161" t="s">
+      <c r="B36" s="148" t="s">
         <v>80</v>
       </c>
-      <c r="C36" s="162" t="s">
+      <c r="C36" s="149" t="s">
+        <v>180</v>
+      </c>
+      <c r="D36" s="150" t="s">
+        <v>81</v>
+      </c>
+      <c r="E36" s="151" t="s">
+        <v>155</v>
+      </c>
+      <c r="F36" s="151" t="s">
+        <v>181</v>
+      </c>
+      <c r="G36" s="152" t="s">
         <v>182</v>
       </c>
-      <c r="D36" s="163" t="s">
-        <v>81</v>
-      </c>
-      <c r="E36" s="164" t="s">
-        <v>157</v>
-      </c>
-      <c r="F36" s="164" t="s">
-        <v>183</v>
-      </c>
-      <c r="G36" s="165" t="s">
-        <v>184</v>
-      </c>
-      <c r="H36" s="166" t="s">
-        <v>246</v>
-      </c>
-      <c r="I36" s="167" t="s">
-        <v>156</v>
-      </c>
-      <c r="J36" s="164" t="s">
-        <v>153</v>
-      </c>
-      <c r="K36" s="164">
+      <c r="H36" s="153" t="s">
+        <v>243</v>
+      </c>
+      <c r="I36" s="154" t="s">
+        <v>154</v>
+      </c>
+      <c r="J36" s="151" t="s">
+        <v>151</v>
+      </c>
+      <c r="K36" s="151">
         <v>2</v>
       </c>
-      <c r="L36" s="164">
+      <c r="L36" s="151">
         <v>10</v>
       </c>
-      <c r="M36" s="166">
+      <c r="M36" s="153">
         <v>1</v>
       </c>
-      <c r="N36" s="168">
+      <c r="N36" s="155">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="O36" s="169" t="s">
-        <v>215</v>
-      </c>
-      <c r="P36" s="170">
+      <c r="O36" s="156" t="s">
+        <v>212</v>
+      </c>
+      <c r="P36" s="157">
         <v>0.93959999999999999</v>
       </c>
-      <c r="Q36" s="171">
+      <c r="Q36" s="158">
         <f t="shared" si="2"/>
         <v>1.8792</v>
       </c>
-      <c r="R36" s="170">
+      <c r="R36" s="157">
         <v>0.67810000000000004</v>
       </c>
-      <c r="S36" s="171">
+      <c r="S36" s="158">
         <f t="shared" si="1"/>
         <v>6.7810000000000006</v>
       </c>
-      <c r="T36" s="172"/>
+      <c r="T36" s="159"/>
     </row>
     <row r="37" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A37" s="27">
         <v>35</v>
       </c>
-      <c r="B37" s="151" t="s">
+      <c r="B37" s="190" t="s">
         <v>82</v>
       </c>
       <c r="C37" s="68" t="s">
@@ -4813,22 +4849,22 @@
         <v>84</v>
       </c>
       <c r="E37" s="48" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="F37" s="14" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="G37" s="15" t="s">
         <v>85</v>
       </c>
       <c r="H37" s="17" t="s">
-        <v>331</v>
+        <v>327</v>
       </c>
       <c r="I37" s="83" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="J37" s="48" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="K37" s="48">
         <v>2</v>
@@ -4843,8 +4879,8 @@
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="O37" s="195" t="s">
-        <v>215</v>
+      <c r="O37" s="179" t="s">
+        <v>212</v>
       </c>
       <c r="P37" s="70">
         <v>4.4379</v>
@@ -4866,7 +4902,7 @@
       <c r="A38" s="27">
         <v>36</v>
       </c>
-      <c r="B38" s="152"/>
+      <c r="B38" s="191"/>
       <c r="C38" s="33" t="s">
         <v>86</v>
       </c>
@@ -4883,13 +4919,13 @@
         <v>94</v>
       </c>
       <c r="H38" s="6" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="I38" s="143" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="J38" s="34" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="K38" s="34">
         <v>2</v>
@@ -4904,8 +4940,8 @@
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="O38" s="196" t="s">
-        <v>315</v>
+      <c r="O38" s="180" t="s">
+        <v>311</v>
       </c>
       <c r="P38" s="37">
         <v>1.6</v>
@@ -4922,14 +4958,14 @@
         <v>9.6000000000000014</v>
       </c>
       <c r="T38" s="100" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
     </row>
     <row r="39" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A39" s="27">
         <v>37</v>
       </c>
-      <c r="B39" s="152"/>
+      <c r="B39" s="191"/>
       <c r="C39" s="25" t="s">
         <v>90</v>
       </c>
@@ -4937,7 +4973,7 @@
         <v>87</v>
       </c>
       <c r="E39" s="4" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="F39" s="4" t="s">
         <v>92</v>
@@ -4946,13 +4982,13 @@
         <v>102</v>
       </c>
       <c r="H39" s="3" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="I39" s="143" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="J39" s="4" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="K39" s="4">
         <v>2</v>
@@ -4967,8 +5003,8 @@
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="O39" s="196" t="s">
-        <v>315</v>
+      <c r="O39" s="180" t="s">
+        <v>311</v>
       </c>
       <c r="P39" s="12">
         <v>1.5</v>
@@ -4985,37 +5021,37 @@
         <v>9</v>
       </c>
       <c r="T39" s="103" t="s">
-        <v>316</v>
+        <v>312</v>
       </c>
     </row>
     <row r="40" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A40" s="27">
         <v>38</v>
       </c>
-      <c r="B40" s="152"/>
+      <c r="B40" s="191"/>
       <c r="C40" s="25" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="D40" s="49" t="s">
         <v>93</v>
       </c>
       <c r="E40" s="4" t="s">
+        <v>185</v>
+      </c>
+      <c r="F40" s="4" t="s">
+        <v>186</v>
+      </c>
+      <c r="G40" s="1" t="s">
         <v>187</v>
       </c>
-      <c r="F40" s="4" t="s">
-        <v>188</v>
-      </c>
-      <c r="G40" s="1" t="s">
-        <v>189</v>
-      </c>
       <c r="H40" s="6" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="I40" s="143" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="J40" s="4" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="K40" s="4"/>
       <c r="L40" s="4"/>
@@ -5043,7 +5079,7 @@
       <c r="A41" s="27">
         <v>39</v>
       </c>
-      <c r="B41" s="152"/>
+      <c r="B41" s="191"/>
       <c r="C41" s="33" t="s">
         <v>95</v>
       </c>
@@ -5051,7 +5087,7 @@
         <v>96</v>
       </c>
       <c r="E41" s="80" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="F41" s="34" t="s">
         <v>97</v>
@@ -5060,13 +5096,13 @@
         <v>98</v>
       </c>
       <c r="H41" s="6" t="s">
-        <v>247</v>
+        <v>244</v>
       </c>
       <c r="I41" s="143" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="J41" s="34" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="K41" s="34">
         <v>2</v>
@@ -5082,7 +5118,7 @@
         <v>5</v>
       </c>
       <c r="O41" s="35" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="P41" s="37">
         <v>0.58430000000000004</v>
@@ -5104,12 +5140,12 @@
       <c r="A42" s="27">
         <v>40</v>
       </c>
-      <c r="B42" s="152"/>
+      <c r="B42" s="191"/>
       <c r="C42" s="25" t="s">
         <v>99</v>
       </c>
       <c r="D42" s="49" t="s">
-        <v>332</v>
+        <v>328</v>
       </c>
       <c r="E42" s="4" t="s">
         <v>100</v>
@@ -5121,13 +5157,13 @@
         <v>94</v>
       </c>
       <c r="H42" s="6" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="I42" s="143" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="J42" s="4" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="K42" s="4">
         <v>4</v>
@@ -5143,7 +5179,7 @@
         <v>15</v>
       </c>
       <c r="O42" s="1" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="P42" s="12">
         <v>0.22459999999999999</v>
@@ -5165,28 +5201,28 @@
       <c r="A43" s="27">
         <v>41</v>
       </c>
-      <c r="B43" s="152"/>
+      <c r="B43" s="191"/>
       <c r="C43" s="25" t="s">
+        <v>188</v>
+      </c>
+      <c r="D43" s="50" t="s">
+        <v>189</v>
+      </c>
+      <c r="E43" s="4" t="s">
         <v>190</v>
       </c>
-      <c r="D43" s="50" t="s">
+      <c r="F43" s="4" t="s">
         <v>191</v>
       </c>
-      <c r="E43" s="4" t="s">
-        <v>192</v>
-      </c>
-      <c r="F43" s="4" t="s">
-        <v>193</v>
-      </c>
       <c r="G43" s="35" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="H43" s="6"/>
       <c r="I43" s="143" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="J43" s="34" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="K43" s="34">
         <v>1</v>
@@ -5216,27 +5252,27 @@
       <c r="A44" s="27">
         <v>42</v>
       </c>
-      <c r="B44" s="152"/>
+      <c r="B44" s="191"/>
       <c r="C44" s="25" t="s">
+        <v>192</v>
+      </c>
+      <c r="D44" s="50" t="s">
+        <v>193</v>
+      </c>
+      <c r="E44" s="4" t="s">
         <v>194</v>
       </c>
-      <c r="D44" s="50" t="s">
+      <c r="F44" s="4" t="s">
         <v>195</v>
       </c>
-      <c r="E44" s="4" t="s">
-        <v>196</v>
-      </c>
-      <c r="F44" s="4" t="s">
+      <c r="G44" s="1" t="s">
         <v>197</v>
       </c>
-      <c r="G44" s="1" t="s">
-        <v>199</v>
-      </c>
       <c r="H44" s="6" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="I44" s="45" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="J44" s="4"/>
       <c r="K44" s="4">
@@ -5253,7 +5289,7 @@
         <v>5</v>
       </c>
       <c r="O44" s="105" t="s">
-        <v>315</v>
+        <v>311</v>
       </c>
       <c r="P44" s="12">
         <v>1</v>
@@ -5270,37 +5306,37 @@
         <v>6</v>
       </c>
       <c r="T44" s="100" t="s">
-        <v>259</v>
+        <v>256</v>
       </c>
     </row>
     <row r="45" spans="1:20" s="116" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A45" s="27">
         <v>43</v>
       </c>
-      <c r="B45" s="153"/>
+      <c r="B45" s="192"/>
       <c r="C45" s="26" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="D45" s="51" t="s">
         <v>103</v>
       </c>
       <c r="E45" s="8" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="F45" s="8" t="s">
         <v>104</v>
       </c>
       <c r="G45" s="115" t="s">
+        <v>149</v>
+      </c>
+      <c r="H45" s="9" t="s">
         <v>151</v>
       </c>
-      <c r="H45" s="9" t="s">
-        <v>153</v>
-      </c>
       <c r="I45" s="46" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="J45" s="8" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="K45" s="8">
         <v>2</v>
@@ -5315,8 +5351,8 @@
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="O45" s="197" t="s">
-        <v>315</v>
+      <c r="O45" s="181" t="s">
+        <v>311</v>
       </c>
       <c r="P45" s="13">
         <v>9.3000000000000007</v>
@@ -5332,25 +5368,25 @@
         <f t="shared" si="1"/>
         <v>55.800000000000004</v>
       </c>
-      <c r="T45" s="198" t="s">
-        <v>261</v>
+      <c r="T45" s="182" t="s">
+        <v>258</v>
       </c>
     </row>
     <row r="46" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A46" s="27">
         <v>44</v>
       </c>
-      <c r="B46" s="151" t="s">
+      <c r="B46" s="190" t="s">
         <v>105</v>
       </c>
       <c r="C46" s="24" t="s">
-        <v>200</v>
-      </c>
-      <c r="D46" s="48" t="s">
-        <v>282</v>
+        <v>198</v>
+      </c>
+      <c r="D46" s="50" t="s">
+        <v>332</v>
       </c>
       <c r="E46" s="14" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="F46" s="14" t="s">
         <v>106</v>
@@ -5359,29 +5395,29 @@
         <v>107</v>
       </c>
       <c r="H46" s="77" t="s">
-        <v>234</v>
+        <v>231</v>
       </c>
       <c r="I46" s="44" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="J46" s="14" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="K46" s="16">
         <v>20</v>
       </c>
       <c r="L46" s="16">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="M46" s="17">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="N46" s="16">
         <f t="shared" si="0"/>
-        <v>40</v>
+        <v>25</v>
       </c>
       <c r="O46" s="15" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="P46" s="18">
         <v>3.1E-2</v>
@@ -5395,7 +5431,7 @@
       </c>
       <c r="S46" s="78">
         <f t="shared" si="1"/>
-        <v>1.8599999999999999</v>
+        <v>1.24</v>
       </c>
       <c r="T46" s="104"/>
     </row>
@@ -5403,60 +5439,60 @@
       <c r="A47" s="27">
         <v>45</v>
       </c>
-      <c r="B47" s="152"/>
+      <c r="B47" s="191"/>
       <c r="C47" s="25" t="s">
         <v>108</v>
       </c>
       <c r="D47" s="49" t="s">
+        <v>333</v>
+      </c>
+      <c r="E47" s="4" t="s">
+        <v>155</v>
+      </c>
+      <c r="F47" s="4" t="s">
         <v>109</v>
-      </c>
-      <c r="E47" s="4" t="s">
-        <v>157</v>
-      </c>
-      <c r="F47" s="4" t="s">
-        <v>110</v>
       </c>
       <c r="G47" s="1" t="s">
         <v>107</v>
       </c>
       <c r="H47" s="72" t="s">
-        <v>235</v>
+        <v>232</v>
       </c>
       <c r="I47" s="45" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="J47" s="4" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="K47" s="5">
         <v>10</v>
       </c>
       <c r="L47" s="5">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="M47" s="6">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N47" s="5">
         <f t="shared" si="0"/>
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="O47" s="1" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="P47" s="12">
         <v>4.9700000000000001E-2</v>
       </c>
       <c r="Q47" s="11">
         <f>P47*M47</f>
-        <v>0.14910000000000001</v>
+        <v>4.9700000000000001E-2</v>
       </c>
       <c r="R47" s="12">
         <v>4.9700000000000001E-2</v>
       </c>
       <c r="S47" s="11">
         <f t="shared" si="1"/>
-        <v>0.99399999999999999</v>
+        <v>0.497</v>
       </c>
       <c r="T47" s="99"/>
     </row>
@@ -5464,46 +5500,46 @@
       <c r="A48" s="27">
         <v>46</v>
       </c>
-      <c r="B48" s="152"/>
+      <c r="B48" s="191"/>
       <c r="C48" s="25" t="s">
+        <v>110</v>
+      </c>
+      <c r="D48" s="49" t="s">
+        <v>335</v>
+      </c>
+      <c r="E48" s="4" t="s">
+        <v>155</v>
+      </c>
+      <c r="F48" s="4" t="s">
         <v>111</v>
-      </c>
-      <c r="D48" s="49" t="s">
-        <v>201</v>
-      </c>
-      <c r="E48" s="4" t="s">
-        <v>157</v>
-      </c>
-      <c r="F48" s="4" t="s">
-        <v>112</v>
       </c>
       <c r="G48" s="1" t="s">
         <v>107</v>
       </c>
       <c r="H48" s="6" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="I48" s="45" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="J48" s="4" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="K48" s="5">
         <v>10</v>
       </c>
       <c r="L48" s="5">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="M48" s="6">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="N48" s="5">
         <f t="shared" si="0"/>
-        <v>25</v>
+        <v>5</v>
       </c>
       <c r="O48" s="105" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="P48" s="12">
         <v>4.5699999999999998E-2</v>
@@ -5517,7 +5553,7 @@
       </c>
       <c r="S48" s="11">
         <f t="shared" si="1"/>
-        <v>1.371</v>
+        <v>0.45699999999999996</v>
       </c>
       <c r="T48" s="99"/>
     </row>
@@ -5525,30 +5561,30 @@
       <c r="A49" s="27">
         <v>47</v>
       </c>
-      <c r="B49" s="152"/>
+      <c r="B49" s="191"/>
       <c r="C49" s="25" t="s">
+        <v>112</v>
+      </c>
+      <c r="D49" s="49" t="s">
+        <v>334</v>
+      </c>
+      <c r="E49" s="4" t="s">
+        <v>155</v>
+      </c>
+      <c r="F49" s="4" t="s">
         <v>113</v>
-      </c>
-      <c r="D49" s="49" t="s">
-        <v>114</v>
-      </c>
-      <c r="E49" s="4" t="s">
-        <v>157</v>
-      </c>
-      <c r="F49" s="4" t="s">
-        <v>115</v>
       </c>
       <c r="G49" s="1" t="s">
         <v>107</v>
       </c>
       <c r="H49" s="72" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="I49" s="45" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="J49" s="4" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="K49" s="5">
         <v>5</v>
@@ -5564,7 +5600,7 @@
         <v>10</v>
       </c>
       <c r="O49" s="1" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="P49" s="12">
         <v>0.10340000000000001</v>
@@ -5586,30 +5622,30 @@
       <c r="A50" s="27">
         <v>48</v>
       </c>
-      <c r="B50" s="152"/>
+      <c r="B50" s="191"/>
       <c r="C50" s="25" t="s">
+        <v>114</v>
+      </c>
+      <c r="D50" s="49" t="s">
+        <v>115</v>
+      </c>
+      <c r="E50" s="4" t="s">
+        <v>155</v>
+      </c>
+      <c r="F50" s="4" t="s">
         <v>116</v>
       </c>
-      <c r="D50" s="49" t="s">
+      <c r="G50" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="E50" s="4" t="s">
-        <v>157</v>
-      </c>
-      <c r="F50" s="4" t="s">
-        <v>118</v>
-      </c>
-      <c r="G50" s="2" t="s">
-        <v>119</v>
-      </c>
       <c r="H50" s="6" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="I50" s="45" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="J50" s="4" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="K50" s="5">
         <v>2</v>
@@ -5625,7 +5661,7 @@
         <v>5</v>
       </c>
       <c r="O50" s="1" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="P50" s="12">
         <v>2.1766000000000001</v>
@@ -5644,277 +5680,345 @@
       <c r="T50" s="99"/>
     </row>
     <row r="51" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A51" s="27">
-        <v>49</v>
-      </c>
-      <c r="B51" s="154"/>
-      <c r="C51" s="67" t="s">
-        <v>205</v>
-      </c>
-      <c r="D51" s="61" t="s">
-        <v>206</v>
-      </c>
-      <c r="E51" s="61" t="s">
-        <v>157</v>
-      </c>
-      <c r="F51" s="62" t="s">
-        <v>207</v>
-      </c>
-      <c r="G51" s="63" t="s">
-        <v>158</v>
-      </c>
-      <c r="H51" s="63"/>
-      <c r="I51" s="63" t="s">
-        <v>158</v>
-      </c>
-      <c r="J51" s="63" t="s">
-        <v>296</v>
-      </c>
-      <c r="K51" s="63"/>
-      <c r="L51" s="63"/>
-      <c r="M51" s="64">
+      <c r="A51" s="27"/>
+      <c r="B51" s="193"/>
+      <c r="C51" s="25" t="s">
+        <v>336</v>
+      </c>
+      <c r="D51" s="49" t="s">
+        <v>337</v>
+      </c>
+      <c r="E51" s="4" t="s">
+        <v>155</v>
+      </c>
+      <c r="F51" s="4" t="s">
+        <v>338</v>
+      </c>
+      <c r="G51" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="H51" s="4" t="s">
+        <v>345</v>
+      </c>
+      <c r="I51" s="4" t="s">
+        <v>345</v>
+      </c>
+      <c r="J51" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="K51" s="5">
         <v>1</v>
       </c>
-      <c r="N51" s="64">
+      <c r="L51" s="5">
+        <v>1</v>
+      </c>
+      <c r="M51" s="6">
+        <v>2</v>
+      </c>
+      <c r="N51" s="5">
+        <f t="shared" si="0"/>
+        <v>10</v>
+      </c>
+      <c r="O51" s="105" t="s">
+        <v>346</v>
+      </c>
+      <c r="P51" s="12">
+        <v>1.1599999999999999</v>
+      </c>
+      <c r="Q51" s="79">
+        <f t="shared" si="2"/>
+        <v>1.1599999999999999</v>
+      </c>
+      <c r="R51" s="12">
+        <v>1.1599999999999999</v>
+      </c>
+      <c r="S51" s="82">
+        <f t="shared" si="1"/>
+        <v>1.1599999999999999</v>
+      </c>
+      <c r="T51" s="99"/>
+    </row>
+    <row r="52" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A52" s="27"/>
+      <c r="B52" s="193"/>
+      <c r="C52" s="25" t="s">
+        <v>339</v>
+      </c>
+      <c r="D52" s="49" t="s">
+        <v>340</v>
+      </c>
+      <c r="E52" s="4" t="s">
+        <v>155</v>
+      </c>
+      <c r="F52" s="4" t="s">
+        <v>341</v>
+      </c>
+      <c r="G52" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="H52" s="4" t="s">
+        <v>345</v>
+      </c>
+      <c r="I52" s="4" t="s">
+        <v>345</v>
+      </c>
+      <c r="J52" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="K52" s="5">
+        <v>1</v>
+      </c>
+      <c r="L52" s="5">
+        <v>1</v>
+      </c>
+      <c r="M52" s="6">
+        <v>1</v>
+      </c>
+      <c r="N52" s="5">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="O51" s="63" t="s">
-        <v>158</v>
-      </c>
-      <c r="P51" s="65" t="s">
-        <v>158</v>
-      </c>
-      <c r="Q51" s="65" t="s">
-        <v>158</v>
-      </c>
-      <c r="R51" s="65" t="s">
-        <v>158</v>
-      </c>
-      <c r="S51" s="65" t="s">
-        <v>158</v>
-      </c>
-      <c r="T51" s="66" t="s">
-        <v>159</v>
-      </c>
+      <c r="O52" s="105" t="s">
+        <v>346</v>
+      </c>
+      <c r="P52" s="12">
+        <v>0.77</v>
+      </c>
+      <c r="Q52" s="79">
+        <f t="shared" si="2"/>
+        <v>0.77</v>
+      </c>
+      <c r="R52" s="12">
+        <v>0.77</v>
+      </c>
+      <c r="S52" s="82">
+        <f t="shared" si="1"/>
+        <v>0.77</v>
+      </c>
+      <c r="T52" s="99"/>
     </row>
-    <row r="52" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A52" s="27">
+    <row r="53" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A53" s="27"/>
+      <c r="B53" s="193"/>
+      <c r="C53" s="25" t="s">
+        <v>342</v>
+      </c>
+      <c r="D53" s="49" t="s">
+        <v>343</v>
+      </c>
+      <c r="E53" s="4" t="s">
+        <v>155</v>
+      </c>
+      <c r="F53" s="4" t="s">
+        <v>344</v>
+      </c>
+      <c r="G53" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="H53" s="4" t="s">
+        <v>345</v>
+      </c>
+      <c r="I53" s="4" t="s">
+        <v>345</v>
+      </c>
+      <c r="J53" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="K53" s="5">
+        <v>1</v>
+      </c>
+      <c r="L53" s="5">
+        <v>3</v>
+      </c>
+      <c r="M53" s="6">
+        <v>5</v>
+      </c>
+      <c r="N53" s="5">
+        <f t="shared" si="0"/>
+        <v>25</v>
+      </c>
+      <c r="O53" s="105" t="s">
+        <v>346</v>
+      </c>
+      <c r="P53" s="12">
+        <v>0.73</v>
+      </c>
+      <c r="Q53" s="79">
+        <f t="shared" si="2"/>
+        <v>0.73</v>
+      </c>
+      <c r="R53" s="12">
+        <v>2.19</v>
+      </c>
+      <c r="S53" s="82">
+        <f t="shared" si="1"/>
+        <v>6.57</v>
+      </c>
+      <c r="T53" s="99"/>
+    </row>
+    <row r="54" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A54" s="27">
+        <v>49</v>
+      </c>
+      <c r="B54" s="193"/>
+      <c r="C54" s="67" t="s">
+        <v>202</v>
+      </c>
+      <c r="D54" s="61" t="s">
+        <v>203</v>
+      </c>
+      <c r="E54" s="61" t="s">
+        <v>155</v>
+      </c>
+      <c r="F54" s="62" t="s">
+        <v>204</v>
+      </c>
+      <c r="G54" s="63" t="s">
+        <v>156</v>
+      </c>
+      <c r="H54" s="63"/>
+      <c r="I54" s="63" t="s">
+        <v>156</v>
+      </c>
+      <c r="J54" s="63" t="s">
+        <v>292</v>
+      </c>
+      <c r="K54" s="63"/>
+      <c r="L54" s="63"/>
+      <c r="M54" s="64">
+        <v>1</v>
+      </c>
+      <c r="N54" s="64">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="O54" s="63" t="s">
+        <v>156</v>
+      </c>
+      <c r="P54" s="65" t="s">
+        <v>156</v>
+      </c>
+      <c r="Q54" s="65" t="s">
+        <v>156</v>
+      </c>
+      <c r="R54" s="65" t="s">
+        <v>156</v>
+      </c>
+      <c r="S54" s="65" t="s">
+        <v>156</v>
+      </c>
+      <c r="T54" s="66" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="55" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A55" s="27">
         <v>50</v>
       </c>
-      <c r="B52" s="153"/>
-      <c r="C52" s="54" t="s">
-        <v>120</v>
-      </c>
-      <c r="D52" s="55" t="s">
-        <v>283</v>
-      </c>
-      <c r="E52" s="55" t="s">
-        <v>157</v>
-      </c>
-      <c r="F52" s="56" t="s">
-        <v>138</v>
-      </c>
-      <c r="G52" s="57" t="s">
-        <v>158</v>
-      </c>
-      <c r="H52" s="57"/>
-      <c r="I52" s="57" t="s">
-        <v>158</v>
-      </c>
-      <c r="J52" s="57" t="s">
-        <v>297</v>
-      </c>
-      <c r="K52" s="57"/>
-      <c r="L52" s="57"/>
-      <c r="M52" s="58">
+      <c r="B55" s="192"/>
+      <c r="C55" s="54" t="s">
+        <v>118</v>
+      </c>
+      <c r="D55" s="55" t="s">
+        <v>279</v>
+      </c>
+      <c r="E55" s="55" t="s">
+        <v>155</v>
+      </c>
+      <c r="F55" s="56" t="s">
+        <v>136</v>
+      </c>
+      <c r="G55" s="57" t="s">
+        <v>156</v>
+      </c>
+      <c r="H55" s="57"/>
+      <c r="I55" s="57" t="s">
+        <v>156</v>
+      </c>
+      <c r="J55" s="57" t="s">
+        <v>293</v>
+      </c>
+      <c r="K55" s="57"/>
+      <c r="L55" s="57"/>
+      <c r="M55" s="58">
         <v>4</v>
       </c>
-      <c r="N52" s="199">
+      <c r="N55" s="183">
         <f t="shared" si="0"/>
         <v>20</v>
       </c>
-      <c r="O52" s="57" t="s">
-        <v>158</v>
-      </c>
-      <c r="P52" s="59" t="s">
-        <v>158</v>
-      </c>
-      <c r="Q52" s="59" t="s">
-        <v>158</v>
-      </c>
-      <c r="R52" s="59" t="s">
-        <v>158</v>
-      </c>
-      <c r="S52" s="59" t="s">
-        <v>158</v>
-      </c>
-      <c r="T52" s="60" t="s">
-        <v>159</v>
+      <c r="O55" s="57" t="s">
+        <v>156</v>
+      </c>
+      <c r="P55" s="59" t="s">
+        <v>156</v>
+      </c>
+      <c r="Q55" s="59" t="s">
+        <v>156</v>
+      </c>
+      <c r="R55" s="59" t="s">
+        <v>156</v>
+      </c>
+      <c r="S55" s="59" t="s">
+        <v>156</v>
+      </c>
+      <c r="T55" s="60" t="s">
+        <v>157</v>
       </c>
     </row>
-    <row r="53" spans="1:20" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A53" s="27">
+    <row r="56" spans="1:20" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A56" s="27">
         <v>51</v>
       </c>
-      <c r="B53" s="156" t="s">
-        <v>325</v>
-      </c>
-      <c r="C53" s="24" t="s">
-        <v>305</v>
-      </c>
-      <c r="D53" s="134"/>
-      <c r="E53" s="14" t="s">
-        <v>157</v>
-      </c>
-      <c r="F53" s="14" t="s">
-        <v>306</v>
-      </c>
-      <c r="G53" s="135"/>
-      <c r="H53" s="135"/>
-      <c r="I53" s="135"/>
-      <c r="J53" s="135"/>
-      <c r="K53" s="135"/>
-      <c r="L53" s="144"/>
-      <c r="M53" s="136">
+      <c r="B56" s="196" t="s">
+        <v>321</v>
+      </c>
+      <c r="C56" s="24" t="s">
+        <v>301</v>
+      </c>
+      <c r="D56" s="134"/>
+      <c r="E56" s="14" t="s">
+        <v>155</v>
+      </c>
+      <c r="F56" s="14" t="s">
+        <v>302</v>
+      </c>
+      <c r="G56" s="135"/>
+      <c r="H56" s="135"/>
+      <c r="I56" s="135"/>
+      <c r="J56" s="135"/>
+      <c r="K56" s="135"/>
+      <c r="L56" s="144"/>
+      <c r="M56" s="136">
         <v>2</v>
       </c>
-      <c r="N53" s="16">
+      <c r="N56" s="16">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="O53" s="111" t="s">
-        <v>317</v>
-      </c>
-      <c r="P53" s="135"/>
-      <c r="Q53" s="135"/>
-      <c r="R53" s="135"/>
-      <c r="S53" s="135"/>
-      <c r="T53" s="137"/>
+      <c r="O56" s="111" t="s">
+        <v>313</v>
+      </c>
+      <c r="P56" s="135"/>
+      <c r="Q56" s="135"/>
+      <c r="R56" s="135"/>
+      <c r="S56" s="135"/>
+      <c r="T56" s="137"/>
     </row>
-    <row r="54" spans="1:20" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A54" s="27">
+    <row r="57" spans="1:20" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A57" s="27">
         <v>52</v>
       </c>
-      <c r="B54" s="157"/>
-      <c r="C54" s="184" t="s">
-        <v>307</v>
-      </c>
-      <c r="D54" s="118"/>
-      <c r="E54" s="4" t="s">
-        <v>157</v>
-      </c>
-      <c r="F54" s="4" t="s">
-        <v>308</v>
-      </c>
-      <c r="G54" s="118"/>
-      <c r="H54" s="118"/>
-      <c r="I54" s="118"/>
-      <c r="J54" s="118"/>
-      <c r="K54" s="118"/>
-      <c r="L54" s="118"/>
-      <c r="M54" s="119">
-        <v>2</v>
-      </c>
-      <c r="N54" s="5">
-        <f t="shared" si="0"/>
-        <v>10</v>
-      </c>
-      <c r="O54" s="105" t="s">
-        <v>317</v>
-      </c>
-      <c r="P54" s="118"/>
-      <c r="Q54" s="118"/>
-      <c r="R54" s="118"/>
-      <c r="S54" s="118"/>
-      <c r="T54" s="138"/>
-    </row>
-    <row r="55" spans="1:20" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A55" s="27">
-        <v>53</v>
-      </c>
-      <c r="B55" s="157"/>
-      <c r="C55" s="184" t="s">
-        <v>322</v>
-      </c>
-      <c r="D55" s="118"/>
-      <c r="E55" s="4" t="s">
-        <v>157</v>
-      </c>
-      <c r="F55" s="4" t="s">
-        <v>318</v>
-      </c>
-      <c r="G55" s="118"/>
-      <c r="H55" s="118"/>
-      <c r="I55" s="118"/>
-      <c r="J55" s="118"/>
-      <c r="K55" s="118"/>
-      <c r="L55" s="118"/>
-      <c r="M55" s="119">
-        <v>1</v>
-      </c>
-      <c r="N55" s="5">
-        <f t="shared" si="0"/>
-        <v>5</v>
-      </c>
-      <c r="O55" s="105" t="s">
-        <v>317</v>
-      </c>
-      <c r="P55" s="118"/>
-      <c r="Q55" s="118"/>
-      <c r="R55" s="118"/>
-      <c r="S55" s="118"/>
-      <c r="T55" s="138"/>
-    </row>
-    <row r="56" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A56" s="27">
-        <v>54</v>
-      </c>
-      <c r="B56" s="157"/>
-      <c r="C56" s="184" t="s">
-        <v>321</v>
-      </c>
-      <c r="D56" s="118"/>
-      <c r="E56" s="4" t="s">
-        <v>157</v>
-      </c>
-      <c r="F56" s="4" t="s">
-        <v>319</v>
-      </c>
-      <c r="G56" s="118"/>
-      <c r="H56" s="118"/>
-      <c r="I56" s="118"/>
-      <c r="J56" s="118"/>
-      <c r="K56" s="118"/>
-      <c r="L56" s="118"/>
-      <c r="M56" s="119">
-        <v>1</v>
-      </c>
-      <c r="N56" s="5">
-        <f t="shared" si="0"/>
-        <v>5</v>
-      </c>
-      <c r="O56" s="105"/>
-      <c r="P56" s="118"/>
-      <c r="Q56" s="118"/>
-      <c r="R56" s="118"/>
-      <c r="S56" s="118"/>
-      <c r="T56" s="138"/>
-    </row>
-    <row r="57" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A57" s="27">
-        <v>55</v>
-      </c>
-      <c r="B57" s="157"/>
-      <c r="C57" s="184" t="s">
-        <v>320</v>
+      <c r="B57" s="195"/>
+      <c r="C57" s="168" t="s">
+        <v>303</v>
       </c>
       <c r="D57" s="118"/>
       <c r="E57" s="4" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="F57" s="4" t="s">
-        <v>326</v>
+        <v>304</v>
       </c>
       <c r="G57" s="118"/>
       <c r="H57" s="118"/>
@@ -5923,14 +6027,14 @@
       <c r="K57" s="118"/>
       <c r="L57" s="118"/>
       <c r="M57" s="119">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N57" s="5">
         <f t="shared" si="0"/>
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="O57" s="105" t="s">
-        <v>317</v>
+        <v>313</v>
       </c>
       <c r="P57" s="118"/>
       <c r="Q57" s="118"/>
@@ -5938,18 +6042,20 @@
       <c r="S57" s="118"/>
       <c r="T57" s="138"/>
     </row>
-    <row r="58" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:20" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A58" s="27">
-        <v>56</v>
-      </c>
-      <c r="B58" s="157"/>
-      <c r="C58" s="185"/>
+        <v>53</v>
+      </c>
+      <c r="B58" s="195"/>
+      <c r="C58" s="168" t="s">
+        <v>318</v>
+      </c>
       <c r="D58" s="118"/>
       <c r="E58" s="4" t="s">
-        <v>157</v>
-      </c>
-      <c r="F58" s="119" t="s">
-        <v>309</v>
+        <v>155</v>
+      </c>
+      <c r="F58" s="4" t="s">
+        <v>314</v>
       </c>
       <c r="G58" s="118"/>
       <c r="H58" s="118"/>
@@ -5964,98 +6070,220 @@
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="O58" s="118"/>
+      <c r="O58" s="105" t="s">
+        <v>313</v>
+      </c>
       <c r="P58" s="118"/>
       <c r="Q58" s="118"/>
       <c r="R58" s="118"/>
       <c r="S58" s="118"/>
       <c r="T58" s="138"/>
     </row>
-    <row r="59" spans="1:20" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A59" s="200">
+    <row r="59" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A59" s="27">
+        <v>54</v>
+      </c>
+      <c r="B59" s="195"/>
+      <c r="C59" s="168" t="s">
+        <v>317</v>
+      </c>
+      <c r="D59" s="118"/>
+      <c r="E59" s="4" t="s">
+        <v>155</v>
+      </c>
+      <c r="F59" s="4" t="s">
+        <v>315</v>
+      </c>
+      <c r="G59" s="118"/>
+      <c r="H59" s="118"/>
+      <c r="I59" s="118"/>
+      <c r="J59" s="118"/>
+      <c r="K59" s="118"/>
+      <c r="L59" s="118"/>
+      <c r="M59" s="119">
+        <v>1</v>
+      </c>
+      <c r="N59" s="5">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="O59" s="105"/>
+      <c r="P59" s="118"/>
+      <c r="Q59" s="118"/>
+      <c r="R59" s="118"/>
+      <c r="S59" s="118"/>
+      <c r="T59" s="138"/>
+    </row>
+    <row r="60" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A60" s="27">
+        <v>55</v>
+      </c>
+      <c r="B60" s="195"/>
+      <c r="C60" s="168" t="s">
+        <v>316</v>
+      </c>
+      <c r="D60" s="118"/>
+      <c r="E60" s="4" t="s">
+        <v>155</v>
+      </c>
+      <c r="F60" s="4" t="s">
+        <v>322</v>
+      </c>
+      <c r="G60" s="118"/>
+      <c r="H60" s="118"/>
+      <c r="I60" s="118"/>
+      <c r="J60" s="118"/>
+      <c r="K60" s="118"/>
+      <c r="L60" s="118"/>
+      <c r="M60" s="119">
+        <v>1</v>
+      </c>
+      <c r="N60" s="5">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="O60" s="105" t="s">
+        <v>313</v>
+      </c>
+      <c r="P60" s="118"/>
+      <c r="Q60" s="118"/>
+      <c r="R60" s="118"/>
+      <c r="S60" s="118"/>
+      <c r="T60" s="138"/>
+    </row>
+    <row r="61" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A61" s="27">
+        <v>56</v>
+      </c>
+      <c r="B61" s="195"/>
+      <c r="C61" s="169"/>
+      <c r="D61" s="118"/>
+      <c r="E61" s="4" t="s">
+        <v>155</v>
+      </c>
+      <c r="F61" s="119" t="s">
+        <v>305</v>
+      </c>
+      <c r="G61" s="118"/>
+      <c r="H61" s="118"/>
+      <c r="I61" s="118"/>
+      <c r="J61" s="118"/>
+      <c r="K61" s="118"/>
+      <c r="L61" s="118"/>
+      <c r="M61" s="119">
+        <v>1</v>
+      </c>
+      <c r="N61" s="5">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="O61" s="118"/>
+      <c r="P61" s="118"/>
+      <c r="Q61" s="118"/>
+      <c r="R61" s="118"/>
+      <c r="S61" s="118"/>
+      <c r="T61" s="138"/>
+    </row>
+    <row r="62" spans="1:20" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A62" s="184">
         <v>57</v>
       </c>
-      <c r="B59" s="158"/>
-      <c r="C59" s="186" t="s">
-        <v>314</v>
-      </c>
-      <c r="D59" s="139"/>
-      <c r="E59" s="8" t="s">
-        <v>157</v>
-      </c>
-      <c r="F59" s="140" t="s">
+      <c r="B62" s="197"/>
+      <c r="C62" s="170" t="s">
         <v>310</v>
       </c>
-      <c r="G59" s="139"/>
-      <c r="H59" s="139"/>
-      <c r="I59" s="139"/>
-      <c r="J59" s="139"/>
-      <c r="K59" s="139"/>
-      <c r="L59" s="145"/>
-      <c r="M59" s="141">
+      <c r="D62" s="139"/>
+      <c r="E62" s="8" t="s">
+        <v>155</v>
+      </c>
+      <c r="F62" s="140" t="s">
+        <v>306</v>
+      </c>
+      <c r="G62" s="139"/>
+      <c r="H62" s="139"/>
+      <c r="I62" s="139"/>
+      <c r="J62" s="139"/>
+      <c r="K62" s="139"/>
+      <c r="L62" s="145"/>
+      <c r="M62" s="141">
         <v>2</v>
       </c>
-      <c r="N59" s="76">
+      <c r="N62" s="76">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="O59" s="109" t="s">
-        <v>317</v>
-      </c>
-      <c r="P59" s="139"/>
-      <c r="Q59" s="139"/>
-      <c r="R59" s="139"/>
-      <c r="S59" s="139"/>
-      <c r="T59" s="142"/>
+      <c r="O62" s="109" t="s">
+        <v>313</v>
+      </c>
+      <c r="P62" s="139"/>
+      <c r="Q62" s="139"/>
+      <c r="R62" s="139"/>
+      <c r="S62" s="139"/>
+      <c r="T62" s="142"/>
     </row>
-    <row r="60" spans="1:20" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="M60" s="149" t="s">
-        <v>154</v>
-      </c>
-      <c r="N60" s="149"/>
-      <c r="O60" s="149"/>
-      <c r="P60" s="149"/>
-      <c r="Q60" s="28"/>
-      <c r="R60" s="29"/>
-      <c r="S60" s="30">
-        <f>SUM(S3:S59)</f>
-        <v>193.27249999999998</v>
+    <row r="63" spans="1:20" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="M63" s="188" t="s">
+        <v>152</v>
+      </c>
+      <c r="N63" s="188"/>
+      <c r="O63" s="188"/>
+      <c r="P63" s="188"/>
+      <c r="Q63" s="28"/>
+      <c r="R63" s="29"/>
+      <c r="S63" s="30">
+        <f>SUM(S3:S62)</f>
+        <v>199.74149999999997</v>
       </c>
     </row>
-    <row r="61" spans="1:20" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="M61" s="150" t="s">
-        <v>155</v>
-      </c>
-      <c r="N61" s="150"/>
-      <c r="O61" s="150"/>
-      <c r="P61" s="150"/>
-      <c r="Q61" s="31">
-        <f>SUM(Q3:Q60)</f>
-        <v>60.550599999999996</v>
-      </c>
-      <c r="R61" s="32"/>
-      <c r="S61" s="31">
-        <f>S60/5</f>
-        <v>38.654499999999999</v>
+    <row r="64" spans="1:20" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="M64" s="189" t="s">
+        <v>153</v>
+      </c>
+      <c r="N64" s="189"/>
+      <c r="O64" s="189"/>
+      <c r="P64" s="189"/>
+      <c r="Q64" s="31">
+        <f>SUM(Q3:Q63)</f>
+        <v>63.111199999999997</v>
+      </c>
+      <c r="R64" s="32"/>
+      <c r="S64" s="31">
+        <f>S63/5</f>
+        <v>39.948299999999996</v>
+      </c>
+    </row>
+    <row r="66" spans="13:19" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="M66" s="189" t="s">
+        <v>347</v>
+      </c>
+      <c r="N66" s="189"/>
+      <c r="O66" s="189"/>
+      <c r="P66" s="189"/>
+      <c r="Q66" s="12">
+        <v>1.54</v>
+      </c>
+      <c r="S66" s="12">
+        <v>1.54</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="12">
+  <mergeCells count="13">
+    <mergeCell ref="M66:P66"/>
     <mergeCell ref="A1:T1"/>
-    <mergeCell ref="M60:P60"/>
-    <mergeCell ref="M61:P61"/>
+    <mergeCell ref="M63:P63"/>
+    <mergeCell ref="M64:P64"/>
     <mergeCell ref="B37:B45"/>
-    <mergeCell ref="B46:B52"/>
+    <mergeCell ref="B46:B55"/>
     <mergeCell ref="B18:B19"/>
     <mergeCell ref="B20:B22"/>
     <mergeCell ref="B23:B35"/>
     <mergeCell ref="B11:B13"/>
     <mergeCell ref="B3:B10"/>
-    <mergeCell ref="B53:B59"/>
+    <mergeCell ref="B56:B62"/>
     <mergeCell ref="B14:B17"/>
   </mergeCells>
   <phoneticPr fontId="17" type="noConversion"/>
-  <conditionalFormatting sqref="Q61">
+  <conditionalFormatting sqref="Q64">
     <cfRule type="dataBar" priority="6">
       <dataBar>
         <cfvo type="min"/>
@@ -6069,7 +6297,7 @@
       </extLst>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="S60:S61">
+  <conditionalFormatting sqref="S63:S64">
     <cfRule type="dataBar" priority="5">
       <dataBar>
         <cfvo type="min"/>
@@ -6083,7 +6311,7 @@
       </extLst>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="T52">
+  <conditionalFormatting sqref="T55">
     <cfRule type="dataBar" priority="21">
       <dataBar>
         <cfvo type="min"/>
@@ -6097,7 +6325,7 @@
       </extLst>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="M52:M59 M3:N50 N53:N59">
+  <conditionalFormatting sqref="M55:M62 M3:N53 N56:N62">
     <cfRule type="colorScale" priority="22">
       <colorScale>
         <cfvo type="min"/>
@@ -6109,7 +6337,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="M51">
+  <conditionalFormatting sqref="M54">
     <cfRule type="colorScale" priority="4">
       <colorScale>
         <cfvo type="min"/>
@@ -6121,7 +6349,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="T51">
+  <conditionalFormatting sqref="T54">
     <cfRule type="dataBar" priority="2">
       <dataBar>
         <cfvo type="min"/>
@@ -6135,7 +6363,7 @@
       </extLst>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="N51:N52">
+  <conditionalFormatting sqref="N54:N55">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
@@ -6147,7 +6375,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="Q3:Q50">
+  <conditionalFormatting sqref="Q3:Q53">
     <cfRule type="dataBar" priority="49">
       <dataBar>
         <cfvo type="min"/>
@@ -6161,7 +6389,7 @@
       </extLst>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="S3:S50">
+  <conditionalFormatting sqref="S3:S53">
     <cfRule type="dataBar" priority="51">
       <dataBar>
         <cfvo type="min"/>
@@ -6239,11 +6467,11 @@
     <hyperlink ref="O10" r:id="rId61"/>
     <hyperlink ref="G25" r:id="rId62" display="https://lcsc.com/brand-detail/396.html"/>
     <hyperlink ref="O25" r:id="rId63"/>
-    <hyperlink ref="O53" r:id="rId64"/>
-    <hyperlink ref="O59" r:id="rId65"/>
-    <hyperlink ref="O54" r:id="rId66" location="customerReviews"/>
-    <hyperlink ref="O55" r:id="rId67"/>
-    <hyperlink ref="O57" r:id="rId68"/>
+    <hyperlink ref="O56" r:id="rId64"/>
+    <hyperlink ref="O62" r:id="rId65"/>
+    <hyperlink ref="O57" r:id="rId66" location="customerReviews"/>
+    <hyperlink ref="O58" r:id="rId67"/>
+    <hyperlink ref="O60" r:id="rId68"/>
     <hyperlink ref="O7" r:id="rId69"/>
     <hyperlink ref="O13" r:id="rId70"/>
     <hyperlink ref="O22" r:id="rId71"/>
@@ -6251,9 +6479,12 @@
     <hyperlink ref="O48" r:id="rId73"/>
     <hyperlink ref="G17" r:id="rId74" display="https://www.digikey.com/en/supplier-centers/sunled"/>
     <hyperlink ref="O17" r:id="rId75"/>
+    <hyperlink ref="O51" r:id="rId76"/>
+    <hyperlink ref="O52" r:id="rId77"/>
+    <hyperlink ref="O53" r:id="rId78"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId76"/>
+  <pageSetup orientation="portrait" r:id="rId79"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
@@ -6268,7 +6499,7 @@
               <x14:axisColor rgb="FF000000"/>
             </x14:dataBar>
           </x14:cfRule>
-          <xm:sqref>Q61</xm:sqref>
+          <xm:sqref>Q64</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
           <x14:cfRule type="dataBar" id="{36ECBF5D-EFFC-4768-AC2E-9F5CCB8EA1CF}">
@@ -6281,7 +6512,7 @@
               <x14:axisColor rgb="FF000000"/>
             </x14:dataBar>
           </x14:cfRule>
-          <xm:sqref>S60:S61</xm:sqref>
+          <xm:sqref>S63:S64</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
           <x14:cfRule type="dataBar" id="{8043E1D2-A386-4972-9379-8F1175F4CD55}">
@@ -6294,7 +6525,7 @@
               <x14:axisColor rgb="FF000000"/>
             </x14:dataBar>
           </x14:cfRule>
-          <xm:sqref>T52</xm:sqref>
+          <xm:sqref>T55</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
           <x14:cfRule type="dataBar" id="{568B2A70-A44C-42B7-B5F8-9C8E28B37608}">
@@ -6307,7 +6538,7 @@
               <x14:axisColor rgb="FF000000"/>
             </x14:dataBar>
           </x14:cfRule>
-          <xm:sqref>T51</xm:sqref>
+          <xm:sqref>T54</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
           <x14:cfRule type="dataBar" id="{B802BE45-AE6E-4AFB-92D7-CAE7DD159284}">
@@ -6320,7 +6551,7 @@
               <x14:axisColor rgb="FF000000"/>
             </x14:dataBar>
           </x14:cfRule>
-          <xm:sqref>Q3:Q50</xm:sqref>
+          <xm:sqref>Q3:Q53</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
           <x14:cfRule type="dataBar" id="{423AC320-90C5-4685-9B12-A5EE24B441D5}">
@@ -6333,7 +6564,7 @@
               <x14:axisColor rgb="FF000000"/>
             </x14:dataBar>
           </x14:cfRule>
-          <xm:sqref>S3:S50</xm:sqref>
+          <xm:sqref>S3:S53</xm:sqref>
         </x14:conditionalFormatting>
       </x14:conditionalFormattings>
     </ext>

</xml_diff>